<commit_message>
Distinguir vigas invertidas de colgantes y corregir donde actua el ala
Las vigas de borde son invertidas (N.S.V 70 cm sobre N.F.L). Se
identifican por coincidencia de su eje con el contorno del edificio.
La losa aporta ala comprimida en el tramo si la viga cuelga y en el
apoyo si es invertida; antes se calculaba todo como rectangular.
VI 11a pasa a empotrada-apoyada sin apoyo intermedio y VI 07c a
empotrada-apoyada por el tabique del extremo derecho.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -1802,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB33"/>
+  <dimension ref="A1:AF33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1830,9 +1830,13 @@
     <col width="15" customWidth="1" min="23" max="23"/>
     <col width="34" customWidth="1" min="24" max="24"/>
     <col width="17" customWidth="1" min="25" max="25"/>
-    <col width="8" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
     <col width="8" customWidth="1" min="27" max="27"/>
-    <col width="7" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="8" customWidth="1" min="30" max="30"/>
+    <col width="8" customWidth="1" min="31" max="31"/>
+    <col width="7" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1931,6 +1935,10 @@
       <c r="Z2" s="18" t="n"/>
       <c r="AA2" s="18" t="n"/>
       <c r="AB2" s="18" t="n"/>
+      <c r="AC2" s="18" t="n"/>
+      <c r="AD2" s="18" t="n"/>
+      <c r="AE2" s="18" t="n"/>
+      <c r="AF2" s="18" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="18" t="n"/>
@@ -2032,15 +2040,35 @@
       </c>
       <c r="Z3" s="19" t="inlineStr">
         <is>
+          <t>tipo</t>
+        </is>
+      </c>
+      <c r="AA3" s="19" t="inlineStr">
+        <is>
+          <t>hf losa</t>
+        </is>
+      </c>
+      <c r="AB3" s="19" t="inlineStr">
+        <is>
+          <t>b ef tramo</t>
+        </is>
+      </c>
+      <c r="AC3" s="19" t="inlineStr">
+        <is>
+          <t>b ef apoyo</t>
+        </is>
+      </c>
+      <c r="AD3" s="19" t="inlineStr">
+        <is>
           <t>B trib.</t>
         </is>
       </c>
-      <c r="AA3" s="19" t="inlineStr">
+      <c r="AE3" s="19" t="inlineStr">
         <is>
           <t>h muro</t>
         </is>
       </c>
-      <c r="AB3" s="19" t="inlineStr">
+      <c r="AF3" s="19" t="inlineStr">
         <is>
           <t>rec.</t>
         </is>
@@ -2061,7 +2089,7 @@
         <v>9.9</v>
       </c>
       <c r="D4" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z4+Datos!$B$7*J4*L4/10000+Datos!$B$16*AA4)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z4)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD4+Datos!$B$7*J4*L4/10000+Datos!$B$16*AE4)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD4)</f>
         <v/>
       </c>
       <c r="E4" s="7" t="n"/>
@@ -2085,14 +2113,14 @@
         <v>15</v>
       </c>
       <c r="K4" s="7">
-        <f>L4-AB4</f>
+        <f>L4-AF4</f>
         <v/>
       </c>
       <c r="L4" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M4" s="25">
-        <f>IF(NOT(ISNUMBER(H4)),"---",IF(H4&lt;=0,"---",IF(H4*100/(Datos!$B$8*J4*K4^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H4*100/(Datos!$B$8*J4*K4^2*Datos!$B$5)))*J4*K4*Datos!$B$5/Datos!$B$6,0.0033*J4*K4))))</f>
+        <f>IF(NOT(ISNUMBER(H4)),"---",IF(H4&lt;=0,"---",IF(H4*100/(Datos!$B$8*AB4*K4^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H4*100/(Datos!$B$8*AB4*K4^2*Datos!$B$5)))*AB4*K4*Datos!$B$5/Datos!$B$6,0.0033*J4*K4))))</f>
         <v/>
       </c>
       <c r="N4" s="24" t="n">
@@ -2102,14 +2130,14 @@
         <v>25</v>
       </c>
       <c r="P4" s="25">
-        <f>IF(NOT(ISNUMBER(I4)),"---",IF(I4&lt;=0,"---",IF(I4*100/(Datos!$B$8*J4*K4^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I4*100/(Datos!$B$8*J4*K4^2*Datos!$B$5)))*J4*K4*Datos!$B$5/Datos!$B$6,0.0033*J4*K4))))</f>
+        <f>IF(NOT(ISNUMBER(I4)),"---",IF(I4&lt;=0,"---",IF(I4*100/(Datos!$B$8*AC4*K4^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I4*100/(Datos!$B$8*AC4*K4^2*Datos!$B$5)))*AC4*K4*Datos!$B$5/Datos!$B$6,0.0033*J4*K4))))</f>
         <v/>
       </c>
       <c r="Q4" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R4" s="24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="S4" s="25">
         <f>F4/(J4*0.85*K4)</f>
@@ -2126,12 +2154,12 @@
         <v>15</v>
       </c>
       <c r="W4" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M4),N4*PI()*(O4/10)^2/4&gt;=M4,TRUE),IF(ISNUMBER(P4),Q4*PI()*(R4/10)^2/4&gt;=P4,TRUE),IF(ISNUMBER(M4),M4&lt;=0.0163*J4*K4,TRUE),IF(ISNUMBER(P4),P4&lt;=0.0163*J4*K4,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F4&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J4*K4+2*PI()*(U4/10)^2/4*Datos!$B$6*K4/V4)),"NO VERIF. CORTE",IF(NOT(L4&gt;=C4*100/VLOOKUP(Y4,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M4),N4*PI()*(O4/10)^2/4&gt;=M4,TRUE),IF(ISNUMBER(P4),Q4*PI()*(R4/10)^2/4&gt;=P4,TRUE),IF(ISNUMBER(M4),M4&lt;=0.0163*AB4*K4,TRUE),IF(ISNUMBER(P4),P4&lt;=0.0163*AC4*K4,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F4&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J4*K4+2*PI()*(U4/10)^2/4*Datos!$B$6*K4/V4)),"NO VERIF. CORTE",IF(NOT(L4&gt;=C4*100/VLOOKUP(Y4,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X4" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm).</t>
+          <t>Armadura en 2 capas (rec. 6 cm). Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
         </is>
       </c>
       <c r="Y4" s="24" t="inlineStr">
@@ -2139,13 +2167,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z4" s="24" t="n">
+      <c r="Z4" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA4" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB4" s="7">
+        <f>IF(Z4="Colgante",MIN(C4*100/4,J4+16*AA4),J4)</f>
+        <v/>
+      </c>
+      <c r="AC4" s="7">
+        <f>IF(Z4="Invertida",MIN(C4*100/4,J4+16*AA4),J4)</f>
+        <v/>
+      </c>
+      <c r="AD4" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA4" s="24" t="n">
+      <c r="AE4" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB4" s="24" t="n">
+      <c r="AF4" s="24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2160,7 +2204,7 @@
         <v>3.95</v>
       </c>
       <c r="D5" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z5+Datos!$B$7*J5*L5/10000+Datos!$B$16*AA5)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z5)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD5+Datos!$B$7*J5*L5/10000+Datos!$B$16*AE5)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD5)</f>
         <v/>
       </c>
       <c r="E5" s="7" t="n"/>
@@ -2184,14 +2228,14 @@
         <v>15</v>
       </c>
       <c r="K5" s="7">
-        <f>L5-AB5</f>
+        <f>L5-AF5</f>
         <v/>
       </c>
       <c r="L5" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M5" s="25">
-        <f>IF(NOT(ISNUMBER(H5)),"---",IF(H5&lt;=0,"---",IF(H5*100/(Datos!$B$8*J5*K5^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H5*100/(Datos!$B$8*J5*K5^2*Datos!$B$5)))*J5*K5*Datos!$B$5/Datos!$B$6,0.0033*J5*K5))))</f>
+        <f>IF(NOT(ISNUMBER(H5)),"---",IF(H5&lt;=0,"---",IF(H5*100/(Datos!$B$8*AB5*K5^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H5*100/(Datos!$B$8*AB5*K5^2*Datos!$B$5)))*AB5*K5*Datos!$B$5/Datos!$B$6,0.0033*J5*K5))))</f>
         <v/>
       </c>
       <c r="N5" s="24" t="n">
@@ -2201,7 +2245,7 @@
         <v>12</v>
       </c>
       <c r="P5" s="25">
-        <f>IF(NOT(ISNUMBER(I5)),"---",IF(I5&lt;=0,"---",IF(I5*100/(Datos!$B$8*J5*K5^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I5*100/(Datos!$B$8*J5*K5^2*Datos!$B$5)))*J5*K5*Datos!$B$5/Datos!$B$6,0.0033*J5*K5))))</f>
+        <f>IF(NOT(ISNUMBER(I5)),"---",IF(I5&lt;=0,"---",IF(I5*100/(Datos!$B$8*AC5*K5^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I5*100/(Datos!$B$8*AC5*K5^2*Datos!$B$5)))*AC5*K5*Datos!$B$5/Datos!$B$6,0.0033*J5*K5))))</f>
         <v/>
       </c>
       <c r="Q5" s="24" t="n">
@@ -2225,22 +2269,42 @@
         <v>30</v>
       </c>
       <c r="W5" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M5),N5*PI()*(O5/10)^2/4&gt;=M5,TRUE),IF(ISNUMBER(P5),Q5*PI()*(R5/10)^2/4&gt;=P5,TRUE),IF(ISNUMBER(M5),M5&lt;=0.0163*J5*K5,TRUE),IF(ISNUMBER(P5),P5&lt;=0.0163*J5*K5,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F5&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J5*K5+2*PI()*(U5/10)^2/4*Datos!$B$6*K5/V5)),"NO VERIF. CORTE",IF(NOT(L5&gt;=C5*100/VLOOKUP(Y5,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X5" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M5),N5*PI()*(O5/10)^2/4&gt;=M5,TRUE),IF(ISNUMBER(P5),Q5*PI()*(R5/10)^2/4&gt;=P5,TRUE),IF(ISNUMBER(M5),M5&lt;=0.0163*AB5*K5,TRUE),IF(ISNUMBER(P5),P5&lt;=0.0163*AC5*K5,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F5&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J5*K5+2*PI()*(U5/10)^2/4*Datos!$B$6*K5/V5)),"NO VERIF. CORTE",IF(NOT(L5&gt;=C5*100/VLOOKUP(Y5,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X5" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y5" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z5" s="24" t="n">
+      <c r="Z5" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA5" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB5" s="7">
+        <f>IF(Z5="Colgante",MIN(C5*100/4,J5+16*AA5),J5)</f>
+        <v/>
+      </c>
+      <c r="AC5" s="7">
+        <f>IF(Z5="Invertida",MIN(C5*100/4,J5+16*AA5),J5)</f>
+        <v/>
+      </c>
+      <c r="AD5" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA5" s="24" t="n">
+      <c r="AE5" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB5" s="24" t="n">
+      <c r="AF5" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2255,7 +2319,7 @@
         <v>9.880000000000001</v>
       </c>
       <c r="D6" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z6+Datos!$B$7*J6*L6/10000+Datos!$B$16*AA6)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z6)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD6+Datos!$B$7*J6*L6/10000+Datos!$B$16*AE6)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD6)</f>
         <v/>
       </c>
       <c r="E6" s="7" t="n"/>
@@ -2279,14 +2343,14 @@
         <v>15</v>
       </c>
       <c r="K6" s="7">
-        <f>L6-AB6</f>
+        <f>L6-AF6</f>
         <v/>
       </c>
       <c r="L6" s="24" t="n">
         <v>60</v>
       </c>
       <c r="M6" s="25">
-        <f>IF(NOT(ISNUMBER(H6)),"---",IF(H6&lt;=0,"---",IF(H6*100/(Datos!$B$8*J6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H6*100/(Datos!$B$8*J6*K6^2*Datos!$B$5)))*J6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
+        <f>IF(NOT(ISNUMBER(H6)),"---",IF(H6&lt;=0,"---",IF(H6*100/(Datos!$B$8*AB6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H6*100/(Datos!$B$8*AB6*K6^2*Datos!$B$5)))*AB6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
         <v/>
       </c>
       <c r="N6" s="24" t="n">
@@ -2296,7 +2360,7 @@
         <v>20</v>
       </c>
       <c r="P6" s="25">
-        <f>IF(NOT(ISNUMBER(I6)),"---",IF(I6&lt;=0,"---",IF(I6*100/(Datos!$B$8*J6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I6*100/(Datos!$B$8*J6*K6^2*Datos!$B$5)))*J6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
+        <f>IF(NOT(ISNUMBER(I6)),"---",IF(I6&lt;=0,"---",IF(I6*100/(Datos!$B$8*AC6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I6*100/(Datos!$B$8*AC6*K6^2*Datos!$B$5)))*AC6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
         <v/>
       </c>
       <c r="Q6" s="24" t="n">
@@ -2320,12 +2384,12 @@
         <v>10</v>
       </c>
       <c r="W6" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M6),N6*PI()*(O6/10)^2/4&gt;=M6,TRUE),IF(ISNUMBER(P6),Q6*PI()*(R6/10)^2/4&gt;=P6,TRUE),IF(ISNUMBER(M6),M6&lt;=0.0163*J6*K6,TRUE),IF(ISNUMBER(P6),P6&lt;=0.0163*J6*K6,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F6&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J6*K6+2*PI()*(U6/10)^2/4*Datos!$B$6*K6/V6)),"NO VERIF. CORTE",IF(NOT(L6&gt;=C6*100/VLOOKUP(Y6,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M6),N6*PI()*(O6/10)^2/4&gt;=M6,TRUE),IF(ISNUMBER(P6),Q6*PI()*(R6/10)^2/4&gt;=P6,TRUE),IF(ISNUMBER(M6),M6&lt;=0.0163*AB6*K6,TRUE),IF(ISNUMBER(P6),P6&lt;=0.0163*AC6*K6,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F6&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J6*K6+2*PI()*(U6/10)^2/4*Datos!$B$6*K6/V6)),"NO VERIF. CORTE",IF(NOT(L6&gt;=C6*100/VLOOKUP(Y6,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X6" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). La armadura de apoyo necesaria supera la cuantia maxima: la seccion 15x60 no alcanza como tramo unico de 9,88 m. Requiere d=65 cm o apoyo intermedio.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Es viga colgante, asi que sobre el apoyo la losa queda traccionada y no aporta ala comprimida: la seccion es rectangular 15x60 y la armadura necesaria (18,6 cm2) supera la cuantia maxima (13,2). Confirmado que no tiene apoyo intermedio. Revisar el ancho tributario real.</t>
         </is>
       </c>
       <c r="Y6" s="24" t="inlineStr">
@@ -2333,13 +2397,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z6" s="24" t="n">
+      <c r="Z6" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA6" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB6" s="7">
+        <f>IF(Z6="Colgante",MIN(C6*100/4,J6+16*AA6),J6)</f>
+        <v/>
+      </c>
+      <c r="AC6" s="7">
+        <f>IF(Z6="Invertida",MIN(C6*100/4,J6+16*AA6),J6)</f>
+        <v/>
+      </c>
+      <c r="AD6" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA6" s="24" t="n">
+      <c r="AE6" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB6" s="24" t="n">
+      <c r="AF6" s="24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2354,7 +2434,7 @@
         <v>3.75</v>
       </c>
       <c r="D7" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z7+Datos!$B$7*J7*L7/10000+Datos!$B$16*AA7)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z7)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD7+Datos!$B$7*J7*L7/10000+Datos!$B$16*AE7)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD7)</f>
         <v/>
       </c>
       <c r="E7" s="7" t="n"/>
@@ -2378,14 +2458,14 @@
         <v>15</v>
       </c>
       <c r="K7" s="7">
-        <f>L7-AB7</f>
+        <f>L7-AF7</f>
         <v/>
       </c>
       <c r="L7" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M7" s="25">
-        <f>IF(NOT(ISNUMBER(H7)),"---",IF(H7&lt;=0,"---",IF(H7*100/(Datos!$B$8*J7*K7^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H7*100/(Datos!$B$8*J7*K7^2*Datos!$B$5)))*J7*K7*Datos!$B$5/Datos!$B$6,0.0033*J7*K7))))</f>
+        <f>IF(NOT(ISNUMBER(H7)),"---",IF(H7&lt;=0,"---",IF(H7*100/(Datos!$B$8*AB7*K7^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H7*100/(Datos!$B$8*AB7*K7^2*Datos!$B$5)))*AB7*K7*Datos!$B$5/Datos!$B$6,0.0033*J7*K7))))</f>
         <v/>
       </c>
       <c r="N7" s="24" t="n">
@@ -2395,7 +2475,7 @@
         <v>12</v>
       </c>
       <c r="P7" s="25">
-        <f>IF(NOT(ISNUMBER(I7)),"---",IF(I7&lt;=0,"---",IF(I7*100/(Datos!$B$8*J7*K7^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I7*100/(Datos!$B$8*J7*K7^2*Datos!$B$5)))*J7*K7*Datos!$B$5/Datos!$B$6,0.0033*J7*K7))))</f>
+        <f>IF(NOT(ISNUMBER(I7)),"---",IF(I7&lt;=0,"---",IF(I7*100/(Datos!$B$8*AC7*K7^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I7*100/(Datos!$B$8*AC7*K7^2*Datos!$B$5)))*AC7*K7*Datos!$B$5/Datos!$B$6,0.0033*J7*K7))))</f>
         <v/>
       </c>
       <c r="Q7" s="24" t="n">
@@ -2419,7 +2499,7 @@
         <v>30</v>
       </c>
       <c r="W7" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M7),N7*PI()*(O7/10)^2/4&gt;=M7,TRUE),IF(ISNUMBER(P7),Q7*PI()*(R7/10)^2/4&gt;=P7,TRUE),IF(ISNUMBER(M7),M7&lt;=0.0163*J7*K7,TRUE),IF(ISNUMBER(P7),P7&lt;=0.0163*J7*K7,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F7&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J7*K7+2*PI()*(U7/10)^2/4*Datos!$B$6*K7/V7)),"NO VERIF. CORTE",IF(NOT(L7&gt;=C7*100/VLOOKUP(Y7,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M7),N7*PI()*(O7/10)^2/4&gt;=M7,TRUE),IF(ISNUMBER(P7),Q7*PI()*(R7/10)^2/4&gt;=P7,TRUE),IF(ISNUMBER(M7),M7&lt;=0.0163*AB7*K7,TRUE),IF(ISNUMBER(P7),P7&lt;=0.0163*AC7*K7,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F7&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J7*K7+2*PI()*(U7/10)^2/4*Datos!$B$6*K7/V7)),"NO VERIF. CORTE",IF(NOT(L7&gt;=C7*100/VLOOKUP(Y7,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X7" s="7" t="n"/>
@@ -2428,13 +2508,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z7" s="24" t="n">
+      <c r="Z7" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA7" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB7" s="7">
+        <f>IF(Z7="Colgante",MIN(C7*100/4,J7+16*AA7),J7)</f>
+        <v/>
+      </c>
+      <c r="AC7" s="7">
+        <f>IF(Z7="Invertida",MIN(C7*100/4,J7+16*AA7),J7)</f>
+        <v/>
+      </c>
+      <c r="AD7" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA7" s="24" t="n">
+      <c r="AE7" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB7" s="24" t="n">
+      <c r="AF7" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2449,7 +2545,7 @@
         <v>3.75</v>
       </c>
       <c r="D8" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z8+Datos!$B$7*J8*L8/10000+Datos!$B$16*AA8)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z8)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD8+Datos!$B$7*J8*L8/10000+Datos!$B$16*AE8)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD8)</f>
         <v/>
       </c>
       <c r="E8" s="7" t="n"/>
@@ -2473,14 +2569,14 @@
         <v>15</v>
       </c>
       <c r="K8" s="7">
-        <f>L8-AB8</f>
+        <f>L8-AF8</f>
         <v/>
       </c>
       <c r="L8" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M8" s="25">
-        <f>IF(NOT(ISNUMBER(H8)),"---",IF(H8&lt;=0,"---",IF(H8*100/(Datos!$B$8*J8*K8^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H8*100/(Datos!$B$8*J8*K8^2*Datos!$B$5)))*J8*K8*Datos!$B$5/Datos!$B$6,0.0033*J8*K8))))</f>
+        <f>IF(NOT(ISNUMBER(H8)),"---",IF(H8&lt;=0,"---",IF(H8*100/(Datos!$B$8*AB8*K8^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H8*100/(Datos!$B$8*AB8*K8^2*Datos!$B$5)))*AB8*K8*Datos!$B$5/Datos!$B$6,0.0033*J8*K8))))</f>
         <v/>
       </c>
       <c r="N8" s="24" t="n">
@@ -2490,7 +2586,7 @@
         <v>12</v>
       </c>
       <c r="P8" s="25">
-        <f>IF(NOT(ISNUMBER(I8)),"---",IF(I8&lt;=0,"---",IF(I8*100/(Datos!$B$8*J8*K8^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I8*100/(Datos!$B$8*J8*K8^2*Datos!$B$5)))*J8*K8*Datos!$B$5/Datos!$B$6,0.0033*J8*K8))))</f>
+        <f>IF(NOT(ISNUMBER(I8)),"---",IF(I8&lt;=0,"---",IF(I8*100/(Datos!$B$8*AC8*K8^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I8*100/(Datos!$B$8*AC8*K8^2*Datos!$B$5)))*AC8*K8*Datos!$B$5/Datos!$B$6,0.0033*J8*K8))))</f>
         <v/>
       </c>
       <c r="Q8" s="24" t="n">
@@ -2514,7 +2610,7 @@
         <v>30</v>
       </c>
       <c r="W8" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*J8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*J8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos!$B$6*K8/V8)),"NO VERIF. CORTE",IF(NOT(L8&gt;=C8*100/VLOOKUP(Y8,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*AB8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*AC8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos!$B$6*K8/V8)),"NO VERIF. CORTE",IF(NOT(L8&gt;=C8*100/VLOOKUP(Y8,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X8" s="7" t="n"/>
@@ -2523,13 +2619,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z8" s="24" t="n">
+      <c r="Z8" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA8" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB8" s="7">
+        <f>IF(Z8="Colgante",MIN(C8*100/4,J8+16*AA8),J8)</f>
+        <v/>
+      </c>
+      <c r="AC8" s="7">
+        <f>IF(Z8="Invertida",MIN(C8*100/4,J8+16*AA8),J8)</f>
+        <v/>
+      </c>
+      <c r="AD8" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA8" s="24" t="n">
+      <c r="AE8" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB8" s="24" t="n">
+      <c r="AF8" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2544,7 +2656,7 @@
         <v>3.8</v>
       </c>
       <c r="D9" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z9+Datos!$B$7*J9*L9/10000+Datos!$B$16*AA9)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z9)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD9+Datos!$B$7*J9*L9/10000+Datos!$B$16*AE9)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD9)</f>
         <v/>
       </c>
       <c r="E9" s="7" t="n"/>
@@ -2568,14 +2680,14 @@
         <v>15</v>
       </c>
       <c r="K9" s="7">
-        <f>L9-AB9</f>
+        <f>L9-AF9</f>
         <v/>
       </c>
       <c r="L9" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M9" s="25">
-        <f>IF(NOT(ISNUMBER(H9)),"---",IF(H9&lt;=0,"---",IF(H9*100/(Datos!$B$8*J9*K9^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H9*100/(Datos!$B$8*J9*K9^2*Datos!$B$5)))*J9*K9*Datos!$B$5/Datos!$B$6,0.0033*J9*K9))))</f>
+        <f>IF(NOT(ISNUMBER(H9)),"---",IF(H9&lt;=0,"---",IF(H9*100/(Datos!$B$8*AB9*K9^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H9*100/(Datos!$B$8*AB9*K9^2*Datos!$B$5)))*AB9*K9*Datos!$B$5/Datos!$B$6,0.0033*J9*K9))))</f>
         <v/>
       </c>
       <c r="N9" s="24" t="n">
@@ -2585,7 +2697,7 @@
         <v>12</v>
       </c>
       <c r="P9" s="25">
-        <f>IF(NOT(ISNUMBER(I9)),"---",IF(I9&lt;=0,"---",IF(I9*100/(Datos!$B$8*J9*K9^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I9*100/(Datos!$B$8*J9*K9^2*Datos!$B$5)))*J9*K9*Datos!$B$5/Datos!$B$6,0.0033*J9*K9))))</f>
+        <f>IF(NOT(ISNUMBER(I9)),"---",IF(I9&lt;=0,"---",IF(I9*100/(Datos!$B$8*AC9*K9^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I9*100/(Datos!$B$8*AC9*K9^2*Datos!$B$5)))*AC9*K9*Datos!$B$5/Datos!$B$6,0.0033*J9*K9))))</f>
         <v/>
       </c>
       <c r="Q9" s="24" t="n">
@@ -2609,7 +2721,7 @@
         <v>30</v>
       </c>
       <c r="W9" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M9),N9*PI()*(O9/10)^2/4&gt;=M9,TRUE),IF(ISNUMBER(P9),Q9*PI()*(R9/10)^2/4&gt;=P9,TRUE),IF(ISNUMBER(M9),M9&lt;=0.0163*J9*K9,TRUE),IF(ISNUMBER(P9),P9&lt;=0.0163*J9*K9,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F9&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J9*K9+2*PI()*(U9/10)^2/4*Datos!$B$6*K9/V9)),"NO VERIF. CORTE",IF(NOT(L9&gt;=C9*100/VLOOKUP(Y9,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M9),N9*PI()*(O9/10)^2/4&gt;=M9,TRUE),IF(ISNUMBER(P9),Q9*PI()*(R9/10)^2/4&gt;=P9,TRUE),IF(ISNUMBER(M9),M9&lt;=0.0163*AB9*K9,TRUE),IF(ISNUMBER(P9),P9&lt;=0.0163*AC9*K9,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F9&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J9*K9+2*PI()*(U9/10)^2/4*Datos!$B$6*K9/V9)),"NO VERIF. CORTE",IF(NOT(L9&gt;=C9*100/VLOOKUP(Y9,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X9" s="7" t="n"/>
@@ -2618,13 +2730,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z9" s="24" t="n">
+      <c r="Z9" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA9" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB9" s="7">
+        <f>IF(Z9="Colgante",MIN(C9*100/4,J9+16*AA9),J9)</f>
+        <v/>
+      </c>
+      <c r="AC9" s="7">
+        <f>IF(Z9="Invertida",MIN(C9*100/4,J9+16*AA9),J9)</f>
+        <v/>
+      </c>
+      <c r="AD9" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA9" s="24" t="n">
+      <c r="AE9" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB9" s="24" t="n">
+      <c r="AF9" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2639,7 +2767,7 @@
         <v>3.37</v>
       </c>
       <c r="D10" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AA10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z10)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AE10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD10)</f>
         <v/>
       </c>
       <c r="E10" s="7" t="n"/>
@@ -2663,14 +2791,14 @@
         <v>15</v>
       </c>
       <c r="K10" s="7">
-        <f>L10-AB10</f>
+        <f>L10-AF10</f>
         <v/>
       </c>
       <c r="L10" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M10" s="25">
-        <f>IF(NOT(ISNUMBER(H10)),"---",IF(H10&lt;=0,"---",IF(H10*100/(Datos!$B$8*J10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H10*100/(Datos!$B$8*J10*K10^2*Datos!$B$5)))*J10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
+        <f>IF(NOT(ISNUMBER(H10)),"---",IF(H10&lt;=0,"---",IF(H10*100/(Datos!$B$8*AB10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H10*100/(Datos!$B$8*AB10*K10^2*Datos!$B$5)))*AB10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
         <v/>
       </c>
       <c r="N10" s="24" t="n">
@@ -2680,7 +2808,7 @@
         <v>12</v>
       </c>
       <c r="P10" s="25">
-        <f>IF(NOT(ISNUMBER(I10)),"---",IF(I10&lt;=0,"---",IF(I10*100/(Datos!$B$8*J10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I10*100/(Datos!$B$8*J10*K10^2*Datos!$B$5)))*J10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
+        <f>IF(NOT(ISNUMBER(I10)),"---",IF(I10&lt;=0,"---",IF(I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)))*AC10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
         <v/>
       </c>
       <c r="Q10" s="24" t="n">
@@ -2704,22 +2832,42 @@
         <v>30</v>
       </c>
       <c r="W10" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*J10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*J10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X10" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X10" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y10" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z10" s="24" t="n">
+      <c r="Z10" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA10" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB10" s="7">
+        <f>IF(Z10="Colgante",MIN(C10*100/4,J10+16*AA10),J10)</f>
+        <v/>
+      </c>
+      <c r="AC10" s="7">
+        <f>IF(Z10="Invertida",MIN(C10*100/4,J10+16*AA10),J10)</f>
+        <v/>
+      </c>
+      <c r="AD10" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA10" s="24" t="n">
+      <c r="AE10" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB10" s="24" t="n">
+      <c r="AF10" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2734,7 +2882,7 @@
         <v>4.03</v>
       </c>
       <c r="D11" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AA11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z11)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AE11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD11)</f>
         <v/>
       </c>
       <c r="E11" s="7" t="n"/>
@@ -2758,14 +2906,14 @@
         <v>15</v>
       </c>
       <c r="K11" s="7">
-        <f>L11-AB11</f>
+        <f>L11-AF11</f>
         <v/>
       </c>
       <c r="L11" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M11" s="25">
-        <f>IF(NOT(ISNUMBER(H11)),"---",IF(H11&lt;=0,"---",IF(H11*100/(Datos!$B$8*J11*K11^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H11*100/(Datos!$B$8*J11*K11^2*Datos!$B$5)))*J11*K11*Datos!$B$5/Datos!$B$6,0.0033*J11*K11))))</f>
+        <f>IF(NOT(ISNUMBER(H11)),"---",IF(H11&lt;=0,"---",IF(H11*100/(Datos!$B$8*AB11*K11^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H11*100/(Datos!$B$8*AB11*K11^2*Datos!$B$5)))*AB11*K11*Datos!$B$5/Datos!$B$6,0.0033*J11*K11))))</f>
         <v/>
       </c>
       <c r="N11" s="24" t="n">
@@ -2775,7 +2923,7 @@
         <v>12</v>
       </c>
       <c r="P11" s="25">
-        <f>IF(NOT(ISNUMBER(I11)),"---",IF(I11&lt;=0,"---",IF(I11*100/(Datos!$B$8*J11*K11^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I11*100/(Datos!$B$8*J11*K11^2*Datos!$B$5)))*J11*K11*Datos!$B$5/Datos!$B$6,0.0033*J11*K11))))</f>
+        <f>IF(NOT(ISNUMBER(I11)),"---",IF(I11&lt;=0,"---",IF(I11*100/(Datos!$B$8*AC11*K11^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I11*100/(Datos!$B$8*AC11*K11^2*Datos!$B$5)))*AC11*K11*Datos!$B$5/Datos!$B$6,0.0033*J11*K11))))</f>
         <v/>
       </c>
       <c r="Q11" s="24" t="n">
@@ -2799,22 +2947,42 @@
         <v>30</v>
       </c>
       <c r="W11" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M11),N11*PI()*(O11/10)^2/4&gt;=M11,TRUE),IF(ISNUMBER(P11),Q11*PI()*(R11/10)^2/4&gt;=P11,TRUE),IF(ISNUMBER(M11),M11&lt;=0.0163*J11*K11,TRUE),IF(ISNUMBER(P11),P11&lt;=0.0163*J11*K11,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F11&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J11*K11+2*PI()*(U11/10)^2/4*Datos!$B$6*K11/V11)),"NO VERIF. CORTE",IF(NOT(L11&gt;=C11*100/VLOOKUP(Y11,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X11" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M11),N11*PI()*(O11/10)^2/4&gt;=M11,TRUE),IF(ISNUMBER(P11),Q11*PI()*(R11/10)^2/4&gt;=P11,TRUE),IF(ISNUMBER(M11),M11&lt;=0.0163*AB11*K11,TRUE),IF(ISNUMBER(P11),P11&lt;=0.0163*AC11*K11,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F11&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J11*K11+2*PI()*(U11/10)^2/4*Datos!$B$6*K11/V11)),"NO VERIF. CORTE",IF(NOT(L11&gt;=C11*100/VLOOKUP(Y11,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X11" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y11" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z11" s="24" t="n">
+      <c r="Z11" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA11" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB11" s="7">
+        <f>IF(Z11="Colgante",MIN(C11*100/4,J11+16*AA11),J11)</f>
+        <v/>
+      </c>
+      <c r="AC11" s="7">
+        <f>IF(Z11="Invertida",MIN(C11*100/4,J11+16*AA11),J11)</f>
+        <v/>
+      </c>
+      <c r="AD11" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA11" s="24" t="n">
+      <c r="AE11" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB11" s="24" t="n">
+      <c r="AF11" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2829,7 +2997,7 @@
         <v>8.6</v>
       </c>
       <c r="D12" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AA12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z12)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AE12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD12)</f>
         <v/>
       </c>
       <c r="E12" s="7" t="n"/>
@@ -2853,14 +3021,14 @@
         <v>15</v>
       </c>
       <c r="K12" s="7">
-        <f>L12-AB12</f>
+        <f>L12-AF12</f>
         <v/>
       </c>
       <c r="L12" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M12" s="25">
-        <f>IF(NOT(ISNUMBER(H12)),"---",IF(H12&lt;=0,"---",IF(H12*100/(Datos!$B$8*J12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H12*100/(Datos!$B$8*J12*K12^2*Datos!$B$5)))*J12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
+        <f>IF(NOT(ISNUMBER(H12)),"---",IF(H12&lt;=0,"---",IF(H12*100/(Datos!$B$8*AB12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H12*100/(Datos!$B$8*AB12*K12^2*Datos!$B$5)))*AB12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
         <v/>
       </c>
       <c r="N12" s="24" t="n">
@@ -2870,7 +3038,7 @@
         <v>25</v>
       </c>
       <c r="P12" s="25">
-        <f>IF(NOT(ISNUMBER(I12)),"---",IF(I12&lt;=0,"---",IF(I12*100/(Datos!$B$8*J12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I12*100/(Datos!$B$8*J12*K12^2*Datos!$B$5)))*J12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
+        <f>IF(NOT(ISNUMBER(I12)),"---",IF(I12&lt;=0,"---",IF(I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)))*AC12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
         <v/>
       </c>
       <c r="Q12" s="24" t="n">
@@ -2894,26 +3062,42 @@
         <v>10</v>
       </c>
       <c r="W12" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*J12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*J12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X12" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm).</t>
+          <t>Armadura en 2 capas (rec. 6 cm). Empotrada-apoyada: columna 30x15 a la izquierda, tabique a la derecha. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
         </is>
       </c>
       <c r="Y12" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
-        </is>
-      </c>
-      <c r="Z12" s="24" t="n">
+          <t>Empotrada-apoyada</t>
+        </is>
+      </c>
+      <c r="Z12" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA12" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB12" s="7">
+        <f>IF(Z12="Colgante",MIN(C12*100/4,J12+16*AA12),J12)</f>
+        <v/>
+      </c>
+      <c r="AC12" s="7">
+        <f>IF(Z12="Invertida",MIN(C12*100/4,J12+16*AA12),J12)</f>
+        <v/>
+      </c>
+      <c r="AD12" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA12" s="24" t="n">
+      <c r="AE12" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB12" s="24" t="n">
+      <c r="AF12" s="24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2928,7 +3112,7 @@
         <v>3.65</v>
       </c>
       <c r="D13" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AA13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z13)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AE13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD13)</f>
         <v/>
       </c>
       <c r="E13" s="7" t="n"/>
@@ -2952,14 +3136,14 @@
         <v>15</v>
       </c>
       <c r="K13" s="7">
-        <f>L13-AB13</f>
+        <f>L13-AF13</f>
         <v/>
       </c>
       <c r="L13" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M13" s="25">
-        <f>IF(NOT(ISNUMBER(H13)),"---",IF(H13&lt;=0,"---",IF(H13*100/(Datos!$B$8*J13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H13*100/(Datos!$B$8*J13*K13^2*Datos!$B$5)))*J13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
+        <f>IF(NOT(ISNUMBER(H13)),"---",IF(H13&lt;=0,"---",IF(H13*100/(Datos!$B$8*AB13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H13*100/(Datos!$B$8*AB13*K13^2*Datos!$B$5)))*AB13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
         <v/>
       </c>
       <c r="N13" s="24" t="n">
@@ -2969,7 +3153,7 @@
         <v>12</v>
       </c>
       <c r="P13" s="25">
-        <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*J13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*J13*K13^2*Datos!$B$5)))*J13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
+        <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)))*AC13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
         <v/>
       </c>
       <c r="Q13" s="24" t="n">
@@ -2993,7 +3177,7 @@
         <v>30</v>
       </c>
       <c r="W13" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*J13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*J13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X13" s="7" t="n"/>
@@ -3002,13 +3186,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z13" s="24" t="n">
+      <c r="Z13" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA13" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB13" s="7">
+        <f>IF(Z13="Colgante",MIN(C13*100/4,J13+16*AA13),J13)</f>
+        <v/>
+      </c>
+      <c r="AC13" s="7">
+        <f>IF(Z13="Invertida",MIN(C13*100/4,J13+16*AA13),J13)</f>
+        <v/>
+      </c>
+      <c r="AD13" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA13" s="24" t="n">
+      <c r="AE13" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB13" s="24" t="n">
+      <c r="AF13" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3023,7 +3223,7 @@
         <v>4.85</v>
       </c>
       <c r="D14" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AA14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z14)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AE14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD14)</f>
         <v/>
       </c>
       <c r="E14" s="7" t="n"/>
@@ -3047,14 +3247,14 @@
         <v>15</v>
       </c>
       <c r="K14" s="7">
-        <f>L14-AB14</f>
+        <f>L14-AF14</f>
         <v/>
       </c>
       <c r="L14" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M14" s="25">
-        <f>IF(NOT(ISNUMBER(H14)),"---",IF(H14&lt;=0,"---",IF(H14*100/(Datos!$B$8*J14*K14^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H14*100/(Datos!$B$8*J14*K14^2*Datos!$B$5)))*J14*K14*Datos!$B$5/Datos!$B$6,0.0033*J14*K14))))</f>
+        <f>IF(NOT(ISNUMBER(H14)),"---",IF(H14&lt;=0,"---",IF(H14*100/(Datos!$B$8*AB14*K14^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H14*100/(Datos!$B$8*AB14*K14^2*Datos!$B$5)))*AB14*K14*Datos!$B$5/Datos!$B$6,0.0033*J14*K14))))</f>
         <v/>
       </c>
       <c r="N14" s="24" t="n">
@@ -3064,7 +3264,7 @@
         <v>12</v>
       </c>
       <c r="P14" s="25">
-        <f>IF(NOT(ISNUMBER(I14)),"---",IF(I14&lt;=0,"---",IF(I14*100/(Datos!$B$8*J14*K14^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I14*100/(Datos!$B$8*J14*K14^2*Datos!$B$5)))*J14*K14*Datos!$B$5/Datos!$B$6,0.0033*J14*K14))))</f>
+        <f>IF(NOT(ISNUMBER(I14)),"---",IF(I14&lt;=0,"---",IF(I14*100/(Datos!$B$8*AC14*K14^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I14*100/(Datos!$B$8*AC14*K14^2*Datos!$B$5)))*AC14*K14*Datos!$B$5/Datos!$B$6,0.0033*J14*K14))))</f>
         <v/>
       </c>
       <c r="Q14" s="24" t="n">
@@ -3088,7 +3288,7 @@
         <v>30</v>
       </c>
       <c r="W14" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M14),N14*PI()*(O14/10)^2/4&gt;=M14,TRUE),IF(ISNUMBER(P14),Q14*PI()*(R14/10)^2/4&gt;=P14,TRUE),IF(ISNUMBER(M14),M14&lt;=0.0163*J14*K14,TRUE),IF(ISNUMBER(P14),P14&lt;=0.0163*J14*K14,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F14&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J14*K14+2*PI()*(U14/10)^2/4*Datos!$B$6*K14/V14)),"NO VERIF. CORTE",IF(NOT(L14&gt;=C14*100/VLOOKUP(Y14,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M14),N14*PI()*(O14/10)^2/4&gt;=M14,TRUE),IF(ISNUMBER(P14),Q14*PI()*(R14/10)^2/4&gt;=P14,TRUE),IF(ISNUMBER(M14),M14&lt;=0.0163*AB14*K14,TRUE),IF(ISNUMBER(P14),P14&lt;=0.0163*AC14*K14,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F14&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J14*K14+2*PI()*(U14/10)^2/4*Datos!$B$6*K14/V14)),"NO VERIF. CORTE",IF(NOT(L14&gt;=C14*100/VLOOKUP(Y14,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X14" s="7" t="n"/>
@@ -3097,13 +3297,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z14" s="24" t="n">
+      <c r="Z14" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA14" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB14" s="7">
+        <f>IF(Z14="Colgante",MIN(C14*100/4,J14+16*AA14),J14)</f>
+        <v/>
+      </c>
+      <c r="AC14" s="7">
+        <f>IF(Z14="Invertida",MIN(C14*100/4,J14+16*AA14),J14)</f>
+        <v/>
+      </c>
+      <c r="AD14" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA14" s="24" t="n">
+      <c r="AE14" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB14" s="24" t="n">
+      <c r="AF14" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3118,7 +3334,7 @@
         <v>4.85</v>
       </c>
       <c r="D15" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z15+Datos!$B$7*J15*L15/10000+Datos!$B$16*AA15)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z15)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD15+Datos!$B$7*J15*L15/10000+Datos!$B$16*AE15)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD15)</f>
         <v/>
       </c>
       <c r="E15" s="7" t="n"/>
@@ -3142,14 +3358,14 @@
         <v>15</v>
       </c>
       <c r="K15" s="7">
-        <f>L15-AB15</f>
+        <f>L15-AF15</f>
         <v/>
       </c>
       <c r="L15" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M15" s="25">
-        <f>IF(NOT(ISNUMBER(H15)),"---",IF(H15&lt;=0,"---",IF(H15*100/(Datos!$B$8*J15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H15*100/(Datos!$B$8*J15*K15^2*Datos!$B$5)))*J15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
+        <f>IF(NOT(ISNUMBER(H15)),"---",IF(H15&lt;=0,"---",IF(H15*100/(Datos!$B$8*AB15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H15*100/(Datos!$B$8*AB15*K15^2*Datos!$B$5)))*AB15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
         <v/>
       </c>
       <c r="N15" s="24" t="n">
@@ -3159,7 +3375,7 @@
         <v>16</v>
       </c>
       <c r="P15" s="25">
-        <f>IF(NOT(ISNUMBER(I15)),"---",IF(I15&lt;=0,"---",IF(I15*100/(Datos!$B$8*J15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I15*100/(Datos!$B$8*J15*K15^2*Datos!$B$5)))*J15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
+        <f>IF(NOT(ISNUMBER(I15)),"---",IF(I15&lt;=0,"---",IF(I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)))*AC15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
         <v/>
       </c>
       <c r="Q15" s="24" t="inlineStr">
@@ -3187,7 +3403,7 @@
         <v>30</v>
       </c>
       <c r="W15" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M15),N15*PI()*(O15/10)^2/4&gt;=M15,TRUE),IF(ISNUMBER(P15),Q15*PI()*(R15/10)^2/4&gt;=P15,TRUE),IF(ISNUMBER(M15),M15&lt;=0.0163*J15*K15,TRUE),IF(ISNUMBER(P15),P15&lt;=0.0163*J15*K15,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F15&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J15*K15+2*PI()*(U15/10)^2/4*Datos!$B$6*K15/V15)),"NO VERIF. CORTE",IF(NOT(L15&gt;=C15*100/VLOOKUP(Y15,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M15),N15*PI()*(O15/10)^2/4&gt;=M15,TRUE),IF(ISNUMBER(P15),Q15*PI()*(R15/10)^2/4&gt;=P15,TRUE),IF(ISNUMBER(M15),M15&lt;=0.0163*AB15*K15,TRUE),IF(ISNUMBER(P15),P15&lt;=0.0163*AC15*K15,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F15&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J15*K15+2*PI()*(U15/10)^2/4*Datos!$B$6*K15/V15)),"NO VERIF. CORTE",IF(NOT(L15&gt;=C15*100/VLOOKUP(Y15,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X15" s="7" t="n"/>
@@ -3196,13 +3412,29 @@
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z15" s="24" t="n">
+      <c r="Z15" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA15" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB15" s="7">
+        <f>IF(Z15="Colgante",MIN(C15*100/4,J15+16*AA15),J15)</f>
+        <v/>
+      </c>
+      <c r="AC15" s="7">
+        <f>IF(Z15="Invertida",MIN(C15*100/4,J15+16*AA15),J15)</f>
+        <v/>
+      </c>
+      <c r="AD15" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA15" s="24" t="n">
+      <c r="AE15" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB15" s="24" t="n">
+      <c r="AF15" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3217,7 +3449,7 @@
         <v>2.55</v>
       </c>
       <c r="D16" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AA16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z16)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AE16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD16)</f>
         <v/>
       </c>
       <c r="E16" s="7" t="n"/>
@@ -3241,14 +3473,14 @@
         <v>15</v>
       </c>
       <c r="K16" s="7">
-        <f>L16-AB16</f>
+        <f>L16-AF16</f>
         <v/>
       </c>
       <c r="L16" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M16" s="25">
-        <f>IF(NOT(ISNUMBER(H16)),"---",IF(H16&lt;=0,"---",IF(H16*100/(Datos!$B$8*J16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H16*100/(Datos!$B$8*J16*K16^2*Datos!$B$5)))*J16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
+        <f>IF(NOT(ISNUMBER(H16)),"---",IF(H16&lt;=0,"---",IF(H16*100/(Datos!$B$8*AB16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H16*100/(Datos!$B$8*AB16*K16^2*Datos!$B$5)))*AB16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
         <v/>
       </c>
       <c r="N16" s="24" t="n">
@@ -3258,7 +3490,7 @@
         <v>12</v>
       </c>
       <c r="P16" s="25">
-        <f>IF(NOT(ISNUMBER(I16)),"---",IF(I16&lt;=0,"---",IF(I16*100/(Datos!$B$8*J16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I16*100/(Datos!$B$8*J16*K16^2*Datos!$B$5)))*J16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
+        <f>IF(NOT(ISNUMBER(I16)),"---",IF(I16&lt;=0,"---",IF(I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)))*AC16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
         <v/>
       </c>
       <c r="Q16" s="24" t="n">
@@ -3282,7 +3514,7 @@
         <v>30</v>
       </c>
       <c r="W16" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M16),N16*PI()*(O16/10)^2/4&gt;=M16,TRUE),IF(ISNUMBER(P16),Q16*PI()*(R16/10)^2/4&gt;=P16,TRUE),IF(ISNUMBER(M16),M16&lt;=0.0163*J16*K16,TRUE),IF(ISNUMBER(P16),P16&lt;=0.0163*J16*K16,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F16&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J16*K16+2*PI()*(U16/10)^2/4*Datos!$B$6*K16/V16)),"NO VERIF. CORTE",IF(NOT(L16&gt;=C16*100/VLOOKUP(Y16,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M16),N16*PI()*(O16/10)^2/4&gt;=M16,TRUE),IF(ISNUMBER(P16),Q16*PI()*(R16/10)^2/4&gt;=P16,TRUE),IF(ISNUMBER(M16),M16&lt;=0.0163*AB16*K16,TRUE),IF(ISNUMBER(P16),P16&lt;=0.0163*AC16*K16,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F16&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J16*K16+2*PI()*(U16/10)^2/4*Datos!$B$6*K16/V16)),"NO VERIF. CORTE",IF(NOT(L16&gt;=C16*100/VLOOKUP(Y16,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X16" s="7" t="n"/>
@@ -3291,13 +3523,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z16" s="24" t="n">
+      <c r="Z16" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA16" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB16" s="7">
+        <f>IF(Z16="Colgante",MIN(C16*100/4,J16+16*AA16),J16)</f>
+        <v/>
+      </c>
+      <c r="AC16" s="7">
+        <f>IF(Z16="Invertida",MIN(C16*100/4,J16+16*AA16),J16)</f>
+        <v/>
+      </c>
+      <c r="AD16" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA16" s="24" t="n">
+      <c r="AE16" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB16" s="24" t="n">
+      <c r="AF16" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3312,7 +3560,7 @@
         <v>4</v>
       </c>
       <c r="D17" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AA17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z17)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AE17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD17)</f>
         <v/>
       </c>
       <c r="E17" s="7" t="n"/>
@@ -3336,14 +3584,14 @@
         <v>15</v>
       </c>
       <c r="K17" s="7">
-        <f>L17-AB17</f>
+        <f>L17-AF17</f>
         <v/>
       </c>
       <c r="L17" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M17" s="25">
-        <f>IF(NOT(ISNUMBER(H17)),"---",IF(H17&lt;=0,"---",IF(H17*100/(Datos!$B$8*J17*K17^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H17*100/(Datos!$B$8*J17*K17^2*Datos!$B$5)))*J17*K17*Datos!$B$5/Datos!$B$6,0.0033*J17*K17))))</f>
+        <f>IF(NOT(ISNUMBER(H17)),"---",IF(H17&lt;=0,"---",IF(H17*100/(Datos!$B$8*AB17*K17^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H17*100/(Datos!$B$8*AB17*K17^2*Datos!$B$5)))*AB17*K17*Datos!$B$5/Datos!$B$6,0.0033*J17*K17))))</f>
         <v/>
       </c>
       <c r="N17" s="24" t="n">
@@ -3353,7 +3601,7 @@
         <v>12</v>
       </c>
       <c r="P17" s="25">
-        <f>IF(NOT(ISNUMBER(I17)),"---",IF(I17&lt;=0,"---",IF(I17*100/(Datos!$B$8*J17*K17^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I17*100/(Datos!$B$8*J17*K17^2*Datos!$B$5)))*J17*K17*Datos!$B$5/Datos!$B$6,0.0033*J17*K17))))</f>
+        <f>IF(NOT(ISNUMBER(I17)),"---",IF(I17&lt;=0,"---",IF(I17*100/(Datos!$B$8*AC17*K17^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I17*100/(Datos!$B$8*AC17*K17^2*Datos!$B$5)))*AC17*K17*Datos!$B$5/Datos!$B$6,0.0033*J17*K17))))</f>
         <v/>
       </c>
       <c r="Q17" s="24" t="n">
@@ -3377,7 +3625,7 @@
         <v>30</v>
       </c>
       <c r="W17" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M17),N17*PI()*(O17/10)^2/4&gt;=M17,TRUE),IF(ISNUMBER(P17),Q17*PI()*(R17/10)^2/4&gt;=P17,TRUE),IF(ISNUMBER(M17),M17&lt;=0.0163*J17*K17,TRUE),IF(ISNUMBER(P17),P17&lt;=0.0163*J17*K17,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F17&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J17*K17+2*PI()*(U17/10)^2/4*Datos!$B$6*K17/V17)),"NO VERIF. CORTE",IF(NOT(L17&gt;=C17*100/VLOOKUP(Y17,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M17),N17*PI()*(O17/10)^2/4&gt;=M17,TRUE),IF(ISNUMBER(P17),Q17*PI()*(R17/10)^2/4&gt;=P17,TRUE),IF(ISNUMBER(M17),M17&lt;=0.0163*AB17*K17,TRUE),IF(ISNUMBER(P17),P17&lt;=0.0163*AC17*K17,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F17&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J17*K17+2*PI()*(U17/10)^2/4*Datos!$B$6*K17/V17)),"NO VERIF. CORTE",IF(NOT(L17&gt;=C17*100/VLOOKUP(Y17,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X17" s="7" t="n"/>
@@ -3386,13 +3634,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z17" s="24" t="n">
+      <c r="Z17" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA17" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB17" s="7">
+        <f>IF(Z17="Colgante",MIN(C17*100/4,J17+16*AA17),J17)</f>
+        <v/>
+      </c>
+      <c r="AC17" s="7">
+        <f>IF(Z17="Invertida",MIN(C17*100/4,J17+16*AA17),J17)</f>
+        <v/>
+      </c>
+      <c r="AD17" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA17" s="24" t="n">
+      <c r="AE17" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB17" s="24" t="n">
+      <c r="AF17" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3407,7 +3671,7 @@
         <v>3.6</v>
       </c>
       <c r="D18" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AA18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z18)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AE18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD18)</f>
         <v/>
       </c>
       <c r="E18" s="7" t="n"/>
@@ -3431,14 +3695,14 @@
         <v>15</v>
       </c>
       <c r="K18" s="7">
-        <f>L18-AB18</f>
+        <f>L18-AF18</f>
         <v/>
       </c>
       <c r="L18" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M18" s="25">
-        <f>IF(NOT(ISNUMBER(H18)),"---",IF(H18&lt;=0,"---",IF(H18*100/(Datos!$B$8*J18*K18^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H18*100/(Datos!$B$8*J18*K18^2*Datos!$B$5)))*J18*K18*Datos!$B$5/Datos!$B$6,0.0033*J18*K18))))</f>
+        <f>IF(NOT(ISNUMBER(H18)),"---",IF(H18&lt;=0,"---",IF(H18*100/(Datos!$B$8*AB18*K18^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H18*100/(Datos!$B$8*AB18*K18^2*Datos!$B$5)))*AB18*K18*Datos!$B$5/Datos!$B$6,0.0033*J18*K18))))</f>
         <v/>
       </c>
       <c r="N18" s="24" t="n">
@@ -3448,7 +3712,7 @@
         <v>12</v>
       </c>
       <c r="P18" s="25">
-        <f>IF(NOT(ISNUMBER(I18)),"---",IF(I18&lt;=0,"---",IF(I18*100/(Datos!$B$8*J18*K18^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I18*100/(Datos!$B$8*J18*K18^2*Datos!$B$5)))*J18*K18*Datos!$B$5/Datos!$B$6,0.0033*J18*K18))))</f>
+        <f>IF(NOT(ISNUMBER(I18)),"---",IF(I18&lt;=0,"---",IF(I18*100/(Datos!$B$8*AC18*K18^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I18*100/(Datos!$B$8*AC18*K18^2*Datos!$B$5)))*AC18*K18*Datos!$B$5/Datos!$B$6,0.0033*J18*K18))))</f>
         <v/>
       </c>
       <c r="Q18" s="24" t="n">
@@ -3472,7 +3736,7 @@
         <v>30</v>
       </c>
       <c r="W18" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M18),N18*PI()*(O18/10)^2/4&gt;=M18,TRUE),IF(ISNUMBER(P18),Q18*PI()*(R18/10)^2/4&gt;=P18,TRUE),IF(ISNUMBER(M18),M18&lt;=0.0163*J18*K18,TRUE),IF(ISNUMBER(P18),P18&lt;=0.0163*J18*K18,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F18&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J18*K18+2*PI()*(U18/10)^2/4*Datos!$B$6*K18/V18)),"NO VERIF. CORTE",IF(NOT(L18&gt;=C18*100/VLOOKUP(Y18,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M18),N18*PI()*(O18/10)^2/4&gt;=M18,TRUE),IF(ISNUMBER(P18),Q18*PI()*(R18/10)^2/4&gt;=P18,TRUE),IF(ISNUMBER(M18),M18&lt;=0.0163*AB18*K18,TRUE),IF(ISNUMBER(P18),P18&lt;=0.0163*AC18*K18,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F18&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J18*K18+2*PI()*(U18/10)^2/4*Datos!$B$6*K18/V18)),"NO VERIF. CORTE",IF(NOT(L18&gt;=C18*100/VLOOKUP(Y18,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X18" s="7" t="n"/>
@@ -3481,13 +3745,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z18" s="24" t="n">
+      <c r="Z18" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA18" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB18" s="7">
+        <f>IF(Z18="Colgante",MIN(C18*100/4,J18+16*AA18),J18)</f>
+        <v/>
+      </c>
+      <c r="AC18" s="7">
+        <f>IF(Z18="Invertida",MIN(C18*100/4,J18+16*AA18),J18)</f>
+        <v/>
+      </c>
+      <c r="AD18" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA18" s="24" t="n">
+      <c r="AE18" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB18" s="24" t="n">
+      <c r="AF18" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3502,7 +3782,7 @@
         <v>7.68</v>
       </c>
       <c r="D19" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AA19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z19)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AE19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD19)</f>
         <v/>
       </c>
       <c r="E19" s="7" t="n"/>
@@ -3526,14 +3806,14 @@
         <v>15</v>
       </c>
       <c r="K19" s="7">
-        <f>L19-AB19</f>
+        <f>L19-AF19</f>
         <v/>
       </c>
       <c r="L19" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M19" s="25">
-        <f>IF(NOT(ISNUMBER(H19)),"---",IF(H19&lt;=0,"---",IF(H19*100/(Datos!$B$8*J19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H19*100/(Datos!$B$8*J19*K19^2*Datos!$B$5)))*J19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
+        <f>IF(NOT(ISNUMBER(H19)),"---",IF(H19&lt;=0,"---",IF(H19*100/(Datos!$B$8*AB19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H19*100/(Datos!$B$8*AB19*K19^2*Datos!$B$5)))*AB19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
         <v/>
       </c>
       <c r="N19" s="24" t="n">
@@ -3543,7 +3823,7 @@
         <v>20</v>
       </c>
       <c r="P19" s="25">
-        <f>IF(NOT(ISNUMBER(I19)),"---",IF(I19&lt;=0,"---",IF(I19*100/(Datos!$B$8*J19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I19*100/(Datos!$B$8*J19*K19^2*Datos!$B$5)))*J19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
+        <f>IF(NOT(ISNUMBER(I19)),"---",IF(I19&lt;=0,"---",IF(I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)))*AC19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
         <v/>
       </c>
       <c r="Q19" s="24" t="n">
@@ -3564,29 +3844,45 @@
         <v>6</v>
       </c>
       <c r="V19" s="24" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="W19" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*J19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*J19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X19" s="26" t="inlineStr">
         <is>
-          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Confirmar en el DWG.</t>
+          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
         </is>
       </c>
       <c r="Y19" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
-        </is>
-      </c>
-      <c r="Z19" s="24" t="n">
+          <t>Empotrada-apoyada</t>
+        </is>
+      </c>
+      <c r="Z19" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA19" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB19" s="7">
+        <f>IF(Z19="Colgante",MIN(C19*100/4,J19+16*AA19),J19)</f>
+        <v/>
+      </c>
+      <c r="AC19" s="7">
+        <f>IF(Z19="Invertida",MIN(C19*100/4,J19+16*AA19),J19)</f>
+        <v/>
+      </c>
+      <c r="AD19" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA19" s="24" t="n">
+      <c r="AE19" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB19" s="24" t="n">
+      <c r="AF19" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3601,7 +3897,7 @@
         <v>3.45</v>
       </c>
       <c r="D20" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AA20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z20)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AE20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD20)</f>
         <v/>
       </c>
       <c r="E20" s="7" t="n"/>
@@ -3625,14 +3921,14 @@
         <v>15</v>
       </c>
       <c r="K20" s="7">
-        <f>L20-AB20</f>
+        <f>L20-AF20</f>
         <v/>
       </c>
       <c r="L20" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M20" s="25">
-        <f>IF(NOT(ISNUMBER(H20)),"---",IF(H20&lt;=0,"---",IF(H20*100/(Datos!$B$8*J20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H20*100/(Datos!$B$8*J20*K20^2*Datos!$B$5)))*J20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
+        <f>IF(NOT(ISNUMBER(H20)),"---",IF(H20&lt;=0,"---",IF(H20*100/(Datos!$B$8*AB20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H20*100/(Datos!$B$8*AB20*K20^2*Datos!$B$5)))*AB20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
         <v/>
       </c>
       <c r="N20" s="24" t="n">
@@ -3642,7 +3938,7 @@
         <v>12</v>
       </c>
       <c r="P20" s="25">
-        <f>IF(NOT(ISNUMBER(I20)),"---",IF(I20&lt;=0,"---",IF(I20*100/(Datos!$B$8*J20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I20*100/(Datos!$B$8*J20*K20^2*Datos!$B$5)))*J20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
+        <f>IF(NOT(ISNUMBER(I20)),"---",IF(I20&lt;=0,"---",IF(I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)))*AC20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
         <v/>
       </c>
       <c r="Q20" s="24" t="n">
@@ -3666,22 +3962,42 @@
         <v>30</v>
       </c>
       <c r="W20" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*J20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*J20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X20" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X20" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y20" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z20" s="24" t="n">
+      <c r="Z20" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA20" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB20" s="7">
+        <f>IF(Z20="Colgante",MIN(C20*100/4,J20+16*AA20),J20)</f>
+        <v/>
+      </c>
+      <c r="AC20" s="7">
+        <f>IF(Z20="Invertida",MIN(C20*100/4,J20+16*AA20),J20)</f>
+        <v/>
+      </c>
+      <c r="AD20" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA20" s="24" t="n">
+      <c r="AE20" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB20" s="24" t="n">
+      <c r="AF20" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3696,7 +4012,7 @@
         <v>5.02</v>
       </c>
       <c r="D21" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AA21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z21)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AE21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD21)</f>
         <v/>
       </c>
       <c r="E21" s="7" t="n"/>
@@ -3720,14 +4036,14 @@
         <v>15</v>
       </c>
       <c r="K21" s="7">
-        <f>L21-AB21</f>
+        <f>L21-AF21</f>
         <v/>
       </c>
       <c r="L21" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M21" s="25">
-        <f>IF(NOT(ISNUMBER(H21)),"---",IF(H21&lt;=0,"---",IF(H21*100/(Datos!$B$8*J21*K21^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H21*100/(Datos!$B$8*J21*K21^2*Datos!$B$5)))*J21*K21*Datos!$B$5/Datos!$B$6,0.0033*J21*K21))))</f>
+        <f>IF(NOT(ISNUMBER(H21)),"---",IF(H21&lt;=0,"---",IF(H21*100/(Datos!$B$8*AB21*K21^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H21*100/(Datos!$B$8*AB21*K21^2*Datos!$B$5)))*AB21*K21*Datos!$B$5/Datos!$B$6,0.0033*J21*K21))))</f>
         <v/>
       </c>
       <c r="N21" s="24" t="n">
@@ -3737,7 +4053,7 @@
         <v>12</v>
       </c>
       <c r="P21" s="25">
-        <f>IF(NOT(ISNUMBER(I21)),"---",IF(I21&lt;=0,"---",IF(I21*100/(Datos!$B$8*J21*K21^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I21*100/(Datos!$B$8*J21*K21^2*Datos!$B$5)))*J21*K21*Datos!$B$5/Datos!$B$6,0.0033*J21*K21))))</f>
+        <f>IF(NOT(ISNUMBER(I21)),"---",IF(I21&lt;=0,"---",IF(I21*100/(Datos!$B$8*AC21*K21^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I21*100/(Datos!$B$8*AC21*K21^2*Datos!$B$5)))*AC21*K21*Datos!$B$5/Datos!$B$6,0.0033*J21*K21))))</f>
         <v/>
       </c>
       <c r="Q21" s="24" t="n">
@@ -3761,22 +4077,42 @@
         <v>30</v>
       </c>
       <c r="W21" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M21),N21*PI()*(O21/10)^2/4&gt;=M21,TRUE),IF(ISNUMBER(P21),Q21*PI()*(R21/10)^2/4&gt;=P21,TRUE),IF(ISNUMBER(M21),M21&lt;=0.0163*J21*K21,TRUE),IF(ISNUMBER(P21),P21&lt;=0.0163*J21*K21,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F21&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J21*K21+2*PI()*(U21/10)^2/4*Datos!$B$6*K21/V21)),"NO VERIF. CORTE",IF(NOT(L21&gt;=C21*100/VLOOKUP(Y21,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X21" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M21),N21*PI()*(O21/10)^2/4&gt;=M21,TRUE),IF(ISNUMBER(P21),Q21*PI()*(R21/10)^2/4&gt;=P21,TRUE),IF(ISNUMBER(M21),M21&lt;=0.0163*AB21*K21,TRUE),IF(ISNUMBER(P21),P21&lt;=0.0163*AC21*K21,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F21&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J21*K21+2*PI()*(U21/10)^2/4*Datos!$B$6*K21/V21)),"NO VERIF. CORTE",IF(NOT(L21&gt;=C21*100/VLOOKUP(Y21,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X21" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y21" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z21" s="24" t="n">
+      <c r="Z21" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA21" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB21" s="7">
+        <f>IF(Z21="Colgante",MIN(C21*100/4,J21+16*AA21),J21)</f>
+        <v/>
+      </c>
+      <c r="AC21" s="7">
+        <f>IF(Z21="Invertida",MIN(C21*100/4,J21+16*AA21),J21)</f>
+        <v/>
+      </c>
+      <c r="AD21" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA21" s="24" t="n">
+      <c r="AE21" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB21" s="24" t="n">
+      <c r="AF21" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3791,7 +4127,7 @@
         <v>3.71</v>
       </c>
       <c r="D22" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AA22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z22)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AE22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD22)</f>
         <v/>
       </c>
       <c r="E22" s="7" t="n"/>
@@ -3815,14 +4151,14 @@
         <v>40</v>
       </c>
       <c r="K22" s="7">
-        <f>L22-AB22</f>
+        <f>L22-AF22</f>
         <v/>
       </c>
       <c r="L22" s="24" t="n">
         <v>13</v>
       </c>
       <c r="M22" s="25">
-        <f>IF(NOT(ISNUMBER(H22)),"---",IF(H22&lt;=0,"---",IF(H22*100/(Datos!$B$8*J22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H22*100/(Datos!$B$8*J22*K22^2*Datos!$B$5)))*J22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
+        <f>IF(NOT(ISNUMBER(H22)),"---",IF(H22&lt;=0,"---",IF(H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)))*AB22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="N22" s="24" t="n">
@@ -3832,7 +4168,7 @@
         <v>8</v>
       </c>
       <c r="P22" s="25">
-        <f>IF(NOT(ISNUMBER(I22)),"---",IF(I22&lt;=0,"---",IF(I22*100/(Datos!$B$8*J22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I22*100/(Datos!$B$8*J22*K22^2*Datos!$B$5)))*J22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
+        <f>IF(NOT(ISNUMBER(I22)),"---",IF(I22&lt;=0,"---",IF(I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)))*AC22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="Q22" s="24" t="n">
@@ -3856,7 +4192,7 @@
         <v>5</v>
       </c>
       <c r="W22" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*J22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*J22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X22" s="26" t="inlineStr">
@@ -3869,13 +4205,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z22" s="24" t="n">
+      <c r="Z22" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA22" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB22" s="7">
+        <f>IF(Z22="Colgante",MIN(C22*100/4,J22+16*AA22),J22)</f>
+        <v/>
+      </c>
+      <c r="AC22" s="7">
+        <f>IF(Z22="Invertida",MIN(C22*100/4,J22+16*AA22),J22)</f>
+        <v/>
+      </c>
+      <c r="AD22" s="24" t="n">
         <v>0.6</v>
       </c>
-      <c r="AA22" s="24" t="n">
+      <c r="AE22" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB22" s="24" t="n">
+      <c r="AF22" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3890,7 +4242,7 @@
         <v>2.13</v>
       </c>
       <c r="D23" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AA23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z23)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AE23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD23)</f>
         <v/>
       </c>
       <c r="E23" s="7" t="n"/>
@@ -3914,14 +4266,14 @@
         <v>40</v>
       </c>
       <c r="K23" s="7">
-        <f>L23-AB23</f>
+        <f>L23-AF23</f>
         <v/>
       </c>
       <c r="L23" s="24" t="n">
         <v>13</v>
       </c>
       <c r="M23" s="25">
-        <f>IF(NOT(ISNUMBER(H23)),"---",IF(H23&lt;=0,"---",IF(H23*100/(Datos!$B$8*J23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H23*100/(Datos!$B$8*J23*K23^2*Datos!$B$5)))*J23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
+        <f>IF(NOT(ISNUMBER(H23)),"---",IF(H23&lt;=0,"---",IF(H23*100/(Datos!$B$8*AB23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H23*100/(Datos!$B$8*AB23*K23^2*Datos!$B$5)))*AB23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="N23" s="24" t="n">
@@ -3931,7 +4283,7 @@
         <v>6</v>
       </c>
       <c r="P23" s="25">
-        <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos!$B$8*J23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos!$B$8*J23*K23^2*Datos!$B$5)))*J23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
+        <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)))*AC23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="Q23" s="24" t="n">
@@ -3955,7 +4307,7 @@
         <v>5</v>
       </c>
       <c r="W23" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M23),N23*PI()*(O23/10)^2/4&gt;=M23,TRUE),IF(ISNUMBER(P23),Q23*PI()*(R23/10)^2/4&gt;=P23,TRUE),IF(ISNUMBER(M23),M23&lt;=0.0163*J23*K23,TRUE),IF(ISNUMBER(P23),P23&lt;=0.0163*J23*K23,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F23&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J23*K23+2*PI()*(U23/10)^2/4*Datos!$B$6*K23/V23)),"NO VERIF. CORTE",IF(NOT(L23&gt;=C23*100/VLOOKUP(Y23,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M23),N23*PI()*(O23/10)^2/4&gt;=M23,TRUE),IF(ISNUMBER(P23),Q23*PI()*(R23/10)^2/4&gt;=P23,TRUE),IF(ISNUMBER(M23),M23&lt;=0.0163*AB23*K23,TRUE),IF(ISNUMBER(P23),P23&lt;=0.0163*AC23*K23,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F23&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J23*K23+2*PI()*(U23/10)^2/4*Datos!$B$6*K23/V23)),"NO VERIF. CORTE",IF(NOT(L23&gt;=C23*100/VLOOKUP(Y23,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X23" s="26" t="inlineStr">
@@ -3968,13 +4320,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z23" s="24" t="n">
+      <c r="Z23" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA23" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB23" s="7">
+        <f>IF(Z23="Colgante",MIN(C23*100/4,J23+16*AA23),J23)</f>
+        <v/>
+      </c>
+      <c r="AC23" s="7">
+        <f>IF(Z23="Invertida",MIN(C23*100/4,J23+16*AA23),J23)</f>
+        <v/>
+      </c>
+      <c r="AD23" s="24" t="n">
         <v>0.6</v>
       </c>
-      <c r="AA23" s="24" t="n">
+      <c r="AE23" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB23" s="24" t="n">
+      <c r="AF23" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3989,7 +4357,7 @@
         <v>3.71</v>
       </c>
       <c r="D24" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*Z24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AA24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*Z24)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
         <v/>
       </c>
       <c r="E24" s="32" t="n"/>
@@ -4013,14 +4381,14 @@
         <v>12</v>
       </c>
       <c r="K24" s="32">
-        <f>L24-AB24</f>
+        <f>L24-AF24</f>
         <v/>
       </c>
       <c r="L24" s="33" t="n">
         <v>45</v>
       </c>
       <c r="M24" s="34">
-        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*J24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*J24*K24^2*Datos!$B$5)))*J24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
         <v/>
       </c>
       <c r="N24" s="33" t="n">
@@ -4030,7 +4398,7 @@
         <v>12</v>
       </c>
       <c r="P24" s="34">
-        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*J24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*J24*K24^2*Datos!$B$5)))*J24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
         <v/>
       </c>
       <c r="Q24" s="33" t="inlineStr">
@@ -4058,7 +4426,7 @@
         <v>20</v>
       </c>
       <c r="W24" s="32">
-        <f>IF(NOT(AND(IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*J24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*J24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X24" s="32" t="n"/>
@@ -4067,13 +4435,29 @@
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z24" s="33" t="n">
+      <c r="Z24" s="33" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA24" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB24" s="32">
+        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="32">
+        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AD24" s="33" t="n">
         <v>0.6</v>
       </c>
-      <c r="AA24" s="33" t="n">
+      <c r="AE24" s="33" t="n">
         <v>2.6</v>
       </c>
-      <c r="AB24" s="33" t="n">
+      <c r="AF24" s="33" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4092,7 +4476,7 @@
         <v>9.9</v>
       </c>
       <c r="D25" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AA25)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z25)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD25)</f>
         <v/>
       </c>
       <c r="E25" s="7" t="n"/>
@@ -4116,14 +4500,14 @@
         <v>15</v>
       </c>
       <c r="K25" s="7">
-        <f>L25-AB25</f>
+        <f>L25-AF25</f>
         <v/>
       </c>
       <c r="L25" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M25" s="25">
-        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*J25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*J25*K25^2*Datos!$B$5)))*J25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
         <v/>
       </c>
       <c r="N25" s="24" t="n">
@@ -4133,7 +4517,7 @@
         <v>25</v>
       </c>
       <c r="P25" s="25">
-        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*J25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*J25*K25^2*Datos!$B$5)))*J25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
         <v/>
       </c>
       <c r="Q25" s="24" t="n">
@@ -4157,7 +4541,7 @@
         <v>15</v>
       </c>
       <c r="W25" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*J25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*J25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X25" s="7" t="n"/>
@@ -4166,13 +4550,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z25" s="24" t="n">
+      <c r="Z25" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA25" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB25" s="7">
+        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="7">
+        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AD25" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA25" s="24" t="n">
+      <c r="AE25" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB25" s="24" t="n">
+      <c r="AF25" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4187,7 +4587,7 @@
         <v>6</v>
       </c>
       <c r="D26" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AA26)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z26)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD26)</f>
         <v/>
       </c>
       <c r="E26" s="7" t="n"/>
@@ -4211,14 +4611,14 @@
         <v>15</v>
       </c>
       <c r="K26" s="7">
-        <f>L26-AB26</f>
+        <f>L26-AF26</f>
         <v/>
       </c>
       <c r="L26" s="24" t="n">
         <v>50</v>
       </c>
       <c r="M26" s="25">
-        <f>IF(NOT(ISNUMBER(H26)),"---",IF(H26&lt;=0,"---",IF(H26*100/(Datos!$B$8*J26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H26*100/(Datos!$B$8*J26*K26^2*Datos!$B$5)))*J26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
+        <f>IF(NOT(ISNUMBER(H26)),"---",IF(H26&lt;=0,"---",IF(H26*100/(Datos!$B$8*AB26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H26*100/(Datos!$B$8*AB26*K26^2*Datos!$B$5)))*AB26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
         <v/>
       </c>
       <c r="N26" s="24" t="n">
@@ -4228,7 +4628,7 @@
         <v>12</v>
       </c>
       <c r="P26" s="25">
-        <f>IF(NOT(ISNUMBER(I26)),"---",IF(I26&lt;=0,"---",IF(I26*100/(Datos!$B$8*J26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I26*100/(Datos!$B$8*J26*K26^2*Datos!$B$5)))*J26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
+        <f>IF(NOT(ISNUMBER(I26)),"---",IF(I26&lt;=0,"---",IF(I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)))*AC26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
         <v/>
       </c>
       <c r="Q26" s="24" t="n">
@@ -4252,7 +4652,7 @@
         <v>20</v>
       </c>
       <c r="W26" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*J26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*J26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*AB26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*AC26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X26" s="7" t="n"/>
@@ -4261,13 +4661,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z26" s="24" t="n">
+      <c r="Z26" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA26" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB26" s="7">
+        <f>IF(Z26="Colgante",MIN(C26*100/4,J26+16*AA26),J26)</f>
+        <v/>
+      </c>
+      <c r="AC26" s="7">
+        <f>IF(Z26="Invertida",MIN(C26*100/4,J26+16*AA26),J26)</f>
+        <v/>
+      </c>
+      <c r="AD26" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA26" s="24" t="n">
+      <c r="AE26" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB26" s="24" t="n">
+      <c r="AF26" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4282,7 +4698,7 @@
         <v>3.75</v>
       </c>
       <c r="D27" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AA27)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z27)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD27)</f>
         <v/>
       </c>
       <c r="E27" s="7" t="n"/>
@@ -4306,14 +4722,14 @@
         <v>15</v>
       </c>
       <c r="K27" s="7">
-        <f>L27-AB27</f>
+        <f>L27-AF27</f>
         <v/>
       </c>
       <c r="L27" s="24" t="n">
         <v>50</v>
       </c>
       <c r="M27" s="25">
-        <f>IF(NOT(ISNUMBER(H27)),"---",IF(H27&lt;=0,"---",IF(H27*100/(Datos!$B$8*J27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H27*100/(Datos!$B$8*J27*K27^2*Datos!$B$5)))*J27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
+        <f>IF(NOT(ISNUMBER(H27)),"---",IF(H27&lt;=0,"---",IF(H27*100/(Datos!$B$8*AB27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H27*100/(Datos!$B$8*AB27*K27^2*Datos!$B$5)))*AB27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="N27" s="24" t="n">
@@ -4323,7 +4739,7 @@
         <v>10</v>
       </c>
       <c r="P27" s="25">
-        <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos!$B$8*J27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos!$B$8*J27*K27^2*Datos!$B$5)))*J27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
+        <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)))*AC27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="Q27" s="24" t="n">
@@ -4347,7 +4763,7 @@
         <v>20</v>
       </c>
       <c r="W27" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*J27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*J27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X27" s="7" t="n"/>
@@ -4356,13 +4772,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z27" s="24" t="n">
+      <c r="Z27" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA27" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB27" s="7">
+        <f>IF(Z27="Colgante",MIN(C27*100/4,J27+16*AA27),J27)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="7">
+        <f>IF(Z27="Invertida",MIN(C27*100/4,J27+16*AA27),J27)</f>
+        <v/>
+      </c>
+      <c r="AD27" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA27" s="24" t="n">
+      <c r="AE27" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB27" s="24" t="n">
+      <c r="AF27" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4377,7 +4809,7 @@
         <v>6</v>
       </c>
       <c r="D28" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AA28)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z28)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD28)</f>
         <v/>
       </c>
       <c r="E28" s="7" t="n"/>
@@ -4401,14 +4833,14 @@
         <v>15</v>
       </c>
       <c r="K28" s="7">
-        <f>L28-AB28</f>
+        <f>L28-AF28</f>
         <v/>
       </c>
       <c r="L28" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M28" s="25">
-        <f>IF(NOT(ISNUMBER(H28)),"---",IF(H28&lt;=0,"---",IF(H28*100/(Datos!$B$8*J28*K28^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H28*100/(Datos!$B$8*J28*K28^2*Datos!$B$5)))*J28*K28*Datos!$B$5/Datos!$B$6,0.0033*J28*K28))))</f>
+        <f>IF(NOT(ISNUMBER(H28)),"---",IF(H28&lt;=0,"---",IF(H28*100/(Datos!$B$8*AB28*K28^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H28*100/(Datos!$B$8*AB28*K28^2*Datos!$B$5)))*AB28*K28*Datos!$B$5/Datos!$B$6,0.0033*J28*K28))))</f>
         <v/>
       </c>
       <c r="N28" s="24" t="n">
@@ -4418,7 +4850,7 @@
         <v>12</v>
       </c>
       <c r="P28" s="25">
-        <f>IF(NOT(ISNUMBER(I28)),"---",IF(I28&lt;=0,"---",IF(I28*100/(Datos!$B$8*J28*K28^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I28*100/(Datos!$B$8*J28*K28^2*Datos!$B$5)))*J28*K28*Datos!$B$5/Datos!$B$6,0.0033*J28*K28))))</f>
+        <f>IF(NOT(ISNUMBER(I28)),"---",IF(I28&lt;=0,"---",IF(I28*100/(Datos!$B$8*AC28*K28^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I28*100/(Datos!$B$8*AC28*K28^2*Datos!$B$5)))*AC28*K28*Datos!$B$5/Datos!$B$6,0.0033*J28*K28))))</f>
         <v/>
       </c>
       <c r="Q28" s="24" t="n">
@@ -4442,7 +4874,7 @@
         <v>30</v>
       </c>
       <c r="W28" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M28),N28*PI()*(O28/10)^2/4&gt;=M28,TRUE),IF(ISNUMBER(P28),Q28*PI()*(R28/10)^2/4&gt;=P28,TRUE),IF(ISNUMBER(M28),M28&lt;=0.0163*J28*K28,TRUE),IF(ISNUMBER(P28),P28&lt;=0.0163*J28*K28,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F28&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J28*K28+2*PI()*(U28/10)^2/4*Datos!$B$6*K28/V28)),"NO VERIF. CORTE",IF(NOT(L28&gt;=C28*100/VLOOKUP(Y28,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M28),N28*PI()*(O28/10)^2/4&gt;=M28,TRUE),IF(ISNUMBER(P28),Q28*PI()*(R28/10)^2/4&gt;=P28,TRUE),IF(ISNUMBER(M28),M28&lt;=0.0163*AB28*K28,TRUE),IF(ISNUMBER(P28),P28&lt;=0.0163*AC28*K28,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F28&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J28*K28+2*PI()*(U28/10)^2/4*Datos!$B$6*K28/V28)),"NO VERIF. CORTE",IF(NOT(L28&gt;=C28*100/VLOOKUP(Y28,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X28" s="7" t="n"/>
@@ -4451,13 +4883,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z28" s="24" t="n">
+      <c r="Z28" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA28" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB28" s="7">
+        <f>IF(Z28="Colgante",MIN(C28*100/4,J28+16*AA28),J28)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="7">
+        <f>IF(Z28="Invertida",MIN(C28*100/4,J28+16*AA28),J28)</f>
+        <v/>
+      </c>
+      <c r="AD28" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA28" s="24" t="n">
+      <c r="AE28" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB28" s="24" t="n">
+      <c r="AF28" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4472,7 +4920,7 @@
         <v>4.03</v>
       </c>
       <c r="D29" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AA29)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z29)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD29)</f>
         <v/>
       </c>
       <c r="E29" s="7" t="n"/>
@@ -4496,14 +4944,14 @@
         <v>15</v>
       </c>
       <c r="K29" s="7">
-        <f>L29-AB29</f>
+        <f>L29-AF29</f>
         <v/>
       </c>
       <c r="L29" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M29" s="25">
-        <f>IF(NOT(ISNUMBER(H29)),"---",IF(H29&lt;=0,"---",IF(H29*100/(Datos!$B$8*J29*K29^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H29*100/(Datos!$B$8*J29*K29^2*Datos!$B$5)))*J29*K29*Datos!$B$5/Datos!$B$6,0.0033*J29*K29))))</f>
+        <f>IF(NOT(ISNUMBER(H29)),"---",IF(H29&lt;=0,"---",IF(H29*100/(Datos!$B$8*AB29*K29^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H29*100/(Datos!$B$8*AB29*K29^2*Datos!$B$5)))*AB29*K29*Datos!$B$5/Datos!$B$6,0.0033*J29*K29))))</f>
         <v/>
       </c>
       <c r="N29" s="24" t="n">
@@ -4513,7 +4961,7 @@
         <v>12</v>
       </c>
       <c r="P29" s="25">
-        <f>IF(NOT(ISNUMBER(I29)),"---",IF(I29&lt;=0,"---",IF(I29*100/(Datos!$B$8*J29*K29^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I29*100/(Datos!$B$8*J29*K29^2*Datos!$B$5)))*J29*K29*Datos!$B$5/Datos!$B$6,0.0033*J29*K29))))</f>
+        <f>IF(NOT(ISNUMBER(I29)),"---",IF(I29&lt;=0,"---",IF(I29*100/(Datos!$B$8*AC29*K29^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I29*100/(Datos!$B$8*AC29*K29^2*Datos!$B$5)))*AC29*K29*Datos!$B$5/Datos!$B$6,0.0033*J29*K29))))</f>
         <v/>
       </c>
       <c r="Q29" s="24" t="n">
@@ -4537,22 +4985,42 @@
         <v>30</v>
       </c>
       <c r="W29" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*J29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*J29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X29" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X29" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y29" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z29" s="24" t="n">
+      <c r="Z29" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA29" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB29" s="7">
+        <f>IF(Z29="Colgante",MIN(C29*100/4,J29+16*AA29),J29)</f>
+        <v/>
+      </c>
+      <c r="AC29" s="7">
+        <f>IF(Z29="Invertida",MIN(C29*100/4,J29+16*AA29),J29)</f>
+        <v/>
+      </c>
+      <c r="AD29" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA29" s="24" t="n">
+      <c r="AE29" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB29" s="24" t="n">
+      <c r="AF29" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4567,7 +5035,7 @@
         <v>4.85</v>
       </c>
       <c r="D30" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AA30)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z30)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD30)</f>
         <v/>
       </c>
       <c r="E30" s="7" t="n"/>
@@ -4591,14 +5059,14 @@
         <v>15</v>
       </c>
       <c r="K30" s="7">
-        <f>L30-AB30</f>
+        <f>L30-AF30</f>
         <v/>
       </c>
       <c r="L30" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M30" s="25">
-        <f>IF(NOT(ISNUMBER(H30)),"---",IF(H30&lt;=0,"---",IF(H30*100/(Datos!$B$8*J30*K30^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H30*100/(Datos!$B$8*J30*K30^2*Datos!$B$5)))*J30*K30*Datos!$B$5/Datos!$B$6,0.0033*J30*K30))))</f>
+        <f>IF(NOT(ISNUMBER(H30)),"---",IF(H30&lt;=0,"---",IF(H30*100/(Datos!$B$8*AB30*K30^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H30*100/(Datos!$B$8*AB30*K30^2*Datos!$B$5)))*AB30*K30*Datos!$B$5/Datos!$B$6,0.0033*J30*K30))))</f>
         <v/>
       </c>
       <c r="N30" s="24" t="n">
@@ -4608,7 +5076,7 @@
         <v>12</v>
       </c>
       <c r="P30" s="25">
-        <f>IF(NOT(ISNUMBER(I30)),"---",IF(I30&lt;=0,"---",IF(I30*100/(Datos!$B$8*J30*K30^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I30*100/(Datos!$B$8*J30*K30^2*Datos!$B$5)))*J30*K30*Datos!$B$5/Datos!$B$6,0.0033*J30*K30))))</f>
+        <f>IF(NOT(ISNUMBER(I30)),"---",IF(I30&lt;=0,"---",IF(I30*100/(Datos!$B$8*AC30*K30^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I30*100/(Datos!$B$8*AC30*K30^2*Datos!$B$5)))*AC30*K30*Datos!$B$5/Datos!$B$6,0.0033*J30*K30))))</f>
         <v/>
       </c>
       <c r="Q30" s="24" t="n">
@@ -4632,22 +5100,42 @@
         <v>30</v>
       </c>
       <c r="W30" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M30),N30*PI()*(O30/10)^2/4&gt;=M30,TRUE),IF(ISNUMBER(P30),Q30*PI()*(R30/10)^2/4&gt;=P30,TRUE),IF(ISNUMBER(M30),M30&lt;=0.0163*J30*K30,TRUE),IF(ISNUMBER(P30),P30&lt;=0.0163*J30*K30,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F30&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J30*K30+2*PI()*(U30/10)^2/4*Datos!$B$6*K30/V30)),"NO VERIF. CORTE",IF(NOT(L30&gt;=C30*100/VLOOKUP(Y30,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
-        <v/>
-      </c>
-      <c r="X30" s="7" t="n"/>
+        <f>IF(NOT(AND(IF(ISNUMBER(M30),N30*PI()*(O30/10)^2/4&gt;=M30,TRUE),IF(ISNUMBER(P30),Q30*PI()*(R30/10)^2/4&gt;=P30,TRUE),IF(ISNUMBER(M30),M30&lt;=0.0163*AB30*K30,TRUE),IF(ISNUMBER(P30),P30&lt;=0.0163*AC30*K30,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F30&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J30*K30+2*PI()*(U30/10)^2/4*Datos!$B$6*K30/V30)),"NO VERIF. CORTE",IF(NOT(L30&gt;=C30*100/VLOOKUP(Y30,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <v/>
+      </c>
+      <c r="X30" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y30" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z30" s="24" t="n">
+      <c r="Z30" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA30" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB30" s="7">
+        <f>IF(Z30="Colgante",MIN(C30*100/4,J30+16*AA30),J30)</f>
+        <v/>
+      </c>
+      <c r="AC30" s="7">
+        <f>IF(Z30="Invertida",MIN(C30*100/4,J30+16*AA30),J30)</f>
+        <v/>
+      </c>
+      <c r="AD30" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA30" s="24" t="n">
+      <c r="AE30" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB30" s="24" t="n">
+      <c r="AF30" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4662,7 +5150,7 @@
         <v>3.58</v>
       </c>
       <c r="D31" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AA31)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z31)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD31)</f>
         <v/>
       </c>
       <c r="E31" s="7" t="n"/>
@@ -4686,14 +5174,14 @@
         <v>15</v>
       </c>
       <c r="K31" s="7">
-        <f>L31-AB31</f>
+        <f>L31-AF31</f>
         <v/>
       </c>
       <c r="L31" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M31" s="25">
-        <f>IF(NOT(ISNUMBER(H31)),"---",IF(H31&lt;=0,"---",IF(H31*100/(Datos!$B$8*J31*K31^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H31*100/(Datos!$B$8*J31*K31^2*Datos!$B$5)))*J31*K31*Datos!$B$5/Datos!$B$6,0.0033*J31*K31))))</f>
+        <f>IF(NOT(ISNUMBER(H31)),"---",IF(H31&lt;=0,"---",IF(H31*100/(Datos!$B$8*AB31*K31^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H31*100/(Datos!$B$8*AB31*K31^2*Datos!$B$5)))*AB31*K31*Datos!$B$5/Datos!$B$6,0.0033*J31*K31))))</f>
         <v/>
       </c>
       <c r="N31" s="24" t="n">
@@ -4703,7 +5191,7 @@
         <v>12</v>
       </c>
       <c r="P31" s="25">
-        <f>IF(NOT(ISNUMBER(I31)),"---",IF(I31&lt;=0,"---",IF(I31*100/(Datos!$B$8*J31*K31^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I31*100/(Datos!$B$8*J31*K31^2*Datos!$B$5)))*J31*K31*Datos!$B$5/Datos!$B$6,0.0033*J31*K31))))</f>
+        <f>IF(NOT(ISNUMBER(I31)),"---",IF(I31&lt;=0,"---",IF(I31*100/(Datos!$B$8*AC31*K31^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I31*100/(Datos!$B$8*AC31*K31^2*Datos!$B$5)))*AC31*K31*Datos!$B$5/Datos!$B$6,0.0033*J31*K31))))</f>
         <v/>
       </c>
       <c r="Q31" s="24" t="n">
@@ -4727,7 +5215,7 @@
         <v>30</v>
       </c>
       <c r="W31" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*J31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*J31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X31" s="7" t="n"/>
@@ -4736,13 +5224,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z31" s="24" t="n">
+      <c r="Z31" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA31" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB31" s="7">
+        <f>IF(Z31="Colgante",MIN(C31*100/4,J31+16*AA31),J31)</f>
+        <v/>
+      </c>
+      <c r="AC31" s="7">
+        <f>IF(Z31="Invertida",MIN(C31*100/4,J31+16*AA31),J31)</f>
+        <v/>
+      </c>
+      <c r="AD31" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA31" s="24" t="n">
+      <c r="AE31" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB31" s="24" t="n">
+      <c r="AF31" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4757,7 +5261,7 @@
         <v>1.12</v>
       </c>
       <c r="D32" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AA32)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z32)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD32)</f>
         <v/>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -4781,14 +5285,14 @@
         <v>15</v>
       </c>
       <c r="K32" s="7">
-        <f>L32-AB32</f>
+        <f>L32-AF32</f>
         <v/>
       </c>
       <c r="L32" s="24" t="n">
         <v>70</v>
       </c>
       <c r="M32" s="25">
-        <f>IF(NOT(ISNUMBER(H32)),"---",IF(H32&lt;=0,"---",IF(H32*100/(Datos!$B$8*J32*K32^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H32*100/(Datos!$B$8*J32*K32^2*Datos!$B$5)))*J32*K32*Datos!$B$5/Datos!$B$6,0.0033*J32*K32))))</f>
+        <f>IF(NOT(ISNUMBER(H32)),"---",IF(H32&lt;=0,"---",IF(H32*100/(Datos!$B$8*AB32*K32^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H32*100/(Datos!$B$8*AB32*K32^2*Datos!$B$5)))*AB32*K32*Datos!$B$5/Datos!$B$6,0.0033*J32*K32))))</f>
         <v/>
       </c>
       <c r="N32" s="24" t="n">
@@ -4798,7 +5302,7 @@
         <v>12</v>
       </c>
       <c r="P32" s="25">
-        <f>IF(NOT(ISNUMBER(I32)),"---",IF(I32&lt;=0,"---",IF(I32*100/(Datos!$B$8*J32*K32^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I32*100/(Datos!$B$8*J32*K32^2*Datos!$B$5)))*J32*K32*Datos!$B$5/Datos!$B$6,0.0033*J32*K32))))</f>
+        <f>IF(NOT(ISNUMBER(I32)),"---",IF(I32&lt;=0,"---",IF(I32*100/(Datos!$B$8*AC32*K32^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I32*100/(Datos!$B$8*AC32*K32^2*Datos!$B$5)))*AC32*K32*Datos!$B$5/Datos!$B$6,0.0033*J32*K32))))</f>
         <v/>
       </c>
       <c r="Q32" s="24" t="n">
@@ -4822,7 +5326,7 @@
         <v>30</v>
       </c>
       <c r="W32" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M32),N32*PI()*(O32/10)^2/4&gt;=M32,TRUE),IF(ISNUMBER(P32),Q32*PI()*(R32/10)^2/4&gt;=P32,TRUE),IF(ISNUMBER(M32),M32&lt;=0.0163*J32*K32,TRUE),IF(ISNUMBER(P32),P32&lt;=0.0163*J32*K32,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F32&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J32*K32+2*PI()*(U32/10)^2/4*Datos!$B$6*K32/V32)),"NO VERIF. CORTE",IF(NOT(L32&gt;=C32*100/VLOOKUP(Y32,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M32),N32*PI()*(O32/10)^2/4&gt;=M32,TRUE),IF(ISNUMBER(P32),Q32*PI()*(R32/10)^2/4&gt;=P32,TRUE),IF(ISNUMBER(M32),M32&lt;=0.0163*AB32*K32,TRUE),IF(ISNUMBER(P32),P32&lt;=0.0163*AC32*K32,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F32&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J32*K32+2*PI()*(U32/10)^2/4*Datos!$B$6*K32/V32)),"NO VERIF. CORTE",IF(NOT(L32&gt;=C32*100/VLOOKUP(Y32,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X32" s="7" t="n"/>
@@ -4831,13 +5335,29 @@
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z32" s="24" t="n">
+      <c r="Z32" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA32" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB32" s="7">
+        <f>IF(Z32="Colgante",MIN(C32*100/4,J32+16*AA32),J32)</f>
+        <v/>
+      </c>
+      <c r="AC32" s="7">
+        <f>IF(Z32="Invertida",MIN(C32*100/4,J32+16*AA32),J32)</f>
+        <v/>
+      </c>
+      <c r="AD32" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="AA32" s="24" t="n">
+      <c r="AE32" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AB32" s="24" t="n">
+      <c r="AF32" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4852,7 +5372,7 @@
         <v>4.35</v>
       </c>
       <c r="D33" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*Z33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AA33)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*Z33)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD33)</f>
         <v/>
       </c>
       <c r="E33" s="32" t="n"/>
@@ -4876,14 +5396,14 @@
         <v>15</v>
       </c>
       <c r="K33" s="32">
-        <f>L33-AB33</f>
+        <f>L33-AF33</f>
         <v/>
       </c>
       <c r="L33" s="33" t="n">
         <v>70</v>
       </c>
       <c r="M33" s="34">
-        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*J33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*J33*K33^2*Datos!$B$5)))*J33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
         <v/>
       </c>
       <c r="N33" s="33" t="n">
@@ -4893,7 +5413,7 @@
         <v>12</v>
       </c>
       <c r="P33" s="34">
-        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*J33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*J33*K33^2*Datos!$B$5)))*J33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
         <v/>
       </c>
       <c r="Q33" s="33" t="inlineStr">
@@ -4921,7 +5441,7 @@
         <v>30</v>
       </c>
       <c r="W33" s="32">
-        <f>IF(NOT(AND(IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*J33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*J33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(NOT(AND(IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
         <v/>
       </c>
       <c r="X33" s="32" t="n"/>
@@ -4930,13 +5450,29 @@
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z33" s="33" t="n">
+      <c r="Z33" s="33" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA33" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB33" s="32">
+        <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="32">
+        <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AD33" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="AA33" s="33" t="n">
+      <c r="AE33" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="AB33" s="33" t="n">
+      <c r="AF33" s="33" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4947,14 +5483,14 @@
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="A25:A33"/>
+    <mergeCell ref="A1:AF1"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="S2:U2"/>
     <mergeCell ref="I2:I3"/>
-    <mergeCell ref="A1:AB1"/>
     <mergeCell ref="V2"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="Y2:AB2"/>
+    <mergeCell ref="Y2:AF2"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="X2:X3"/>
     <mergeCell ref="M2:O2"/>
@@ -4975,9 +5511,12 @@
       <formula>"VERIFICAR FLECHA"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="Y4:Y33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos!$A$19:$A$23</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z4:Z33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Invertida,Colgante"</formula1>
     </dataValidation>
     <dataValidation sqref="O4:O33 R4:R33 U4:U33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16,20,25"</formula1>
@@ -4995,7 +5534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5289,12 +5828,12 @@
     <row r="34">
       <c r="A34" s="36" t="inlineStr">
         <is>
-          <t>6. RESULTADO</t>
+          <t>6. VIGAS INVERTIDAS</t>
         </is>
       </c>
       <c r="B34" s="36" t="inlineStr">
         <is>
-          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
+          <t>Las vigas de BORDE son invertidas: sobresalen 70 cm por encima del fondo de</t>
         </is>
       </c>
     </row>
@@ -5302,7 +5841,7 @@
       <c r="A35" s="36" t="inlineStr"/>
       <c r="B35" s="37" t="inlineStr">
         <is>
-          <t>VI 02 (15x60, 9,88 m): la armadura de apoyo necesaria (18,6 cm2) supera la cuantia</t>
+          <t>losa (cotas N.F.L +3,50 / N.S.V +4,20 y N.F.L +6,80 / N.S.V +7,50 del plano).</t>
         </is>
       </c>
     </row>
@@ -5310,7 +5849,7 @@
       <c r="A36" s="36" t="inlineStr"/>
       <c r="B36" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   maxima de la seccion (13,2 cm2). No alcanza como tramo unico: necesita d = 65 cm o</t>
+          <t>Son VI 01a, VI 01b, VI 07a, VI 07b, VI 07c, VI 11a, VI 11b, VI 11c, VI 15a y VI 15b,</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5857,7 @@
       <c r="A37" s="36" t="inlineStr"/>
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   un apoyo intermedio. Como la casa esta construida, lo mas probable es que exista una</t>
+          <t>identificadas por coincidir su eje con el contorno del edificio.</t>
         </is>
       </c>
     </row>
@@ -5326,7 +5865,7 @@
       <c r="A38" s="36" t="inlineStr"/>
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   columna intermedia no identificada al leer el plano.</t>
+          <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
@@ -5334,7 +5873,7 @@
       <c r="A39" s="36" t="inlineStr"/>
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
@@ -5342,23 +5881,23 @@
       <c r="A40" s="36" t="inlineStr"/>
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="36" t="inlineStr"/>
-      <c r="B41" s="37" t="inlineStr"/>
+      <c r="B41" s="37" t="inlineStr">
+        <is>
+          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
+        </is>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="36" t="inlineStr">
-        <is>
-          <t>7. ALCANCE</t>
-        </is>
-      </c>
-      <c r="B42" s="36" t="inlineStr">
-        <is>
-          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+      <c r="A42" s="36" t="inlineStr"/>
+      <c r="B42" s="37" t="inlineStr">
+        <is>
+          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
@@ -5366,31 +5905,31 @@
       <c r="A43" s="36" t="inlineStr"/>
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
+          <t>PENDIENTE: una viga invertida de borde recibe la reaccion de la losa excentrica</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="36" t="inlineStr"/>
-      <c r="B44" s="37" t="inlineStr"/>
+      <c r="B44" s="37" t="inlineStr">
+        <is>
+          <t>respecto de su eje y queda sometida a TORSION. Esta planilla no la verifica.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
-      <c r="A45" s="36" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B45" s="36" t="inlineStr">
-        <is>
-          <t>El ancho tributario B se adopto uniforme en 2,00 m (0,60 m en vigas chatas) por no</t>
-        </is>
-      </c>
+      <c r="A45" s="36" t="inlineStr"/>
+      <c r="B45" s="37" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="36" t="inlineStr"/>
-      <c r="B46" s="37" t="inlineStr">
-        <is>
-          <t>disponer de la planta acotada con el reparto de losas. Es la hipotesis mas influyente:</t>
+      <c r="A46" s="36" t="inlineStr">
+        <is>
+          <t>7. RESULTADO</t>
+        </is>
+      </c>
+      <c r="B46" s="36" t="inlineStr">
+        <is>
+          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
@@ -5398,7 +5937,7 @@
       <c r="A47" s="36" t="inlineStr"/>
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>ajustarla viga por viga en la columna B trib. y todo se recalcula.</t>
+          <t>VI 02 (15x60, 9,88 m): la armadura de apoyo necesaria (18,6 cm2) supera la cuantia</t>
         </is>
       </c>
     </row>
@@ -5406,13 +5945,109 @@
       <c r="A48" s="36" t="inlineStr"/>
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+          <t xml:space="preserve">   maxima (13,2 cm2). Se verifico en el plano que NO tiene apoyo intermedio, y por ser</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="36" t="inlineStr"/>
       <c r="B49" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   viga colgante tampoco tiene ala comprimida sobre el apoyo. Queda como el unico punto</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="36" t="inlineStr"/>
+      <c r="B50" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   abierto: revisar el ancho tributario real, hoy adoptado en 2,00 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="36" t="inlineStr"/>
+      <c r="B51" s="37" t="inlineStr">
+        <is>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="36" t="inlineStr"/>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="36" t="inlineStr"/>
+      <c r="B53" s="37" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="36" t="inlineStr">
+        <is>
+          <t>8. ALCANCE</t>
+        </is>
+      </c>
+      <c r="B54" s="37" t="inlineStr">
+        <is>
+          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="36" t="inlineStr"/>
+      <c r="B55" s="37" t="inlineStr">
+        <is>
+          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="36" t="inlineStr"/>
+      <c r="B56" s="37" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="36" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B57" s="36" t="inlineStr">
+        <is>
+          <t>El ancho tributario B se adopto uniforme en 2,00 m (0,60 m en vigas chatas) por no</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="36" t="inlineStr"/>
+      <c r="B58" s="37" t="inlineStr">
+        <is>
+          <t>disponer de la planta acotada con el reparto de losas. Es la hipotesis mas influyente:</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="36" t="inlineStr"/>
+      <c r="B59" s="37" t="inlineStr">
+        <is>
+          <t>ajustarla viga por viga en la columna B trib. y todo se recalcula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="36" t="inlineStr"/>
+      <c r="B60" s="37" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="36" t="inlineStr"/>
+      <c r="B61" s="37" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>

<commit_message>
Cargar los anchos tributarios relevados de VI 02 y VCH 03a
VI 02 solo recibe el voladizo L02 de 0,80 m: la carga baja de 2999 a
1823 kg/m y la viga pasa a verificar. VCH 03a recibe L03 y L04 a cada
lado, 3,94 m de ancho tributario, y la seccion 40x13 queda muy por
debajo de lo necesario. 29 de 30 vigas verifican.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -2354,7 +2354,7 @@
         <v/>
       </c>
       <c r="N6" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="O6" s="24" t="n">
         <v>20</v>
@@ -2364,7 +2364,7 @@
         <v/>
       </c>
       <c r="Q6" s="24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="R6" s="24" t="n">
         <v>25</v>
@@ -2378,10 +2378,10 @@
         <v/>
       </c>
       <c r="U6" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V6" s="24" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="W6" s="7">
         <f>IF(NOT(AND(IF(ISNUMBER(M6),N6*PI()*(O6/10)^2/4&gt;=M6,TRUE),IF(ISNUMBER(P6),Q6*PI()*(R6/10)^2/4&gt;=P6,TRUE),IF(ISNUMBER(M6),M6&lt;=0.0163*AB6*K6,TRUE),IF(ISNUMBER(P6),P6&lt;=0.0163*AC6*K6,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F6&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J6*K6+2*PI()*(U6/10)^2/4*Datos!$B$6*K6/V6)),"NO VERIF. CORTE",IF(NOT(L6&gt;=C6*100/VLOOKUP(Y6,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
@@ -2389,7 +2389,7 @@
       </c>
       <c r="X6" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Es viga colgante, asi que sobre el apoyo la losa queda traccionada y no aporta ala comprimida: la seccion es rectangular 15x60 y la armadura necesaria (18,6 cm2) supera la cuantia maxima (13,2). Confirmado que no tiene apoyo intermedio. Revisar el ancho tributario real.</t>
+          <t>Ancho tributario relevado: solo recibe L02, voladizo de 0,80 m, que entrega su carga entera. Con B=0,80 la viga VERIFICA. El voladizo ademas le transmite torsion, no verificada aqui.</t>
         </is>
       </c>
       <c r="Y6" s="24" t="inlineStr">
@@ -2414,13 +2414,13 @@
         <v/>
       </c>
       <c r="AD6" s="24" t="n">
-        <v>2</v>
+        <v>0.8</v>
       </c>
       <c r="AE6" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF6" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7" ht="46" customHeight="1">
@@ -4162,20 +4162,20 @@
         <v/>
       </c>
       <c r="N22" s="24" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="O22" s="24" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="P22" s="25">
         <f>IF(NOT(ISNUMBER(I22)),"---",IF(I22&lt;=0,"---",IF(I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)))*AC22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="Q22" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="R22" s="24" t="n">
         <v>6</v>
-      </c>
-      <c r="R22" s="24" t="n">
-        <v>12</v>
       </c>
       <c r="S22" s="25">
         <f>F22/(J22*0.85*K22)</f>
@@ -4222,7 +4222,7 @@
         <v/>
       </c>
       <c r="AD22" s="24" t="n">
-        <v>0.6</v>
+        <v>3.94</v>
       </c>
       <c r="AE22" s="24" t="n">
         <v>2.6</v>
@@ -5937,7 +5937,7 @@
       <c r="A47" s="36" t="inlineStr"/>
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>VI 02 (15x60, 9,88 m): la armadura de apoyo necesaria (18,6 cm2) supera la cuantia</t>
+          <t>VI 02 quedo resuelta: con el ancho tributario relevado (solo el voladizo L02 de</t>
         </is>
       </c>
     </row>
@@ -5945,7 +5945,7 @@
       <c r="A48" s="36" t="inlineStr"/>
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   maxima (13,2 cm2). Se verifico en el plano que NO tiene apoyo intermedio, y por ser</t>
+          <t xml:space="preserve">   0,80 m) la carga baja de 2999 a 1823 kg/m y la viga verifica con 9,94 cm2.</t>
         </is>
       </c>
     </row>
@@ -5953,7 +5953,7 @@
       <c r="A49" s="36" t="inlineStr"/>
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   viga colgante tampoco tiene ala comprimida sobre el apoyo. Queda como el unico punto</t>
+          <t>VCH 03a (40x13, 3,71 m) es el unico punto abierto: con L03 y L04 apoyando a cada</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       <c r="A50" s="36" t="inlineStr"/>
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   abierto: revisar el ancho tributario real, hoy adoptado en 2,00 m.</t>
+          <t xml:space="preserve">   lado el ancho tributario es 3,94 m y el momento supera lo que admite la seccion.</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="B57" s="36" t="inlineStr">
         <is>
-          <t>El ancho tributario B se adopto uniforme en 2,00 m (0,60 m en vigas chatas) por no</t>
+          <t>El ancho tributario B esta relevado solo en VI 02 (0,80 m) y VCH 03a (3,94 m). En</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6025,7 @@
       <c r="A58" s="36" t="inlineStr"/>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t>disponer de la planta acotada con el reparto de losas. Es la hipotesis mas influyente:</t>
+          <t>las demas sigue adoptado en 2,00 m, a falta del reparto completo de losas. Es la</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6033,7 @@
       <c r="A59" s="36" t="inlineStr"/>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t>ajustarla viga por viga en la columna B trib. y todo se recalcula.</t>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corregir VCH 03a a L03 sola y arreglar la verificacion de seccion insuficiente
VCH 03a recibe solo L03: B pasa de 3,94 a 2,08 m. Sigue sin verificar.
Ademas, cuando la seccion no admite el momento la celda devolvia
REVISAR y la formula de verificacion lo daba por valido; ahora informa
SECCION INSUF. y se marca en rojo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -2154,7 +2154,7 @@
         <v>15</v>
       </c>
       <c r="W4" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M4),N4*PI()*(O4/10)^2/4&gt;=M4,TRUE),IF(ISNUMBER(P4),Q4*PI()*(R4/10)^2/4&gt;=P4,TRUE),IF(ISNUMBER(M4),M4&lt;=0.0163*AB4*K4,TRUE),IF(ISNUMBER(P4),P4&lt;=0.0163*AC4*K4,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F4&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J4*K4+2*PI()*(U4/10)^2/4*Datos!$B$6*K4/V4)),"NO VERIF. CORTE",IF(NOT(L4&gt;=C4*100/VLOOKUP(Y4,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M4="REVISAR",P4="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M4&lt;&gt;"REVISAR",P4&lt;&gt;"REVISAR",IF(ISNUMBER(M4),N4*PI()*(O4/10)^2/4&gt;=M4,TRUE),IF(ISNUMBER(P4),Q4*PI()*(R4/10)^2/4&gt;=P4,TRUE),IF(ISNUMBER(M4),M4&lt;=0.0163*AB4*K4,TRUE),IF(ISNUMBER(P4),P4&lt;=0.0163*AC4*K4,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F4&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J4*K4+2*PI()*(U4/10)^2/4*Datos!$B$6*K4/V4)),"NO VERIF. CORTE",IF(NOT(L4&gt;=C4*100/VLOOKUP(Y4,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X4" s="26" t="inlineStr">
@@ -2269,7 +2269,7 @@
         <v>30</v>
       </c>
       <c r="W5" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M5),N5*PI()*(O5/10)^2/4&gt;=M5,TRUE),IF(ISNUMBER(P5),Q5*PI()*(R5/10)^2/4&gt;=P5,TRUE),IF(ISNUMBER(M5),M5&lt;=0.0163*AB5*K5,TRUE),IF(ISNUMBER(P5),P5&lt;=0.0163*AC5*K5,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F5&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J5*K5+2*PI()*(U5/10)^2/4*Datos!$B$6*K5/V5)),"NO VERIF. CORTE",IF(NOT(L5&gt;=C5*100/VLOOKUP(Y5,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M5="REVISAR",P5="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M5&lt;&gt;"REVISAR",P5&lt;&gt;"REVISAR",IF(ISNUMBER(M5),N5*PI()*(O5/10)^2/4&gt;=M5,TRUE),IF(ISNUMBER(P5),Q5*PI()*(R5/10)^2/4&gt;=P5,TRUE),IF(ISNUMBER(M5),M5&lt;=0.0163*AB5*K5,TRUE),IF(ISNUMBER(P5),P5&lt;=0.0163*AC5*K5,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F5&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J5*K5+2*PI()*(U5/10)^2/4*Datos!$B$6*K5/V5)),"NO VERIF. CORTE",IF(NOT(L5&gt;=C5*100/VLOOKUP(Y5,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X5" s="26" t="inlineStr">
@@ -2384,7 +2384,7 @@
         <v>15</v>
       </c>
       <c r="W6" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M6),N6*PI()*(O6/10)^2/4&gt;=M6,TRUE),IF(ISNUMBER(P6),Q6*PI()*(R6/10)^2/4&gt;=P6,TRUE),IF(ISNUMBER(M6),M6&lt;=0.0163*AB6*K6,TRUE),IF(ISNUMBER(P6),P6&lt;=0.0163*AC6*K6,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F6&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J6*K6+2*PI()*(U6/10)^2/4*Datos!$B$6*K6/V6)),"NO VERIF. CORTE",IF(NOT(L6&gt;=C6*100/VLOOKUP(Y6,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M6="REVISAR",P6="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M6&lt;&gt;"REVISAR",P6&lt;&gt;"REVISAR",IF(ISNUMBER(M6),N6*PI()*(O6/10)^2/4&gt;=M6,TRUE),IF(ISNUMBER(P6),Q6*PI()*(R6/10)^2/4&gt;=P6,TRUE),IF(ISNUMBER(M6),M6&lt;=0.0163*AB6*K6,TRUE),IF(ISNUMBER(P6),P6&lt;=0.0163*AC6*K6,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F6&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J6*K6+2*PI()*(U6/10)^2/4*Datos!$B$6*K6/V6)),"NO VERIF. CORTE",IF(NOT(L6&gt;=C6*100/VLOOKUP(Y6,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X6" s="26" t="inlineStr">
@@ -2499,7 +2499,7 @@
         <v>30</v>
       </c>
       <c r="W7" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M7),N7*PI()*(O7/10)^2/4&gt;=M7,TRUE),IF(ISNUMBER(P7),Q7*PI()*(R7/10)^2/4&gt;=P7,TRUE),IF(ISNUMBER(M7),M7&lt;=0.0163*AB7*K7,TRUE),IF(ISNUMBER(P7),P7&lt;=0.0163*AC7*K7,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F7&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J7*K7+2*PI()*(U7/10)^2/4*Datos!$B$6*K7/V7)),"NO VERIF. CORTE",IF(NOT(L7&gt;=C7*100/VLOOKUP(Y7,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M7="REVISAR",P7="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M7&lt;&gt;"REVISAR",P7&lt;&gt;"REVISAR",IF(ISNUMBER(M7),N7*PI()*(O7/10)^2/4&gt;=M7,TRUE),IF(ISNUMBER(P7),Q7*PI()*(R7/10)^2/4&gt;=P7,TRUE),IF(ISNUMBER(M7),M7&lt;=0.0163*AB7*K7,TRUE),IF(ISNUMBER(P7),P7&lt;=0.0163*AC7*K7,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F7&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J7*K7+2*PI()*(U7/10)^2/4*Datos!$B$6*K7/V7)),"NO VERIF. CORTE",IF(NOT(L7&gt;=C7*100/VLOOKUP(Y7,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X7" s="7" t="n"/>
@@ -2610,7 +2610,7 @@
         <v>30</v>
       </c>
       <c r="W8" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*AB8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*AC8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos!$B$6*K8/V8)),"NO VERIF. CORTE",IF(NOT(L8&gt;=C8*100/VLOOKUP(Y8,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M8="REVISAR",P8="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M8&lt;&gt;"REVISAR",P8&lt;&gt;"REVISAR",IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*AB8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*AC8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos!$B$6*K8/V8)),"NO VERIF. CORTE",IF(NOT(L8&gt;=C8*100/VLOOKUP(Y8,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X8" s="7" t="n"/>
@@ -2721,7 +2721,7 @@
         <v>30</v>
       </c>
       <c r="W9" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M9),N9*PI()*(O9/10)^2/4&gt;=M9,TRUE),IF(ISNUMBER(P9),Q9*PI()*(R9/10)^2/4&gt;=P9,TRUE),IF(ISNUMBER(M9),M9&lt;=0.0163*AB9*K9,TRUE),IF(ISNUMBER(P9),P9&lt;=0.0163*AC9*K9,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F9&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J9*K9+2*PI()*(U9/10)^2/4*Datos!$B$6*K9/V9)),"NO VERIF. CORTE",IF(NOT(L9&gt;=C9*100/VLOOKUP(Y9,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M9="REVISAR",P9="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M9&lt;&gt;"REVISAR",P9&lt;&gt;"REVISAR",IF(ISNUMBER(M9),N9*PI()*(O9/10)^2/4&gt;=M9,TRUE),IF(ISNUMBER(P9),Q9*PI()*(R9/10)^2/4&gt;=P9,TRUE),IF(ISNUMBER(M9),M9&lt;=0.0163*AB9*K9,TRUE),IF(ISNUMBER(P9),P9&lt;=0.0163*AC9*K9,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F9&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J9*K9+2*PI()*(U9/10)^2/4*Datos!$B$6*K9/V9)),"NO VERIF. CORTE",IF(NOT(L9&gt;=C9*100/VLOOKUP(Y9,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X9" s="7" t="n"/>
@@ -2832,7 +2832,7 @@
         <v>30</v>
       </c>
       <c r="W10" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M10="REVISAR",P10="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M10&lt;&gt;"REVISAR",P10&lt;&gt;"REVISAR",IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X10" s="26" t="inlineStr">
@@ -2947,7 +2947,7 @@
         <v>30</v>
       </c>
       <c r="W11" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M11),N11*PI()*(O11/10)^2/4&gt;=M11,TRUE),IF(ISNUMBER(P11),Q11*PI()*(R11/10)^2/4&gt;=P11,TRUE),IF(ISNUMBER(M11),M11&lt;=0.0163*AB11*K11,TRUE),IF(ISNUMBER(P11),P11&lt;=0.0163*AC11*K11,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F11&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J11*K11+2*PI()*(U11/10)^2/4*Datos!$B$6*K11/V11)),"NO VERIF. CORTE",IF(NOT(L11&gt;=C11*100/VLOOKUP(Y11,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M11="REVISAR",P11="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M11&lt;&gt;"REVISAR",P11&lt;&gt;"REVISAR",IF(ISNUMBER(M11),N11*PI()*(O11/10)^2/4&gt;=M11,TRUE),IF(ISNUMBER(P11),Q11*PI()*(R11/10)^2/4&gt;=P11,TRUE),IF(ISNUMBER(M11),M11&lt;=0.0163*AB11*K11,TRUE),IF(ISNUMBER(P11),P11&lt;=0.0163*AC11*K11,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F11&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J11*K11+2*PI()*(U11/10)^2/4*Datos!$B$6*K11/V11)),"NO VERIF. CORTE",IF(NOT(L11&gt;=C11*100/VLOOKUP(Y11,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X11" s="26" t="inlineStr">
@@ -3062,7 +3062,7 @@
         <v>10</v>
       </c>
       <c r="W12" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M12="REVISAR",P12="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M12&lt;&gt;"REVISAR",P12&lt;&gt;"REVISAR",IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X12" s="26" t="inlineStr">
@@ -3177,7 +3177,7 @@
         <v>30</v>
       </c>
       <c r="W13" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M13="REVISAR",P13="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M13&lt;&gt;"REVISAR",P13&lt;&gt;"REVISAR",IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X13" s="7" t="n"/>
@@ -3288,7 +3288,7 @@
         <v>30</v>
       </c>
       <c r="W14" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M14),N14*PI()*(O14/10)^2/4&gt;=M14,TRUE),IF(ISNUMBER(P14),Q14*PI()*(R14/10)^2/4&gt;=P14,TRUE),IF(ISNUMBER(M14),M14&lt;=0.0163*AB14*K14,TRUE),IF(ISNUMBER(P14),P14&lt;=0.0163*AC14*K14,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F14&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J14*K14+2*PI()*(U14/10)^2/4*Datos!$B$6*K14/V14)),"NO VERIF. CORTE",IF(NOT(L14&gt;=C14*100/VLOOKUP(Y14,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M14="REVISAR",P14="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M14&lt;&gt;"REVISAR",P14&lt;&gt;"REVISAR",IF(ISNUMBER(M14),N14*PI()*(O14/10)^2/4&gt;=M14,TRUE),IF(ISNUMBER(P14),Q14*PI()*(R14/10)^2/4&gt;=P14,TRUE),IF(ISNUMBER(M14),M14&lt;=0.0163*AB14*K14,TRUE),IF(ISNUMBER(P14),P14&lt;=0.0163*AC14*K14,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F14&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J14*K14+2*PI()*(U14/10)^2/4*Datos!$B$6*K14/V14)),"NO VERIF. CORTE",IF(NOT(L14&gt;=C14*100/VLOOKUP(Y14,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X14" s="7" t="n"/>
@@ -3403,7 +3403,7 @@
         <v>30</v>
       </c>
       <c r="W15" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M15),N15*PI()*(O15/10)^2/4&gt;=M15,TRUE),IF(ISNUMBER(P15),Q15*PI()*(R15/10)^2/4&gt;=P15,TRUE),IF(ISNUMBER(M15),M15&lt;=0.0163*AB15*K15,TRUE),IF(ISNUMBER(P15),P15&lt;=0.0163*AC15*K15,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F15&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J15*K15+2*PI()*(U15/10)^2/4*Datos!$B$6*K15/V15)),"NO VERIF. CORTE",IF(NOT(L15&gt;=C15*100/VLOOKUP(Y15,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M15="REVISAR",P15="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M15&lt;&gt;"REVISAR",P15&lt;&gt;"REVISAR",IF(ISNUMBER(M15),N15*PI()*(O15/10)^2/4&gt;=M15,TRUE),IF(ISNUMBER(P15),Q15*PI()*(R15/10)^2/4&gt;=P15,TRUE),IF(ISNUMBER(M15),M15&lt;=0.0163*AB15*K15,TRUE),IF(ISNUMBER(P15),P15&lt;=0.0163*AC15*K15,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F15&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J15*K15+2*PI()*(U15/10)^2/4*Datos!$B$6*K15/V15)),"NO VERIF. CORTE",IF(NOT(L15&gt;=C15*100/VLOOKUP(Y15,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X15" s="7" t="n"/>
@@ -3514,7 +3514,7 @@
         <v>30</v>
       </c>
       <c r="W16" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M16),N16*PI()*(O16/10)^2/4&gt;=M16,TRUE),IF(ISNUMBER(P16),Q16*PI()*(R16/10)^2/4&gt;=P16,TRUE),IF(ISNUMBER(M16),M16&lt;=0.0163*AB16*K16,TRUE),IF(ISNUMBER(P16),P16&lt;=0.0163*AC16*K16,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F16&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J16*K16+2*PI()*(U16/10)^2/4*Datos!$B$6*K16/V16)),"NO VERIF. CORTE",IF(NOT(L16&gt;=C16*100/VLOOKUP(Y16,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M16="REVISAR",P16="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M16&lt;&gt;"REVISAR",P16&lt;&gt;"REVISAR",IF(ISNUMBER(M16),N16*PI()*(O16/10)^2/4&gt;=M16,TRUE),IF(ISNUMBER(P16),Q16*PI()*(R16/10)^2/4&gt;=P16,TRUE),IF(ISNUMBER(M16),M16&lt;=0.0163*AB16*K16,TRUE),IF(ISNUMBER(P16),P16&lt;=0.0163*AC16*K16,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F16&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J16*K16+2*PI()*(U16/10)^2/4*Datos!$B$6*K16/V16)),"NO VERIF. CORTE",IF(NOT(L16&gt;=C16*100/VLOOKUP(Y16,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X16" s="7" t="n"/>
@@ -3625,7 +3625,7 @@
         <v>30</v>
       </c>
       <c r="W17" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M17),N17*PI()*(O17/10)^2/4&gt;=M17,TRUE),IF(ISNUMBER(P17),Q17*PI()*(R17/10)^2/4&gt;=P17,TRUE),IF(ISNUMBER(M17),M17&lt;=0.0163*AB17*K17,TRUE),IF(ISNUMBER(P17),P17&lt;=0.0163*AC17*K17,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F17&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J17*K17+2*PI()*(U17/10)^2/4*Datos!$B$6*K17/V17)),"NO VERIF. CORTE",IF(NOT(L17&gt;=C17*100/VLOOKUP(Y17,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M17="REVISAR",P17="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M17&lt;&gt;"REVISAR",P17&lt;&gt;"REVISAR",IF(ISNUMBER(M17),N17*PI()*(O17/10)^2/4&gt;=M17,TRUE),IF(ISNUMBER(P17),Q17*PI()*(R17/10)^2/4&gt;=P17,TRUE),IF(ISNUMBER(M17),M17&lt;=0.0163*AB17*K17,TRUE),IF(ISNUMBER(P17),P17&lt;=0.0163*AC17*K17,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F17&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J17*K17+2*PI()*(U17/10)^2/4*Datos!$B$6*K17/V17)),"NO VERIF. CORTE",IF(NOT(L17&gt;=C17*100/VLOOKUP(Y17,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X17" s="7" t="n"/>
@@ -3736,7 +3736,7 @@
         <v>30</v>
       </c>
       <c r="W18" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M18),N18*PI()*(O18/10)^2/4&gt;=M18,TRUE),IF(ISNUMBER(P18),Q18*PI()*(R18/10)^2/4&gt;=P18,TRUE),IF(ISNUMBER(M18),M18&lt;=0.0163*AB18*K18,TRUE),IF(ISNUMBER(P18),P18&lt;=0.0163*AC18*K18,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F18&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J18*K18+2*PI()*(U18/10)^2/4*Datos!$B$6*K18/V18)),"NO VERIF. CORTE",IF(NOT(L18&gt;=C18*100/VLOOKUP(Y18,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M18="REVISAR",P18="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M18&lt;&gt;"REVISAR",P18&lt;&gt;"REVISAR",IF(ISNUMBER(M18),N18*PI()*(O18/10)^2/4&gt;=M18,TRUE),IF(ISNUMBER(P18),Q18*PI()*(R18/10)^2/4&gt;=P18,TRUE),IF(ISNUMBER(M18),M18&lt;=0.0163*AB18*K18,TRUE),IF(ISNUMBER(P18),P18&lt;=0.0163*AC18*K18,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F18&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J18*K18+2*PI()*(U18/10)^2/4*Datos!$B$6*K18/V18)),"NO VERIF. CORTE",IF(NOT(L18&gt;=C18*100/VLOOKUP(Y18,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X18" s="7" t="n"/>
@@ -3847,7 +3847,7 @@
         <v>10</v>
       </c>
       <c r="W19" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M19="REVISAR",P19="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M19&lt;&gt;"REVISAR",P19&lt;&gt;"REVISAR",IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X19" s="26" t="inlineStr">
@@ -3962,7 +3962,7 @@
         <v>30</v>
       </c>
       <c r="W20" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M20="REVISAR",P20="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M20&lt;&gt;"REVISAR",P20&lt;&gt;"REVISAR",IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X20" s="26" t="inlineStr">
@@ -4077,7 +4077,7 @@
         <v>30</v>
       </c>
       <c r="W21" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M21),N21*PI()*(O21/10)^2/4&gt;=M21,TRUE),IF(ISNUMBER(P21),Q21*PI()*(R21/10)^2/4&gt;=P21,TRUE),IF(ISNUMBER(M21),M21&lt;=0.0163*AB21*K21,TRUE),IF(ISNUMBER(P21),P21&lt;=0.0163*AC21*K21,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F21&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J21*K21+2*PI()*(U21/10)^2/4*Datos!$B$6*K21/V21)),"NO VERIF. CORTE",IF(NOT(L21&gt;=C21*100/VLOOKUP(Y21,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M21="REVISAR",P21="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M21&lt;&gt;"REVISAR",P21&lt;&gt;"REVISAR",IF(ISNUMBER(M21),N21*PI()*(O21/10)^2/4&gt;=M21,TRUE),IF(ISNUMBER(P21),Q21*PI()*(R21/10)^2/4&gt;=P21,TRUE),IF(ISNUMBER(M21),M21&lt;=0.0163*AB21*K21,TRUE),IF(ISNUMBER(P21),P21&lt;=0.0163*AC21*K21,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F21&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J21*K21+2*PI()*(U21/10)^2/4*Datos!$B$6*K21/V21)),"NO VERIF. CORTE",IF(NOT(L21&gt;=C21*100/VLOOKUP(Y21,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X21" s="26" t="inlineStr">
@@ -4162,10 +4162,10 @@
         <v/>
       </c>
       <c r="N22" s="24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="O22" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P22" s="25">
         <f>IF(NOT(ISNUMBER(I22)),"---",IF(I22&lt;=0,"---",IF(I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)))*AC22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
@@ -4192,7 +4192,7 @@
         <v>5</v>
       </c>
       <c r="W22" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M22="REVISAR",P22="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M22&lt;&gt;"REVISAR",P22&lt;&gt;"REVISAR",IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X22" s="26" t="inlineStr">
@@ -4222,7 +4222,7 @@
         <v/>
       </c>
       <c r="AD22" s="24" t="n">
-        <v>3.94</v>
+        <v>2.08</v>
       </c>
       <c r="AE22" s="24" t="n">
         <v>2.6</v>
@@ -4307,7 +4307,7 @@
         <v>5</v>
       </c>
       <c r="W23" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M23),N23*PI()*(O23/10)^2/4&gt;=M23,TRUE),IF(ISNUMBER(P23),Q23*PI()*(R23/10)^2/4&gt;=P23,TRUE),IF(ISNUMBER(M23),M23&lt;=0.0163*AB23*K23,TRUE),IF(ISNUMBER(P23),P23&lt;=0.0163*AC23*K23,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F23&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J23*K23+2*PI()*(U23/10)^2/4*Datos!$B$6*K23/V23)),"NO VERIF. CORTE",IF(NOT(L23&gt;=C23*100/VLOOKUP(Y23,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M23="REVISAR",P23="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M23&lt;&gt;"REVISAR",P23&lt;&gt;"REVISAR",IF(ISNUMBER(M23),N23*PI()*(O23/10)^2/4&gt;=M23,TRUE),IF(ISNUMBER(P23),Q23*PI()*(R23/10)^2/4&gt;=P23,TRUE),IF(ISNUMBER(M23),M23&lt;=0.0163*AB23*K23,TRUE),IF(ISNUMBER(P23),P23&lt;=0.0163*AC23*K23,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F23&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J23*K23+2*PI()*(U23/10)^2/4*Datos!$B$6*K23/V23)),"NO VERIF. CORTE",IF(NOT(L23&gt;=C23*100/VLOOKUP(Y23,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X23" s="26" t="inlineStr">
@@ -4426,7 +4426,7 @@
         <v>20</v>
       </c>
       <c r="W24" s="32">
-        <f>IF(NOT(AND(IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X24" s="32" t="n"/>
@@ -4541,7 +4541,7 @@
         <v>15</v>
       </c>
       <c r="W25" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X25" s="7" t="n"/>
@@ -4652,7 +4652,7 @@
         <v>20</v>
       </c>
       <c r="W26" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*AB26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*AC26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M26="REVISAR",P26="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M26&lt;&gt;"REVISAR",P26&lt;&gt;"REVISAR",IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*AB26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*AC26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X26" s="7" t="n"/>
@@ -4763,7 +4763,7 @@
         <v>20</v>
       </c>
       <c r="W27" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M27="REVISAR",P27="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M27&lt;&gt;"REVISAR",P27&lt;&gt;"REVISAR",IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X27" s="7" t="n"/>
@@ -4874,7 +4874,7 @@
         <v>30</v>
       </c>
       <c r="W28" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M28),N28*PI()*(O28/10)^2/4&gt;=M28,TRUE),IF(ISNUMBER(P28),Q28*PI()*(R28/10)^2/4&gt;=P28,TRUE),IF(ISNUMBER(M28),M28&lt;=0.0163*AB28*K28,TRUE),IF(ISNUMBER(P28),P28&lt;=0.0163*AC28*K28,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F28&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J28*K28+2*PI()*(U28/10)^2/4*Datos!$B$6*K28/V28)),"NO VERIF. CORTE",IF(NOT(L28&gt;=C28*100/VLOOKUP(Y28,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M28="REVISAR",P28="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M28&lt;&gt;"REVISAR",P28&lt;&gt;"REVISAR",IF(ISNUMBER(M28),N28*PI()*(O28/10)^2/4&gt;=M28,TRUE),IF(ISNUMBER(P28),Q28*PI()*(R28/10)^2/4&gt;=P28,TRUE),IF(ISNUMBER(M28),M28&lt;=0.0163*AB28*K28,TRUE),IF(ISNUMBER(P28),P28&lt;=0.0163*AC28*K28,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F28&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J28*K28+2*PI()*(U28/10)^2/4*Datos!$B$6*K28/V28)),"NO VERIF. CORTE",IF(NOT(L28&gt;=C28*100/VLOOKUP(Y28,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X28" s="7" t="n"/>
@@ -4985,7 +4985,7 @@
         <v>30</v>
       </c>
       <c r="W29" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M29="REVISAR",P29="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M29&lt;&gt;"REVISAR",P29&lt;&gt;"REVISAR",IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X29" s="26" t="inlineStr">
@@ -5100,7 +5100,7 @@
         <v>30</v>
       </c>
       <c r="W30" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M30),N30*PI()*(O30/10)^2/4&gt;=M30,TRUE),IF(ISNUMBER(P30),Q30*PI()*(R30/10)^2/4&gt;=P30,TRUE),IF(ISNUMBER(M30),M30&lt;=0.0163*AB30*K30,TRUE),IF(ISNUMBER(P30),P30&lt;=0.0163*AC30*K30,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F30&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J30*K30+2*PI()*(U30/10)^2/4*Datos!$B$6*K30/V30)),"NO VERIF. CORTE",IF(NOT(L30&gt;=C30*100/VLOOKUP(Y30,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M30="REVISAR",P30="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M30&lt;&gt;"REVISAR",P30&lt;&gt;"REVISAR",IF(ISNUMBER(M30),N30*PI()*(O30/10)^2/4&gt;=M30,TRUE),IF(ISNUMBER(P30),Q30*PI()*(R30/10)^2/4&gt;=P30,TRUE),IF(ISNUMBER(M30),M30&lt;=0.0163*AB30*K30,TRUE),IF(ISNUMBER(P30),P30&lt;=0.0163*AC30*K30,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F30&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J30*K30+2*PI()*(U30/10)^2/4*Datos!$B$6*K30/V30)),"NO VERIF. CORTE",IF(NOT(L30&gt;=C30*100/VLOOKUP(Y30,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X30" s="26" t="inlineStr">
@@ -5215,7 +5215,7 @@
         <v>30</v>
       </c>
       <c r="W31" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M31="REVISAR",P31="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M31&lt;&gt;"REVISAR",P31&lt;&gt;"REVISAR",IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X31" s="7" t="n"/>
@@ -5326,7 +5326,7 @@
         <v>30</v>
       </c>
       <c r="W32" s="7">
-        <f>IF(NOT(AND(IF(ISNUMBER(M32),N32*PI()*(O32/10)^2/4&gt;=M32,TRUE),IF(ISNUMBER(P32),Q32*PI()*(R32/10)^2/4&gt;=P32,TRUE),IF(ISNUMBER(M32),M32&lt;=0.0163*AB32*K32,TRUE),IF(ISNUMBER(P32),P32&lt;=0.0163*AC32*K32,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F32&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J32*K32+2*PI()*(U32/10)^2/4*Datos!$B$6*K32/V32)),"NO VERIF. CORTE",IF(NOT(L32&gt;=C32*100/VLOOKUP(Y32,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M32="REVISAR",P32="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M32&lt;&gt;"REVISAR",P32&lt;&gt;"REVISAR",IF(ISNUMBER(M32),N32*PI()*(O32/10)^2/4&gt;=M32,TRUE),IF(ISNUMBER(P32),Q32*PI()*(R32/10)^2/4&gt;=P32,TRUE),IF(ISNUMBER(M32),M32&lt;=0.0163*AB32*K32,TRUE),IF(ISNUMBER(P32),P32&lt;=0.0163*AC32*K32,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F32&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J32*K32+2*PI()*(U32/10)^2/4*Datos!$B$6*K32/V32)),"NO VERIF. CORTE",IF(NOT(L32&gt;=C32*100/VLOOKUP(Y32,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X32" s="7" t="n"/>
@@ -5441,7 +5441,7 @@
         <v>30</v>
       </c>
       <c r="W33" s="32">
-        <f>IF(NOT(AND(IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA")))</f>
+        <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
       <c r="X33" s="32" t="n"/>
@@ -5534,7 +5534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B61"/>
+  <dimension ref="A1:B64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5953,7 +5953,7 @@
       <c r="A49" s="36" t="inlineStr"/>
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m) es el unico punto abierto: con L03 y L04 apoyando a cada</t>
+          <t>VCH 03a (40x13, 3,71 m) es el unico punto abierto. Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       <c r="A50" s="36" t="inlineStr"/>
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   lado el ancho tributario es 3,94 m y el momento supera lo que admite la seccion.</t>
+          <t xml:space="preserve">   verifica: haria falta un espesor de 18 cm. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
       <c r="A51" s="36" t="inlineStr"/>
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
@@ -5977,23 +5977,23 @@
       <c r="A52" s="36" t="inlineStr"/>
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="36" t="inlineStr"/>
-      <c r="B53" s="37" t="inlineStr"/>
+      <c r="B53" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
-      <c r="A54" s="36" t="inlineStr">
-        <is>
-          <t>8. ALCANCE</t>
-        </is>
-      </c>
+      <c r="A54" s="36" t="inlineStr"/>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6001,7 @@
       <c r="A55" s="36" t="inlineStr"/>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
@@ -6012,12 +6012,12 @@
     <row r="57">
       <c r="A57" s="36" t="inlineStr">
         <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B57" s="36" t="inlineStr">
-        <is>
-          <t>El ancho tributario B esta relevado solo en VI 02 (0,80 m) y VCH 03a (3,94 m). En</t>
+          <t>8. ALCANCE</t>
+        </is>
+      </c>
+      <c r="B57" s="37" t="inlineStr">
+        <is>
+          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
         </is>
       </c>
     </row>
@@ -6025,29 +6025,53 @@
       <c r="A58" s="36" t="inlineStr"/>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t>las demas sigue adoptado en 2,00 m, a falta del reparto completo de losas. Es la</t>
+          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="36" t="inlineStr"/>
-      <c r="B59" s="37" t="inlineStr">
-        <is>
-          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
-        </is>
-      </c>
+      <c r="B59" s="37" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="36" t="inlineStr"/>
-      <c r="B60" s="37" t="inlineStr">
-        <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+      <c r="A60" s="36" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B60" s="36" t="inlineStr">
+        <is>
+          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="36" t="inlineStr"/>
       <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="36" t="inlineStr"/>
+      <c r="B62" s="37" t="inlineStr">
+        <is>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="36" t="inlineStr"/>
+      <c r="B63" s="37" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="36" t="inlineStr"/>
+      <c r="B64" s="37" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>

<commit_message>
Registrar los apoyos confirmados de VI 02 y VCH 03a
VI 02: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo
intermedio. VCH 03a: tabique T06 en la union con VCH 03b y COL 02 en
el otro extremo. Ninguna de las dos parte su luz, de modo que el
resultado queda firme. Se anota la seccion que harian falta: 15x75
y 40x20 respectivamente.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -2393,7 +2393,7 @@
       </c>
       <c r="X6" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Extremos confirmados en COL 02 y tabique T07: revisar si hay apoyo intermedio o si la seccion real es mayor.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Apoyos confirmados en obra: tabique T07 perpendicular en el extremo superior y COL 02 en el inferior, sin apoyo intermedio. Para esta carga harian falta 15x75 (As 16,2 cm2). Verificar la seccion real construida.</t>
         </is>
       </c>
       <c r="Y6" s="24" t="inlineStr">
@@ -5953,7 +5953,7 @@
       <c r="A48" s="36" t="inlineStr"/>
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   necesaria ronda los 28 cm2 y no entra en 15 cm de ancho ni cumple la cuantia</t>
+          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
@@ -5961,7 +5961,7 @@
       <c r="A49" s="36" t="inlineStr"/>
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   maxima. Sus dos extremos estan confirmados (COL 02 y tabique T07), asi que o</t>
+          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
@@ -5969,7 +5969,7 @@
       <c r="A50" s="36" t="inlineStr"/>
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   tiene un apoyo intermedio no relevado, o la seccion real es mayor que 15x60.</t>
+          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar el archivo suelto de vigas con los ultimos cambios
Queda al dia con el libro unico: secciones del computo metrico,
VI 06 incorporada y las 28 vigas tratadas como invertidas.
Verifican 29 de 31.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla vigas'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1123,6 +1123,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1802,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF33"/>
+  <dimension ref="A1:AF34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2159,7 +2184,7 @@
       </c>
       <c r="X4" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde sobre la medianera: NO recibe losa. Solo peso propio y mamposteria. Apoya en el tabique T01a y en la columna COL 01 de 10x10. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde sobre la medianera: NO recibe losa. Solo peso propio y mamposteria. Apoya en el tabique T01a y en la columna COL 01 de 10x10. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y4" s="24" t="inlineStr">
@@ -2274,7 +2299,7 @@
       </c>
       <c r="X5" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y5" s="24" t="inlineStr">
@@ -2347,31 +2372,27 @@
         <v/>
       </c>
       <c r="L6" s="24" t="n">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="M6" s="25">
         <f>IF(NOT(ISNUMBER(H6)),"---",IF(H6&lt;=0,"---",IF(H6*100/(Datos!$B$8*AB6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H6*100/(Datos!$B$8*AB6*K6^2*Datos!$B$5)))*AB6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
         <v/>
       </c>
       <c r="N6" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O6" s="24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="P6" s="25">
         <f>IF(NOT(ISNUMBER(I6)),"---",IF(I6&lt;=0,"---",IF(I6*100/(Datos!$B$8*AC6*K6^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I6*100/(Datos!$B$8*AC6*K6^2*Datos!$B$5)))*AC6*K6*Datos!$B$5/Datos!$B$6,0.0033*J6*K6))))</f>
         <v/>
       </c>
-      <c r="Q6" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R6" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+      <c r="Q6" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="R6" s="24" t="n">
+        <v>25</v>
       </c>
       <c r="S6" s="25">
         <f>F6/(J6*0.85*K6)</f>
@@ -2393,7 +2414,7 @@
       </c>
       <c r="X6" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). NO VERIFICA. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Apoyos confirmados en obra: tabique T07 perpendicular en el extremo superior y COL 02 en el inferior, sin apoyo intermedio. Para esta carga harian falta 15x75 (As 16,2 cm2). Verificar la seccion real construida.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). NO USAR TEXTO VIEJO. Recibe L03 (2,08 m) y el alero L02, computado como 0,59 m equivalentes por tener menor carga que un entrepiso. Con 9,88 m de luz y 15x60 la armadura de apoyo necesaria (25,5 cm2) supera la cuantia maxima (13,2). Apoyos confirmados en obra: tabique T07 perpendicular en el extremo superior y COL 02 en el inferior, sin apoyo intermedio. Para esta carga harian falta 15x75 (As 16,2 cm2). Verificar la seccion real construida.</t>
         </is>
       </c>
       <c r="Y6" s="24" t="inlineStr">
@@ -2403,7 +2424,7 @@
       </c>
       <c r="Z6" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA6" s="24" t="n">
@@ -2418,7 +2439,7 @@
         <v/>
       </c>
       <c r="AD6" s="24" t="n">
-        <v>2.664</v>
+        <v>2.689</v>
       </c>
       <c r="AE6" s="24" t="n">
         <v>2.6</v>
@@ -2514,7 +2535,7 @@
       </c>
       <c r="Z7" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA7" s="24" t="n">
@@ -2529,7 +2550,7 @@
         <v/>
       </c>
       <c r="AD7" s="24" t="n">
-        <v>2.075</v>
+        <v>2.1</v>
       </c>
       <c r="AE7" s="24" t="n">
         <v>2.6</v>
@@ -2625,7 +2646,7 @@
       </c>
       <c r="Z8" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA8" s="24" t="n">
@@ -2736,7 +2757,7 @@
       </c>
       <c r="Z9" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA9" s="24" t="n">
@@ -2751,7 +2772,7 @@
         <v/>
       </c>
       <c r="AD9" s="24" t="n">
-        <v>1.552</v>
+        <v>1.549</v>
       </c>
       <c r="AE9" s="24" t="n">
         <v>2.6</v>
@@ -2764,11 +2785,11 @@
       <c r="A10" s="27" t="n"/>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>VI 07a</t>
+          <t>VI 06</t>
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>3.37</v>
+        <v>14</v>
       </c>
       <c r="D10" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AE10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD10)</f>
@@ -2806,20 +2827,24 @@
         <v/>
       </c>
       <c r="N10" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O10" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="P10" s="25">
         <f>IF(NOT(ISNUMBER(I10)),"---",IF(I10&lt;=0,"---",IF(I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)))*AC10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
         <v/>
       </c>
-      <c r="Q10" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="R10" s="24" t="n">
-        <v>12</v>
+      <c r="Q10" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R10" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
       </c>
       <c r="S10" s="25">
         <f>F10/(J10*0.85*K10)</f>
@@ -2830,10 +2855,10 @@
         <v/>
       </c>
       <c r="U10" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V10" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W10" s="7">
         <f>IF(OR(M10="REVISAR",P10="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M10&lt;&gt;"REVISAR",P10&lt;&gt;"REVISAR",IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -2841,7 +2866,7 @@
       </c>
       <c r="X10" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Armadura en 2 capas (rec. 6 cm).</t>
         </is>
       </c>
       <c r="Y10" s="24" t="inlineStr">
@@ -2866,24 +2891,24 @@
         <v/>
       </c>
       <c r="AD10" s="24" t="n">
-        <v>0.75</v>
+        <v>1.549</v>
       </c>
       <c r="AE10" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF10" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="27" t="n"/>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>VI 07b</t>
+          <t>VI 07a</t>
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>4.03</v>
+        <v>3.37</v>
       </c>
       <c r="D11" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AE11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD11)</f>
@@ -2956,7 +2981,7 @@
       </c>
       <c r="X11" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y11" s="24" t="inlineStr">
@@ -2981,7 +3006,7 @@
         <v/>
       </c>
       <c r="AD11" s="24" t="n">
-        <v>0</v>
+        <v>0.78</v>
       </c>
       <c r="AE11" s="24" t="n">
         <v>2.6</v>
@@ -2994,11 +3019,11 @@
       <c r="A12" s="27" t="n"/>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>VI 07c</t>
+          <t>VI 07b</t>
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>8.6</v>
+        <v>4.03</v>
       </c>
       <c r="D12" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AE12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD12)</f>
@@ -3036,20 +3061,20 @@
         <v/>
       </c>
       <c r="N12" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O12" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P12" s="25">
         <f>IF(NOT(ISNUMBER(I12)),"---",IF(I12&lt;=0,"---",IF(I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)))*AC12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
         <v/>
       </c>
       <c r="Q12" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R12" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S12" s="25">
         <f>F12/(J12*0.85*K12)</f>
@@ -3060,10 +3085,10 @@
         <v/>
       </c>
       <c r="U12" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V12" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W12" s="7">
         <f>IF(OR(M12="REVISAR",P12="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M12&lt;&gt;"REVISAR",P12&lt;&gt;"REVISAR",IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3071,12 +3096,12 @@
       </c>
       <c r="X12" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y12" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z12" s="24" t="inlineStr">
@@ -3096,24 +3121,24 @@
         <v/>
       </c>
       <c r="AD12" s="24" t="n">
-        <v>3.73</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF12" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="27" t="n"/>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>VI 08a</t>
+          <t>VI 07c</t>
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>3.65</v>
+        <v>8.6</v>
       </c>
       <c r="D13" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AE13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD13)</f>
@@ -3151,20 +3176,20 @@
         <v/>
       </c>
       <c r="N13" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P13" s="25">
         <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)))*AC13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
         <v/>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S13" s="25">
         <f>F13/(J13*0.85*K13)</f>
@@ -3175,24 +3200,28 @@
         <v/>
       </c>
       <c r="U13" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V13" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W13" s="7">
         <f>IF(OR(M13="REVISAR",P13="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M13&lt;&gt;"REVISAR",P13&lt;&gt;"REVISAR",IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X13" s="7" t="n"/>
+      <c r="X13" s="26" t="inlineStr">
+        <is>
+          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y13" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z13" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA13" s="24" t="n">
@@ -3207,24 +3236,24 @@
         <v/>
       </c>
       <c r="AD13" s="24" t="n">
-        <v>1.075</v>
+        <v>3.71</v>
       </c>
       <c r="AE13" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF13" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="27" t="n"/>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>VI 08b</t>
+          <t>VI 08a</t>
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>4.85</v>
+        <v>3.65</v>
       </c>
       <c r="D14" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AE14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD14)</f>
@@ -3303,7 +3332,7 @@
       </c>
       <c r="Z14" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA14" s="24" t="n">
@@ -3318,7 +3347,7 @@
         <v/>
       </c>
       <c r="AD14" s="24" t="n">
-        <v>1.075</v>
+        <v>1.065</v>
       </c>
       <c r="AE14" s="24" t="n">
         <v>2.6</v>
@@ -3331,11 +3360,11 @@
       <c r="A15" s="27" t="n"/>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>VI 09</t>
+          <t>VI 08b</t>
         </is>
       </c>
       <c r="C15" s="22" t="n">
-        <v>4.85</v>
+        <v>4.87</v>
       </c>
       <c r="D15" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD15+Datos!$B$7*J15*L15/10000+Datos!$B$16*AE15)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD15)</f>
@@ -3382,15 +3411,11 @@
         <f>IF(NOT(ISNUMBER(I15)),"---",IF(I15&lt;=0,"---",IF(I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)))*AC15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
         <v/>
       </c>
-      <c r="Q15" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R15" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+      <c r="Q15" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="24" t="n">
+        <v>12</v>
       </c>
       <c r="S15" s="25">
         <f>F15/(J15*0.85*K15)</f>
@@ -3413,12 +3438,12 @@
       <c r="X15" s="7" t="n"/>
       <c r="Y15" s="24" t="inlineStr">
         <is>
-          <t>Simplemente apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z15" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA15" s="24" t="n">
@@ -3433,7 +3458,7 @@
         <v/>
       </c>
       <c r="AD15" s="24" t="n">
-        <v>1.552</v>
+        <v>1.065</v>
       </c>
       <c r="AE15" s="24" t="n">
         <v>2.6</v>
@@ -3446,11 +3471,11 @@
       <c r="A16" s="27" t="n"/>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>VI 10a</t>
+          <t>VI 09</t>
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>2.55</v>
+        <v>4.87</v>
       </c>
       <c r="D16" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AE16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD16)</f>
@@ -3497,11 +3522,15 @@
         <f>IF(NOT(ISNUMBER(I16)),"---",IF(I16&lt;=0,"---",IF(I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)))*AC16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
         <v/>
       </c>
-      <c r="Q16" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="R16" s="24" t="n">
-        <v>12</v>
+      <c r="Q16" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R16" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
       </c>
       <c r="S16" s="25">
         <f>F16/(J16*0.85*K16)</f>
@@ -3524,12 +3553,12 @@
       <c r="X16" s="7" t="n"/>
       <c r="Y16" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Simplemente apoyada</t>
         </is>
       </c>
       <c r="Z16" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA16" s="24" t="n">
@@ -3544,7 +3573,7 @@
         <v/>
       </c>
       <c r="AD16" s="24" t="n">
-        <v>0</v>
+        <v>1.549</v>
       </c>
       <c r="AE16" s="24" t="n">
         <v>2.6</v>
@@ -3557,11 +3586,11 @@
       <c r="A17" s="27" t="n"/>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>VI 10b</t>
+          <t>VI 10a</t>
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>4</v>
+        <v>2.55</v>
       </c>
       <c r="D17" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AE17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD17)</f>
@@ -3640,7 +3669,7 @@
       </c>
       <c r="Z17" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA17" s="24" t="n">
@@ -3655,7 +3684,7 @@
         <v/>
       </c>
       <c r="AD17" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE17" s="24" t="n">
         <v>2.6</v>
@@ -3668,11 +3697,11 @@
       <c r="A18" s="27" t="n"/>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>VI 10c</t>
+          <t>VI 10b</t>
         </is>
       </c>
       <c r="C18" s="22" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="D18" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AE18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD18)</f>
@@ -3751,7 +3780,7 @@
       </c>
       <c r="Z18" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA18" s="24" t="n">
@@ -3766,7 +3795,7 @@
         <v/>
       </c>
       <c r="AD18" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE18" s="24" t="n">
         <v>2.6</v>
@@ -3779,11 +3808,11 @@
       <c r="A19" s="27" t="n"/>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>VI 11a</t>
+          <t>VI 10c</t>
         </is>
       </c>
       <c r="C19" s="22" t="n">
-        <v>7.68</v>
+        <v>3.6</v>
       </c>
       <c r="D19" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AE19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD19)</f>
@@ -3821,20 +3850,20 @@
         <v/>
       </c>
       <c r="N19" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P19" s="25">
         <f>IF(NOT(ISNUMBER(I19)),"---",IF(I19&lt;=0,"---",IF(I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)))*AC19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
         <v/>
       </c>
       <c r="Q19" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R19" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S19" s="25">
         <f>F19/(J19*0.85*K19)</f>
@@ -3848,20 +3877,16 @@
         <v>6</v>
       </c>
       <c r="V19" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W19" s="7">
         <f>IF(OR(M19="REVISAR",P19="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M19&lt;&gt;"REVISAR",P19&lt;&gt;"REVISAR",IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X19" s="26" t="inlineStr">
-        <is>
-          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X19" s="7" t="n"/>
       <c r="Y19" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z19" s="24" t="inlineStr">
@@ -3881,7 +3906,7 @@
         <v/>
       </c>
       <c r="AD19" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE19" s="24" t="n">
         <v>2.6</v>
@@ -3894,11 +3919,11 @@
       <c r="A20" s="27" t="n"/>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>VI 11b</t>
+          <t>VI 11a</t>
         </is>
       </c>
       <c r="C20" s="22" t="n">
-        <v>3.45</v>
+        <v>7.68</v>
       </c>
       <c r="D20" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AE20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD20)</f>
@@ -3936,20 +3961,20 @@
         <v/>
       </c>
       <c r="N20" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P20" s="25">
         <f>IF(NOT(ISNUMBER(I20)),"---",IF(I20&lt;=0,"---",IF(I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)))*AC20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
         <v/>
       </c>
       <c r="Q20" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S20" s="25">
         <f>F20/(J20*0.85*K20)</f>
@@ -3963,7 +3988,7 @@
         <v>6</v>
       </c>
       <c r="V20" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W20" s="7">
         <f>IF(OR(M20="REVISAR",P20="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M20&lt;&gt;"REVISAR",P20&lt;&gt;"REVISAR",IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3971,12 +3996,12 @@
       </c>
       <c r="X20" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y20" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z20" s="24" t="inlineStr">
@@ -3996,7 +4021,7 @@
         <v/>
       </c>
       <c r="AD20" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE20" s="24" t="n">
         <v>2.6</v>
@@ -4009,11 +4034,11 @@
       <c r="A21" s="27" t="n"/>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>VI 11c</t>
+          <t>VI 11b</t>
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>5.02</v>
+        <v>3.45</v>
       </c>
       <c r="D21" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AE21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD21)</f>
@@ -4086,7 +4111,7 @@
       </c>
       <c r="X21" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y21" s="24" t="inlineStr">
@@ -4111,7 +4136,7 @@
         <v/>
       </c>
       <c r="AD21" s="24" t="n">
-        <v>1.552</v>
+        <v>0</v>
       </c>
       <c r="AE21" s="24" t="n">
         <v>2.6</v>
@@ -4124,11 +4149,11 @@
       <c r="A22" s="27" t="n"/>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>VCH 03a</t>
+          <t>VI 11c</t>
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>3.83</v>
+        <v>5.02</v>
       </c>
       <c r="D22" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AE22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD22)</f>
@@ -4152,14 +4177,14 @@
         <v/>
       </c>
       <c r="J22" s="24" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="K22" s="7">
         <f>L22-AF22</f>
         <v/>
       </c>
       <c r="L22" s="24" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="M22" s="25">
         <f>IF(NOT(ISNUMBER(H22)),"---",IF(H22&lt;=0,"---",IF(H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)))*AB22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
@@ -4169,17 +4194,17 @@
         <v>3</v>
       </c>
       <c r="O22" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P22" s="25">
         <f>IF(NOT(ISNUMBER(I22)),"---",IF(I22&lt;=0,"---",IF(I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I22*100/(Datos!$B$8*AC22*K22^2*Datos!$B$5)))*AC22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="Q22" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R22" s="24" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="S22" s="25">
         <f>F22/(J22*0.85*K22)</f>
@@ -4190,10 +4215,10 @@
         <v/>
       </c>
       <c r="U22" s="24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="V22" s="24" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="W22" s="7">
         <f>IF(OR(M22="REVISAR",P22="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M22&lt;&gt;"REVISAR",P22&lt;&gt;"REVISAR",IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4201,7 +4226,7 @@
       </c>
       <c r="X22" s="26" t="inlineStr">
         <is>
-          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y22" s="24" t="inlineStr">
@@ -4211,7 +4236,7 @@
       </c>
       <c r="Z22" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA22" s="24" t="n">
@@ -4226,7 +4251,7 @@
         <v/>
       </c>
       <c r="AD22" s="24" t="n">
-        <v>2.075</v>
+        <v>1.549</v>
       </c>
       <c r="AE22" s="24" t="n">
         <v>2.6</v>
@@ -4239,11 +4264,11 @@
       <c r="A23" s="27" t="n"/>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>VCH 03b</t>
+          <t>VCH 03a</t>
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>2.15</v>
+        <v>3.71</v>
       </c>
       <c r="D23" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AE23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD23)</f>
@@ -4281,20 +4306,20 @@
         <v/>
       </c>
       <c r="N23" s="24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O23" s="24" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="P23" s="25">
         <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)))*AC23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="Q23" s="24" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="R23" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S23" s="25">
         <f>F23/(J23*0.85*K23)</f>
@@ -4316,7 +4341,7 @@
       </c>
       <c r="X23" s="26" t="inlineStr">
         <is>
-          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
         </is>
       </c>
       <c r="Y23" s="24" t="inlineStr">
@@ -4341,7 +4366,7 @@
         <v/>
       </c>
       <c r="AD23" s="24" t="n">
-        <v>2.075</v>
+        <v>2.1</v>
       </c>
       <c r="AE23" s="24" t="n">
         <v>2.6</v>
@@ -4351,251 +4376,251 @@
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="28" t="n"/>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>VCH 03b</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="D24" s="23">
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="23">
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
+        <v/>
+      </c>
+      <c r="G24" s="23">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="23">
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
+        <v/>
+      </c>
+      <c r="I24" s="23">
+        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
+        <v/>
+      </c>
+      <c r="J24" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="K24" s="7">
+        <f>L24-AF24</f>
+        <v/>
+      </c>
+      <c r="L24" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="M24" s="25">
+        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <v/>
+      </c>
+      <c r="N24" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="O24" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="P24" s="25">
+        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="R24" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="S24" s="25">
+        <f>F24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="T24" s="25">
+        <f>G24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="U24" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="V24" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="W24" s="7">
+        <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X24" s="26" t="inlineStr">
+        <is>
+          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+        </is>
+      </c>
+      <c r="Y24" s="24" t="inlineStr">
+        <is>
+          <t>Continua</t>
+        </is>
+      </c>
+      <c r="Z24" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA24" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB24" s="7">
+        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="7">
+        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AD24" s="24" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AE24" s="24" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AF24" s="24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="28" t="n"/>
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>VCH 05</t>
         </is>
       </c>
-      <c r="C24" s="30" t="n">
+      <c r="C25" s="30" t="n">
         <v>3.71</v>
       </c>
-      <c r="D24" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
-        <v/>
-      </c>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="31">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
-        <v/>
-      </c>
-      <c r="G24" s="31">
-        <f>F24</f>
-        <v/>
-      </c>
-      <c r="H24" s="31">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
-        <v/>
-      </c>
-      <c r="I24" s="31">
-        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
-        <v/>
-      </c>
-      <c r="J24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="K24" s="32">
-        <f>L24-AF24</f>
-        <v/>
-      </c>
-      <c r="L24" s="33" t="n">
+      <c r="D25" s="31">
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="31">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="31">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
+        <v/>
+      </c>
+      <c r="I25" s="31">
+        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
+        <v/>
+      </c>
+      <c r="J25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="K25" s="32">
+        <f>L25-AF25</f>
+        <v/>
+      </c>
+      <c r="L25" s="33" t="n">
         <v>45</v>
       </c>
-      <c r="M24" s="34">
-        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
-        <v/>
-      </c>
-      <c r="N24" s="33" t="n">
+      <c r="M25" s="34">
+        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="N25" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="O24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P24" s="34">
-        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="33" t="inlineStr">
+      <c r="O25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P25" s="34">
+        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R24" s="33" t="inlineStr">
+      <c r="R25" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="S24" s="34">
-        <f>F24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="T24" s="34">
-        <f>G24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="U24" s="33" t="n">
+      <c r="S25" s="34">
+        <f>F25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="T25" s="34">
+        <f>G25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="U25" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="V24" s="33" t="n">
+      <c r="V25" s="33" t="n">
         <v>20</v>
       </c>
-      <c r="W24" s="32">
-        <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X24" s="32" t="n"/>
-      <c r="Y24" s="33" t="inlineStr">
+      <c r="W25" s="32">
+        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X25" s="32" t="n"/>
+      <c r="Y25" s="33" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z24" s="33" t="inlineStr">
+      <c r="Z25" s="33" t="inlineStr">
         <is>
           <t>Colgante</t>
         </is>
       </c>
-      <c r="AA24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB24" s="32">
-        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AC24" s="32">
-        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AD24" s="33" t="n">
+      <c r="AA25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB25" s="32">
+        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="32">
+        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AD25" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE24" s="33" t="n">
+      <c r="AE25" s="33" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF24" s="33" t="n">
+      <c r="AF25" s="33" t="n">
         <v>3</v>
       </c>
     </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>TECHO</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>VI 12</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C26" s="22" t="n">
         <v>9.9</v>
       </c>
-      <c r="D25" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD25)</f>
-        <v/>
-      </c>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="23">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
-        <v/>
-      </c>
-      <c r="G25" s="23">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="H25" s="23">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
-        <v/>
-      </c>
-      <c r="I25" s="23">
-        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
-        <v/>
-      </c>
-      <c r="J25" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K25" s="7">
-        <f>L25-AF25</f>
-        <v/>
-      </c>
-      <c r="L25" s="24" t="n">
-        <v>70</v>
-      </c>
-      <c r="M25" s="25">
-        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="N25" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="O25" s="24" t="n">
-        <v>25</v>
-      </c>
-      <c r="P25" s="25">
-        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="24" t="n">
-        <v>4</v>
-      </c>
-      <c r="R25" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="S25" s="25">
-        <f>F25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="T25" s="25">
-        <f>G25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="U25" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="V25" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="W25" s="7">
-        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X25" s="26" t="inlineStr">
-        <is>
-          <t>Armadura en 2 capas (rec. 6 cm).</t>
-        </is>
-      </c>
-      <c r="Y25" s="24" t="inlineStr">
-        <is>
-          <t>Continua</t>
-        </is>
-      </c>
-      <c r="Z25" s="24" t="inlineStr">
-        <is>
-          <t>Colgante</t>
-        </is>
-      </c>
-      <c r="AA25" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB25" s="7">
-        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AC25" s="7">
-        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AD25" s="24" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="AE25" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF25" s="24" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="21" t="inlineStr">
-        <is>
-          <t>VI 13a</t>
-        </is>
-      </c>
-      <c r="C26" s="22" t="n">
-        <v>6</v>
-      </c>
       <c r="D26" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD26)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD26)</f>
         <v/>
       </c>
       <c r="E26" s="7" t="n"/>
@@ -4623,7 +4648,7 @@
         <v/>
       </c>
       <c r="L26" s="24" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="M26" s="25">
         <f>IF(NOT(ISNUMBER(H26)),"---",IF(H26&lt;=0,"---",IF(H26*100/(Datos!$B$8*AB26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H26*100/(Datos!$B$8*AB26*K26^2*Datos!$B$5)))*AB26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
@@ -4633,7 +4658,7 @@
         <v>2</v>
       </c>
       <c r="O26" s="24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P26" s="25">
         <f>IF(NOT(ISNUMBER(I26)),"---",IF(I26&lt;=0,"---",IF(I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)))*AC26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
@@ -4654,10 +4679,10 @@
         <v/>
       </c>
       <c r="U26" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V26" s="24" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="W26" s="7">
         <f>IF(OR(M26="REVISAR",P26="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M26&lt;&gt;"REVISAR",P26&lt;&gt;"REVISAR",IF(ISNUMBER(M26),N26*PI()*(O26/10)^2/4&gt;=M26,TRUE),IF(ISNUMBER(P26),Q26*PI()*(R26/10)^2/4&gt;=P26,TRUE),IF(ISNUMBER(M26),M26&lt;=0.0163*AB26*K26,TRUE),IF(ISNUMBER(P26),P26&lt;=0.0163*AC26*K26,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F26&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J26*K26+2*PI()*(U26/10)^2/4*Datos!$B$6*K26/V26)),"NO VERIF. CORTE",IF(NOT(L26&gt;=C26*100/VLOOKUP(Y26,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4671,7 +4696,7 @@
       </c>
       <c r="Z26" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA26" s="24" t="n">
@@ -4686,7 +4711,7 @@
         <v/>
       </c>
       <c r="AD26" s="24" t="n">
-        <v>3.799</v>
+        <v>2.1</v>
       </c>
       <c r="AE26" s="24" t="n">
         <v>1</v>
@@ -4699,14 +4724,14 @@
       <c r="A27" s="27" t="n"/>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>VI 13b</t>
+          <t>VI 13a</t>
         </is>
       </c>
       <c r="C27" s="22" t="n">
-        <v>3.75</v>
+        <v>6</v>
       </c>
       <c r="D27" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD27)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD27)</f>
         <v/>
       </c>
       <c r="E27" s="7" t="n"/>
@@ -4734,27 +4759,27 @@
         <v/>
       </c>
       <c r="L27" s="24" t="n">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="M27" s="25">
         <f>IF(NOT(ISNUMBER(H27)),"---",IF(H27&lt;=0,"---",IF(H27*100/(Datos!$B$8*AB27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H27*100/(Datos!$B$8*AB27*K27^2*Datos!$B$5)))*AB27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="N27" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" s="24" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="P27" s="25">
         <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)))*AC27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="Q27" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R27" s="24" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="S27" s="25">
         <f>F27/(J27*0.85*K27)</f>
@@ -4768,7 +4793,7 @@
         <v>6</v>
       </c>
       <c r="V27" s="24" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="W27" s="7">
         <f>IF(OR(M27="REVISAR",P27="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M27&lt;&gt;"REVISAR",P27&lt;&gt;"REVISAR",IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4782,7 +4807,7 @@
       </c>
       <c r="Z27" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA27" s="24" t="n">
@@ -4797,7 +4822,7 @@
         <v/>
       </c>
       <c r="AD27" s="24" t="n">
-        <v>2.1</v>
+        <v>3.799</v>
       </c>
       <c r="AE27" s="24" t="n">
         <v>1</v>
@@ -4810,14 +4835,14 @@
       <c r="A28" s="27" t="n"/>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>VI 14</t>
+          <t>VI 13b</t>
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D28" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD28)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD28)</f>
         <v/>
       </c>
       <c r="E28" s="7" t="n"/>
@@ -4893,7 +4918,7 @@
       </c>
       <c r="Z28" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA28" s="24" t="n">
@@ -4908,7 +4933,7 @@
         <v/>
       </c>
       <c r="AD28" s="24" t="n">
-        <v>1.699</v>
+        <v>2.1</v>
       </c>
       <c r="AE28" s="24" t="n">
         <v>1</v>
@@ -4921,14 +4946,14 @@
       <c r="A29" s="27" t="n"/>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>VI 15a</t>
+          <t>VI 14</t>
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>4.03</v>
+        <v>6</v>
       </c>
       <c r="D29" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD29)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD29)</f>
         <v/>
       </c>
       <c r="E29" s="7" t="n"/>
@@ -4996,11 +5021,7 @@
         <f>IF(OR(M29="REVISAR",P29="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M29&lt;&gt;"REVISAR",P29&lt;&gt;"REVISAR",IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X29" s="26" t="inlineStr">
-        <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X29" s="7" t="n"/>
       <c r="Y29" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5023,7 +5044,7 @@
         <v/>
       </c>
       <c r="AD29" s="24" t="n">
-        <v>0</v>
+        <v>1.699</v>
       </c>
       <c r="AE29" s="24" t="n">
         <v>1</v>
@@ -5036,14 +5057,14 @@
       <c r="A30" s="27" t="n"/>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>VI 15b</t>
+          <t>VI 15a</t>
         </is>
       </c>
       <c r="C30" s="22" t="n">
-        <v>4.85</v>
+        <v>4.03</v>
       </c>
       <c r="D30" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD30)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD30)</f>
         <v/>
       </c>
       <c r="E30" s="7" t="n"/>
@@ -5113,7 +5134,7 @@
       </c>
       <c r="X30" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde INVERTIDA: sobresale 70 cm sobre el fondo de losa. Verificar torsion, no incluida en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y30" s="24" t="inlineStr">
@@ -5138,7 +5159,7 @@
         <v/>
       </c>
       <c r="AD30" s="24" t="n">
-        <v>1.699</v>
+        <v>0</v>
       </c>
       <c r="AE30" s="24" t="n">
         <v>1</v>
@@ -5151,14 +5172,14 @@
       <c r="A31" s="27" t="n"/>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>VI 16a</t>
+          <t>VI 15b</t>
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>3.58</v>
+        <v>4.85</v>
       </c>
       <c r="D31" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD31)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD31)</f>
         <v/>
       </c>
       <c r="E31" s="7" t="n"/>
@@ -5226,7 +5247,11 @@
         <f>IF(OR(M31="REVISAR",P31="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M31&lt;&gt;"REVISAR",P31&lt;&gt;"REVISAR",IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X31" s="7" t="n"/>
+      <c r="X31" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y31" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5234,7 +5259,7 @@
       </c>
       <c r="Z31" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA31" s="24" t="n">
@@ -5262,14 +5287,14 @@
       <c r="A32" s="27" t="n"/>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>VI 16b</t>
+          <t>VI 16a</t>
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.12</v>
+        <v>3.58</v>
       </c>
       <c r="D32" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD32)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD32)</f>
         <v/>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -5345,7 +5370,7 @@
       </c>
       <c r="Z32" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA32" s="24" t="n">
@@ -5370,130 +5395,241 @@
       </c>
     </row>
     <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="28" t="n"/>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>VI 16b</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D33" s="23">
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD33)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="23">
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
+        <v/>
+      </c>
+      <c r="G33" s="23">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="23">
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
+        <v/>
+      </c>
+      <c r="I33" s="23">
+        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
+        <v/>
+      </c>
+      <c r="J33" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="K33" s="7">
+        <f>L33-AF33</f>
+        <v/>
+      </c>
+      <c r="L33" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="M33" s="25">
+        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <v/>
+      </c>
+      <c r="N33" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="P33" s="25">
+        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="S33" s="25">
+        <f>F33/(J33*0.85*K33)</f>
+        <v/>
+      </c>
+      <c r="T33" s="25">
+        <f>G33/(J33*0.85*K33)</f>
+        <v/>
+      </c>
+      <c r="U33" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="V33" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="W33" s="7">
+        <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X33" s="7" t="n"/>
+      <c r="Y33" s="24" t="inlineStr">
+        <is>
+          <t>Continua</t>
+        </is>
+      </c>
+      <c r="Z33" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB33" s="7">
+        <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="7">
+        <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AD33" s="24" t="n">
+        <v>1.699</v>
+      </c>
+      <c r="AE33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF33" s="24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="28" t="n"/>
+      <c r="B34" s="29" t="inlineStr">
         <is>
           <t>VI 17</t>
         </is>
       </c>
-      <c r="C33" s="30" t="n">
+      <c r="C34" s="30" t="n">
         <v>4.35</v>
       </c>
-      <c r="D33" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="31">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
-        <v/>
-      </c>
-      <c r="G33" s="31">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="H33" s="31">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
-        <v/>
-      </c>
-      <c r="I33" s="31">
-        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
-        <v/>
-      </c>
-      <c r="J33" s="33" t="n">
+      <c r="D34" s="31">
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD34+Datos!$B$7*J34*L34/10000+Datos!$B$16*AE34)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD34)</f>
+        <v/>
+      </c>
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="31">
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,4,0)*D34*C34</f>
+        <v/>
+      </c>
+      <c r="G34" s="31">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="31">
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,2,0)*D34*C34^2</f>
+        <v/>
+      </c>
+      <c r="I34" s="31">
+        <f>IF(VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)*D34*C34^2)</f>
+        <v/>
+      </c>
+      <c r="J34" s="33" t="n">
         <v>15</v>
       </c>
-      <c r="K33" s="32">
-        <f>L33-AF33</f>
-        <v/>
-      </c>
-      <c r="L33" s="33" t="n">
+      <c r="K34" s="32">
+        <f>L34-AF34</f>
+        <v/>
+      </c>
+      <c r="L34" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="M33" s="34">
-        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
-        <v/>
-      </c>
-      <c r="N33" s="33" t="n">
+      <c r="M34" s="34">
+        <f>IF(NOT(ISNUMBER(H34)),"---",IF(H34&lt;=0,"---",IF(H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)))*AB34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
+        <v/>
+      </c>
+      <c r="N34" s="33" t="n">
         <v>3</v>
       </c>
-      <c r="O33" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P33" s="34">
-        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
-        <v/>
-      </c>
-      <c r="Q33" s="33" t="inlineStr">
+      <c r="O34" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P34" s="34">
+        <f>IF(NOT(ISNUMBER(I34)),"---",IF(I34&lt;=0,"---",IF(I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)))*AC34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
+        <v/>
+      </c>
+      <c r="Q34" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R33" s="33" t="inlineStr">
+      <c r="R34" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="S33" s="34">
-        <f>F33/(J33*0.85*K33)</f>
-        <v/>
-      </c>
-      <c r="T33" s="34">
-        <f>G33/(J33*0.85*K33)</f>
-        <v/>
-      </c>
-      <c r="U33" s="33" t="n">
+      <c r="S34" s="34">
+        <f>F34/(J34*0.85*K34)</f>
+        <v/>
+      </c>
+      <c r="T34" s="34">
+        <f>G34/(J34*0.85*K34)</f>
+        <v/>
+      </c>
+      <c r="U34" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="V33" s="33" t="n">
+      <c r="V34" s="33" t="n">
         <v>30</v>
       </c>
-      <c r="W33" s="32">
-        <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X33" s="32" t="n"/>
-      <c r="Y33" s="33" t="inlineStr">
+      <c r="W34" s="32">
+        <f>IF(OR(M34="REVISAR",P34="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M34&lt;&gt;"REVISAR",P34&lt;&gt;"REVISAR",IF(ISNUMBER(M34),N34*PI()*(O34/10)^2/4&gt;=M34,TRUE),IF(ISNUMBER(P34),Q34*PI()*(R34/10)^2/4&gt;=P34,TRUE),IF(ISNUMBER(M34),M34&lt;=0.0163*AB34*K34,TRUE),IF(ISNUMBER(P34),P34&lt;=0.0163*AC34*K34,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F34&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J34*K34+2*PI()*(U34/10)^2/4*Datos!$B$6*K34/V34)),"NO VERIF. CORTE",IF(NOT(L34&gt;=C34*100/VLOOKUP(Y34,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X34" s="32" t="n"/>
+      <c r="Y34" s="33" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z33" s="33" t="inlineStr">
-        <is>
-          <t>Colgante</t>
-        </is>
-      </c>
-      <c r="AA33" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB33" s="32">
-        <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
-        <v/>
-      </c>
-      <c r="AC33" s="32">
-        <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
-        <v/>
-      </c>
-      <c r="AD33" s="33" t="n">
+      <c r="Z34" s="33" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA34" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB34" s="32">
+        <f>IF(Z34="Colgante",MIN(C34*100/4,J34+16*AA34),J34)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="32">
+        <f>IF(Z34="Invertida",MIN(C34*100/4,J34+16*AA34),J34)</f>
+        <v/>
+      </c>
+      <c r="AD34" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE33" s="33" t="n">
+      <c r="AE34" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="AF33" s="33" t="n">
+      <c r="AF34" s="33" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A4:A24"/>
     <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A4:A25"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A25:A33"/>
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="S2:U2"/>
+    <mergeCell ref="A26:A34"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="V2"/>
     <mergeCell ref="B2:B3"/>
@@ -5505,7 +5641,7 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="W2:W3"/>
   </mergeCells>
-  <conditionalFormatting sqref="W4:W33">
+  <conditionalFormatting sqref="W4:W34">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VERIFICA"</formula>
     </cfRule>
@@ -5520,13 +5656,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="Y4:Y33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y4:Y34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos!$A$19:$A$23</formula1>
     </dataValidation>
-    <dataValidation sqref="Z4:Z33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Z4:Z34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Invertida,Colgante"</formula1>
     </dataValidation>
-    <dataValidation sqref="O4:O33 R4:R33 U4:U33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O34 R4:R34 U4:U34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16,20,25"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5542,7 +5678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B66"/>
+  <dimension ref="A1:B68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5857,7 +5993,7 @@
       <c r="A36" s="36" t="inlineStr"/>
       <c r="B36" s="37" t="inlineStr">
         <is>
-          <t>Son VI 01a, VI 01b, VI 07a, VI 07b, VI 07c, VI 11a, VI 11b, VI 11c, VI 15a y VI 15b,</t>
+          <t>losa. Lo confirman las cotas del plano y el hecho de que el cielorraso sea de</t>
         </is>
       </c>
     </row>
@@ -5865,7 +6001,7 @@
       <c r="A37" s="36" t="inlineStr"/>
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t>identificadas por coincidir su eje con el contorno del edificio.</t>
+          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
@@ -5873,7 +6009,7 @@
       <c r="A38" s="36" t="inlineStr"/>
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>Esto define donde la losa aporta ala comprimida:</t>
+          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
@@ -5881,7 +6017,7 @@
       <c r="A39" s="36" t="inlineStr"/>
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
+          <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
@@ -5889,7 +6025,7 @@
       <c r="A40" s="36" t="inlineStr"/>
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
+          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
@@ -5897,7 +6033,7 @@
       <c r="A41" s="36" t="inlineStr"/>
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
+          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
@@ -5905,7 +6041,7 @@
       <c r="A42" s="36" t="inlineStr"/>
       <c r="B42" s="37" t="inlineStr">
         <is>
-          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
+          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
@@ -5913,7 +6049,7 @@
       <c r="A43" s="36" t="inlineStr"/>
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>PENDIENTE: una viga invertida de borde recibe la reaccion de la losa excentrica</t>
+          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
@@ -5921,39 +6057,39 @@
       <c r="A44" s="36" t="inlineStr"/>
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>respecto de su eje y queda sometida a TORSION. Esta planilla no la verifica.</t>
+          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="36" t="inlineStr"/>
-      <c r="B45" s="37" t="inlineStr"/>
+      <c r="B45" s="37" t="inlineStr">
+        <is>
+          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
+        </is>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="36" t="inlineStr">
-        <is>
-          <t>7. RESULTADO</t>
-        </is>
-      </c>
-      <c r="B46" s="36" t="inlineStr">
-        <is>
-          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
+      <c r="A46" s="36" t="inlineStr"/>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="36" t="inlineStr"/>
-      <c r="B47" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
-        </is>
-      </c>
+      <c r="B47" s="37" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="36" t="inlineStr"/>
-      <c r="B48" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
+      <c r="A48" s="36" t="inlineStr">
+        <is>
+          <t>7. RESULTADO</t>
+        </is>
+      </c>
+      <c r="B48" s="36" t="inlineStr">
+        <is>
+          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
@@ -5961,7 +6097,7 @@
       <c r="A49" s="36" t="inlineStr"/>
       <c r="B49" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
+          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
@@ -5969,7 +6105,7 @@
       <c r="A50" s="36" t="inlineStr"/>
       <c r="B50" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
+          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
@@ -5977,7 +6113,7 @@
       <c r="A51" s="36" t="inlineStr"/>
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
+          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
@@ -5985,7 +6121,7 @@
       <c r="A52" s="36" t="inlineStr"/>
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
+          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
@@ -5993,7 +6129,7 @@
       <c r="A53" s="36" t="inlineStr"/>
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
+          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6137,7 @@
       <c r="A54" s="36" t="inlineStr"/>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
+          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6145,7 @@
       <c r="A55" s="36" t="inlineStr"/>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
+          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6153,7 @@
       <c r="A56" s="36" t="inlineStr"/>
       <c r="B56" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
@@ -6025,63 +6161,63 @@
       <c r="A57" s="36" t="inlineStr"/>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="36" t="inlineStr"/>
-      <c r="B58" s="37" t="inlineStr"/>
+      <c r="B58" s="37" t="inlineStr">
+        <is>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+        </is>
+      </c>
     </row>
     <row r="59">
-      <c r="A59" s="36" t="inlineStr">
-        <is>
-          <t>8. ALCANCE</t>
-        </is>
-      </c>
+      <c r="A59" s="36" t="inlineStr"/>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="36" t="inlineStr"/>
-      <c r="B60" s="37" t="inlineStr">
+      <c r="B60" s="37" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="36" t="inlineStr">
+        <is>
+          <t>8. ALCANCE</t>
+        </is>
+      </c>
+      <c r="B61" s="37" t="inlineStr">
+        <is>
+          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="36" t="inlineStr"/>
+      <c r="B62" s="37" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="36" t="inlineStr"/>
-      <c r="B61" s="37" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="36" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B62" s="36" t="inlineStr">
-        <is>
-          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="36" t="inlineStr"/>
-      <c r="B63" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
-        </is>
-      </c>
+      <c r="B63" s="37" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="36" t="inlineStr"/>
-      <c r="B64" s="37" t="inlineStr">
-        <is>
-          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+      <c r="A64" s="36" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B64" s="36" t="inlineStr">
+        <is>
+          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
@@ -6089,13 +6225,29 @@
       <c r="A65" s="36" t="inlineStr"/>
       <c r="B65" s="37" t="inlineStr">
         <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="36" t="inlineStr"/>
       <c r="B66" s="37" t="inlineStr">
+        <is>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="36" t="inlineStr"/>
+      <c r="B67" s="37" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="36" t="inlineStr"/>
+      <c r="B68" s="37" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>

<commit_message>
Quitar VI 06, que no existe en obra
El computo metrico la lista como 15x70x14,00 pero el proyectista
confirma que no esta construida. Se la saca de la planilla para que
no quede una fila sin verificar que no corresponde a nada, y se deja
la nota en la memoria. La cuarta cara de L07 queda sin identificar.
Con esto las vigas quedan en 29 de 30: solo VCH 03a sin verificar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla vigas'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$33</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1123,31 +1123,6 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>4</col>
-      <colOff>0</colOff>
-      <row>33</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="2095500" cy="571500"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="31" name="Image 31" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1827,7 +1802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF34"/>
+  <dimension ref="A1:AF33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2785,11 +2760,11 @@
       <c r="A10" s="27" t="n"/>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>VI 06</t>
+          <t>VI 07a</t>
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>14</v>
+        <v>3.37</v>
       </c>
       <c r="D10" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AE10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD10)</f>
@@ -2827,24 +2802,20 @@
         <v/>
       </c>
       <c r="N10" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O10" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="P10" s="25">
         <f>IF(NOT(ISNUMBER(I10)),"---",IF(I10&lt;=0,"---",IF(I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)))*AC10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
         <v/>
       </c>
-      <c r="Q10" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R10" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+      <c r="Q10" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R10" s="24" t="n">
+        <v>12</v>
       </c>
       <c r="S10" s="25">
         <f>F10/(J10*0.85*K10)</f>
@@ -2855,10 +2826,10 @@
         <v/>
       </c>
       <c r="U10" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V10" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W10" s="7">
         <f>IF(OR(M10="REVISAR",P10="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M10&lt;&gt;"REVISAR",P10&lt;&gt;"REVISAR",IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -2866,7 +2837,7 @@
       </c>
       <c r="X10" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm).</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y10" s="24" t="inlineStr">
@@ -2891,24 +2862,24 @@
         <v/>
       </c>
       <c r="AD10" s="24" t="n">
-        <v>1.549</v>
+        <v>0.78</v>
       </c>
       <c r="AE10" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF10" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="27" t="n"/>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>VI 07a</t>
+          <t>VI 07b</t>
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>3.37</v>
+        <v>4.03</v>
       </c>
       <c r="D11" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AE11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD11)</f>
@@ -3006,7 +2977,7 @@
         <v/>
       </c>
       <c r="AD11" s="24" t="n">
-        <v>0.78</v>
+        <v>0</v>
       </c>
       <c r="AE11" s="24" t="n">
         <v>2.6</v>
@@ -3019,11 +2990,11 @@
       <c r="A12" s="27" t="n"/>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>VI 07b</t>
+          <t>VI 07c</t>
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>4.03</v>
+        <v>8.6</v>
       </c>
       <c r="D12" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AE12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD12)</f>
@@ -3061,20 +3032,20 @@
         <v/>
       </c>
       <c r="N12" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O12" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P12" s="25">
         <f>IF(NOT(ISNUMBER(I12)),"---",IF(I12&lt;=0,"---",IF(I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)))*AC12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
         <v/>
       </c>
       <c r="Q12" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R12" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S12" s="25">
         <f>F12/(J12*0.85*K12)</f>
@@ -3085,10 +3056,10 @@
         <v/>
       </c>
       <c r="U12" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V12" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W12" s="7">
         <f>IF(OR(M12="REVISAR",P12="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M12&lt;&gt;"REVISAR",P12&lt;&gt;"REVISAR",IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3096,12 +3067,12 @@
       </c>
       <c r="X12" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y12" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z12" s="24" t="inlineStr">
@@ -3121,24 +3092,24 @@
         <v/>
       </c>
       <c r="AD12" s="24" t="n">
-        <v>0</v>
+        <v>3.71</v>
       </c>
       <c r="AE12" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF12" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="27" t="n"/>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>VI 07c</t>
+          <t>VI 08a</t>
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>8.6</v>
+        <v>3.65</v>
       </c>
       <c r="D13" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AE13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD13)</f>
@@ -3176,20 +3147,20 @@
         <v/>
       </c>
       <c r="N13" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P13" s="25">
         <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)))*AC13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
         <v/>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S13" s="25">
         <f>F13/(J13*0.85*K13)</f>
@@ -3200,23 +3171,19 @@
         <v/>
       </c>
       <c r="U13" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V13" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W13" s="7">
         <f>IF(OR(M13="REVISAR",P13="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M13&lt;&gt;"REVISAR",P13&lt;&gt;"REVISAR",IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X13" s="26" t="inlineStr">
-        <is>
-          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X13" s="7" t="n"/>
       <c r="Y13" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z13" s="24" t="inlineStr">
@@ -3236,24 +3203,24 @@
         <v/>
       </c>
       <c r="AD13" s="24" t="n">
-        <v>3.71</v>
+        <v>1.065</v>
       </c>
       <c r="AE13" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF13" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="27" t="n"/>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>VI 08a</t>
+          <t>VI 08b</t>
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>3.65</v>
+        <v>4.87</v>
       </c>
       <c r="D14" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AE14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD14)</f>
@@ -3360,7 +3327,7 @@
       <c r="A15" s="27" t="n"/>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>VI 08b</t>
+          <t>VI 09</t>
         </is>
       </c>
       <c r="C15" s="22" t="n">
@@ -3411,11 +3378,15 @@
         <f>IF(NOT(ISNUMBER(I15)),"---",IF(I15&lt;=0,"---",IF(I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)))*AC15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
         <v/>
       </c>
-      <c r="Q15" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="R15" s="24" t="n">
-        <v>12</v>
+      <c r="Q15" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R15" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
       </c>
       <c r="S15" s="25">
         <f>F15/(J15*0.85*K15)</f>
@@ -3438,7 +3409,7 @@
       <c r="X15" s="7" t="n"/>
       <c r="Y15" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Simplemente apoyada</t>
         </is>
       </c>
       <c r="Z15" s="24" t="inlineStr">
@@ -3458,7 +3429,7 @@
         <v/>
       </c>
       <c r="AD15" s="24" t="n">
-        <v>1.065</v>
+        <v>1.549</v>
       </c>
       <c r="AE15" s="24" t="n">
         <v>2.6</v>
@@ -3471,11 +3442,11 @@
       <c r="A16" s="27" t="n"/>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>VI 09</t>
+          <t>VI 10a</t>
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>4.87</v>
+        <v>2.55</v>
       </c>
       <c r="D16" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AE16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD16)</f>
@@ -3522,15 +3493,11 @@
         <f>IF(NOT(ISNUMBER(I16)),"---",IF(I16&lt;=0,"---",IF(I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)))*AC16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
         <v/>
       </c>
-      <c r="Q16" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R16" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+      <c r="Q16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" s="24" t="n">
+        <v>12</v>
       </c>
       <c r="S16" s="25">
         <f>F16/(J16*0.85*K16)</f>
@@ -3553,7 +3520,7 @@
       <c r="X16" s="7" t="n"/>
       <c r="Y16" s="24" t="inlineStr">
         <is>
-          <t>Simplemente apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z16" s="24" t="inlineStr">
@@ -3573,7 +3540,7 @@
         <v/>
       </c>
       <c r="AD16" s="24" t="n">
-        <v>1.549</v>
+        <v>0</v>
       </c>
       <c r="AE16" s="24" t="n">
         <v>2.6</v>
@@ -3586,11 +3553,11 @@
       <c r="A17" s="27" t="n"/>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>VI 10a</t>
+          <t>VI 10b</t>
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>2.55</v>
+        <v>4</v>
       </c>
       <c r="D17" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AE17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD17)</f>
@@ -3684,7 +3651,7 @@
         <v/>
       </c>
       <c r="AD17" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE17" s="24" t="n">
         <v>2.6</v>
@@ -3697,11 +3664,11 @@
       <c r="A18" s="27" t="n"/>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>VI 10b</t>
+          <t>VI 10c</t>
         </is>
       </c>
       <c r="C18" s="22" t="n">
-        <v>4</v>
+        <v>3.6</v>
       </c>
       <c r="D18" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AE18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD18)</f>
@@ -3795,7 +3762,7 @@
         <v/>
       </c>
       <c r="AD18" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE18" s="24" t="n">
         <v>2.6</v>
@@ -3808,11 +3775,11 @@
       <c r="A19" s="27" t="n"/>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>VI 10c</t>
+          <t>VI 11a</t>
         </is>
       </c>
       <c r="C19" s="22" t="n">
-        <v>3.6</v>
+        <v>7.68</v>
       </c>
       <c r="D19" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AE19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD19)</f>
@@ -3850,20 +3817,20 @@
         <v/>
       </c>
       <c r="N19" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O19" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P19" s="25">
         <f>IF(NOT(ISNUMBER(I19)),"---",IF(I19&lt;=0,"---",IF(I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)))*AC19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
         <v/>
       </c>
       <c r="Q19" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R19" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S19" s="25">
         <f>F19/(J19*0.85*K19)</f>
@@ -3877,16 +3844,20 @@
         <v>6</v>
       </c>
       <c r="V19" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W19" s="7">
         <f>IF(OR(M19="REVISAR",P19="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M19&lt;&gt;"REVISAR",P19&lt;&gt;"REVISAR",IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X19" s="7" t="n"/>
+      <c r="X19" s="26" t="inlineStr">
+        <is>
+          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y19" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z19" s="24" t="inlineStr">
@@ -3906,7 +3877,7 @@
         <v/>
       </c>
       <c r="AD19" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE19" s="24" t="n">
         <v>2.6</v>
@@ -3919,11 +3890,11 @@
       <c r="A20" s="27" t="n"/>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>VI 11a</t>
+          <t>VI 11b</t>
         </is>
       </c>
       <c r="C20" s="22" t="n">
-        <v>7.68</v>
+        <v>3.45</v>
       </c>
       <c r="D20" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AE20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD20)</f>
@@ -3961,20 +3932,20 @@
         <v/>
       </c>
       <c r="N20" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O20" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P20" s="25">
         <f>IF(NOT(ISNUMBER(I20)),"---",IF(I20&lt;=0,"---",IF(I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)))*AC20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
         <v/>
       </c>
       <c r="Q20" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R20" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S20" s="25">
         <f>F20/(J20*0.85*K20)</f>
@@ -3988,7 +3959,7 @@
         <v>6</v>
       </c>
       <c r="V20" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W20" s="7">
         <f>IF(OR(M20="REVISAR",P20="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M20&lt;&gt;"REVISAR",P20&lt;&gt;"REVISAR",IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3996,12 +3967,12 @@
       </c>
       <c r="X20" s="26" t="inlineStr">
         <is>
-          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y20" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z20" s="24" t="inlineStr">
@@ -4021,7 +3992,7 @@
         <v/>
       </c>
       <c r="AD20" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE20" s="24" t="n">
         <v>2.6</v>
@@ -4034,11 +4005,11 @@
       <c r="A21" s="27" t="n"/>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>VI 11b</t>
+          <t>VI 11c</t>
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>3.45</v>
+        <v>5.02</v>
       </c>
       <c r="D21" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AE21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD21)</f>
@@ -4136,7 +4107,7 @@
         <v/>
       </c>
       <c r="AD21" s="24" t="n">
-        <v>0</v>
+        <v>1.549</v>
       </c>
       <c r="AE21" s="24" t="n">
         <v>2.6</v>
@@ -4149,11 +4120,11 @@
       <c r="A22" s="27" t="n"/>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>VI 11c</t>
+          <t>VCH 03a</t>
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>5.02</v>
+        <v>3.71</v>
       </c>
       <c r="D22" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AE22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD22)</f>
@@ -4177,21 +4148,21 @@
         <v/>
       </c>
       <c r="J22" s="24" t="n">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="K22" s="7">
         <f>L22-AF22</f>
         <v/>
       </c>
       <c r="L22" s="24" t="n">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="M22" s="25">
         <f>IF(NOT(ISNUMBER(H22)),"---",IF(H22&lt;=0,"---",IF(H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)))*AB22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="N22" s="24" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="O22" s="24" t="n">
         <v>12</v>
@@ -4201,10 +4172,10 @@
         <v/>
       </c>
       <c r="Q22" s="24" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="R22" s="24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="S22" s="25">
         <f>F22/(J22*0.85*K22)</f>
@@ -4215,10 +4186,10 @@
         <v/>
       </c>
       <c r="U22" s="24" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="V22" s="24" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="W22" s="7">
         <f>IF(OR(M22="REVISAR",P22="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M22&lt;&gt;"REVISAR",P22&lt;&gt;"REVISAR",IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4226,7 +4197,7 @@
       </c>
       <c r="X22" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
         </is>
       </c>
       <c r="Y22" s="24" t="inlineStr">
@@ -4236,7 +4207,7 @@
       </c>
       <c r="Z22" s="24" t="inlineStr">
         <is>
-          <t>Invertida</t>
+          <t>Colgante</t>
         </is>
       </c>
       <c r="AA22" s="24" t="n">
@@ -4251,7 +4222,7 @@
         <v/>
       </c>
       <c r="AD22" s="24" t="n">
-        <v>1.549</v>
+        <v>2.1</v>
       </c>
       <c r="AE22" s="24" t="n">
         <v>2.6</v>
@@ -4264,11 +4235,11 @@
       <c r="A23" s="27" t="n"/>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>VCH 03a</t>
+          <t>VCH 03b</t>
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>3.71</v>
+        <v>2.13</v>
       </c>
       <c r="D23" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AE23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD23)</f>
@@ -4306,20 +4277,20 @@
         <v/>
       </c>
       <c r="N23" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="O23" s="24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="P23" s="25">
         <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)))*AC23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="Q23" s="24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R23" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S23" s="25">
         <f>F23/(J23*0.85*K23)</f>
@@ -4341,7 +4312,7 @@
       </c>
       <c r="X23" s="26" t="inlineStr">
         <is>
-          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
         </is>
       </c>
       <c r="Y23" s="24" t="inlineStr">
@@ -4376,251 +4347,247 @@
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="21" t="inlineStr">
-        <is>
-          <t>VCH 03b</t>
-        </is>
-      </c>
-      <c r="C24" s="22" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="D24" s="23">
+      <c r="A24" s="28" t="n"/>
+      <c r="B24" s="29" t="inlineStr">
+        <is>
+          <t>VCH 05</t>
+        </is>
+      </c>
+      <c r="C24" s="30" t="n">
+        <v>3.71</v>
+      </c>
+      <c r="D24" s="31">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
         <v/>
       </c>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="23">
+      <c r="E24" s="32" t="n"/>
+      <c r="F24" s="31">
         <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
         <v/>
       </c>
-      <c r="G24" s="23">
+      <c r="G24" s="31">
         <f>F24</f>
         <v/>
       </c>
-      <c r="H24" s="23">
+      <c r="H24" s="31">
         <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
         <v/>
       </c>
-      <c r="I24" s="23">
+      <c r="I24" s="31">
         <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
         <v/>
       </c>
-      <c r="J24" s="24" t="n">
-        <v>40</v>
-      </c>
-      <c r="K24" s="7">
+      <c r="J24" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="K24" s="32">
         <f>L24-AF24</f>
         <v/>
       </c>
-      <c r="L24" s="24" t="n">
-        <v>13</v>
-      </c>
-      <c r="M24" s="25">
+      <c r="L24" s="33" t="n">
+        <v>45</v>
+      </c>
+      <c r="M24" s="34">
         <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
         <v/>
       </c>
-      <c r="N24" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="O24" s="24" t="n">
+      <c r="N24" s="33" t="n">
+        <v>2</v>
+      </c>
+      <c r="O24" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P24" s="34">
+        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="33" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R24" s="33" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="S24" s="34">
+        <f>F24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="T24" s="34">
+        <f>G24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="U24" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="P24" s="25">
-        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="R24" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="S24" s="25">
-        <f>F24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="T24" s="25">
-        <f>G24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="U24" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="V24" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="W24" s="7">
+      <c r="V24" s="33" t="n">
+        <v>20</v>
+      </c>
+      <c r="W24" s="32">
         <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X24" s="26" t="inlineStr">
-        <is>
-          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
-        </is>
-      </c>
-      <c r="Y24" s="24" t="inlineStr">
+      <c r="X24" s="32" t="n"/>
+      <c r="Y24" s="33" t="inlineStr">
+        <is>
+          <t>Simplemente apoyada</t>
+        </is>
+      </c>
+      <c r="Z24" s="33" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA24" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB24" s="32">
+        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="32">
+        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AD24" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="33" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AF24" s="33" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>TECHO</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="inlineStr">
+        <is>
+          <t>VI 12</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="D25" s="23">
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="23">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="23">
+        <f>F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="23">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
+        <v/>
+      </c>
+      <c r="I25" s="23">
+        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
+        <v/>
+      </c>
+      <c r="J25" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="K25" s="7">
+        <f>L25-AF25</f>
+        <v/>
+      </c>
+      <c r="L25" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="M25" s="25">
+        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="N25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="O25" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="P25" s="25">
+        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="R25" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="S25" s="25">
+        <f>F25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="T25" s="25">
+        <f>G25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="U25" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="V25" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="W25" s="7">
+        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X25" s="7" t="n"/>
+      <c r="Y25" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
         </is>
       </c>
-      <c r="Z24" s="24" t="inlineStr">
-        <is>
-          <t>Colgante</t>
-        </is>
-      </c>
-      <c r="AA24" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB24" s="7">
-        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AC24" s="7">
-        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AD24" s="24" t="n">
+      <c r="Z25" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA25" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB25" s="7">
+        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="7">
+        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AD25" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE24" s="24" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="AF24" s="24" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="28" t="n"/>
-      <c r="B25" s="29" t="inlineStr">
-        <is>
-          <t>VCH 05</t>
-        </is>
-      </c>
-      <c r="C25" s="30" t="n">
-        <v>3.71</v>
-      </c>
-      <c r="D25" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD25)</f>
-        <v/>
-      </c>
-      <c r="E25" s="32" t="n"/>
-      <c r="F25" s="31">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
-        <v/>
-      </c>
-      <c r="G25" s="31">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="H25" s="31">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
-        <v/>
-      </c>
-      <c r="I25" s="31">
-        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
-        <v/>
-      </c>
-      <c r="J25" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="K25" s="32">
-        <f>L25-AF25</f>
-        <v/>
-      </c>
-      <c r="L25" s="33" t="n">
-        <v>45</v>
-      </c>
-      <c r="M25" s="34">
-        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="N25" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="O25" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P25" s="34">
-        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="33" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R25" s="33" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="S25" s="34">
-        <f>F25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="T25" s="34">
-        <f>G25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="U25" s="33" t="n">
+      <c r="AE25" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" s="24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="27" t="n"/>
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t>VI 13a</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="V25" s="33" t="n">
-        <v>20</v>
-      </c>
-      <c r="W25" s="32">
-        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X25" s="32" t="n"/>
-      <c r="Y25" s="33" t="inlineStr">
-        <is>
-          <t>Simplemente apoyada</t>
-        </is>
-      </c>
-      <c r="Z25" s="33" t="inlineStr">
-        <is>
-          <t>Colgante</t>
-        </is>
-      </c>
-      <c r="AA25" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB25" s="32">
-        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AC25" s="32">
-        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AD25" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE25" s="33" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="AF25" s="33" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="20" t="inlineStr">
-        <is>
-          <t>TECHO</t>
-        </is>
-      </c>
-      <c r="B26" s="21" t="inlineStr">
-        <is>
-          <t>VI 12</t>
-        </is>
-      </c>
-      <c r="C26" s="22" t="n">
-        <v>9.9</v>
-      </c>
       <c r="D26" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD26)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD26)</f>
         <v/>
       </c>
       <c r="E26" s="7" t="n"/>
@@ -4658,7 +4625,7 @@
         <v>2</v>
       </c>
       <c r="O26" s="24" t="n">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="P26" s="25">
         <f>IF(NOT(ISNUMBER(I26)),"---",IF(I26&lt;=0,"---",IF(I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)))*AC26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
@@ -4668,7 +4635,7 @@
         <v>2</v>
       </c>
       <c r="R26" s="24" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="S26" s="25">
         <f>F26/(J26*0.85*K26)</f>
@@ -4711,7 +4678,7 @@
         <v/>
       </c>
       <c r="AD26" s="24" t="n">
-        <v>2.1</v>
+        <v>3.799</v>
       </c>
       <c r="AE26" s="24" t="n">
         <v>1</v>
@@ -4724,14 +4691,14 @@
       <c r="A27" s="27" t="n"/>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>VI 13a</t>
+          <t>VI 13b</t>
         </is>
       </c>
       <c r="C27" s="22" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D27" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD27)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD27)</f>
         <v/>
       </c>
       <c r="E27" s="7" t="n"/>
@@ -4766,20 +4733,20 @@
         <v/>
       </c>
       <c r="N27" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O27" s="24" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="P27" s="25">
         <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)))*AC27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="Q27" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R27" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="S27" s="25">
         <f>F27/(J27*0.85*K27)</f>
@@ -4793,7 +4760,7 @@
         <v>6</v>
       </c>
       <c r="V27" s="24" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="W27" s="7">
         <f>IF(OR(M27="REVISAR",P27="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M27&lt;&gt;"REVISAR",P27&lt;&gt;"REVISAR",IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4822,7 +4789,7 @@
         <v/>
       </c>
       <c r="AD27" s="24" t="n">
-        <v>3.799</v>
+        <v>2.1</v>
       </c>
       <c r="AE27" s="24" t="n">
         <v>1</v>
@@ -4835,14 +4802,14 @@
       <c r="A28" s="27" t="n"/>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>VI 13b</t>
+          <t>VI 14</t>
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>3.75</v>
+        <v>6</v>
       </c>
       <c r="D28" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD28)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD28)</f>
         <v/>
       </c>
       <c r="E28" s="7" t="n"/>
@@ -4933,7 +4900,7 @@
         <v/>
       </c>
       <c r="AD28" s="24" t="n">
-        <v>2.1</v>
+        <v>1.699</v>
       </c>
       <c r="AE28" s="24" t="n">
         <v>1</v>
@@ -4946,14 +4913,14 @@
       <c r="A29" s="27" t="n"/>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>VI 14</t>
+          <t>VI 15a</t>
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>6</v>
+        <v>4.03</v>
       </c>
       <c r="D29" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD29)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD29)</f>
         <v/>
       </c>
       <c r="E29" s="7" t="n"/>
@@ -5021,7 +4988,11 @@
         <f>IF(OR(M29="REVISAR",P29="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M29&lt;&gt;"REVISAR",P29&lt;&gt;"REVISAR",IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X29" s="7" t="n"/>
+      <c r="X29" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y29" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5044,7 +5015,7 @@
         <v/>
       </c>
       <c r="AD29" s="24" t="n">
-        <v>1.699</v>
+        <v>0</v>
       </c>
       <c r="AE29" s="24" t="n">
         <v>1</v>
@@ -5057,14 +5028,14 @@
       <c r="A30" s="27" t="n"/>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>VI 15a</t>
+          <t>VI 15b</t>
         </is>
       </c>
       <c r="C30" s="22" t="n">
-        <v>4.03</v>
+        <v>4.85</v>
       </c>
       <c r="D30" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD30)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD30)</f>
         <v/>
       </c>
       <c r="E30" s="7" t="n"/>
@@ -5159,7 +5130,7 @@
         <v/>
       </c>
       <c r="AD30" s="24" t="n">
-        <v>0</v>
+        <v>1.699</v>
       </c>
       <c r="AE30" s="24" t="n">
         <v>1</v>
@@ -5172,14 +5143,14 @@
       <c r="A31" s="27" t="n"/>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>VI 15b</t>
+          <t>VI 16a</t>
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>4.85</v>
+        <v>3.58</v>
       </c>
       <c r="D31" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD31)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD31)</f>
         <v/>
       </c>
       <c r="E31" s="7" t="n"/>
@@ -5247,11 +5218,7 @@
         <f>IF(OR(M31="REVISAR",P31="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M31&lt;&gt;"REVISAR",P31&lt;&gt;"REVISAR",IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X31" s="26" t="inlineStr">
-        <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X31" s="7" t="n"/>
       <c r="Y31" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5287,14 +5254,14 @@
       <c r="A32" s="27" t="n"/>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>VI 16a</t>
+          <t>VI 16b</t>
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>3.58</v>
+        <v>1.12</v>
       </c>
       <c r="D32" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD32)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD32)</f>
         <v/>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -5395,241 +5362,130 @@
       </c>
     </row>
     <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="21" t="inlineStr">
-        <is>
-          <t>VI 16b</t>
-        </is>
-      </c>
-      <c r="C33" s="22" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="D33" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="23">
+      <c r="A33" s="28" t="n"/>
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>VI 17</t>
+        </is>
+      </c>
+      <c r="C33" s="30" t="n">
+        <v>4.35</v>
+      </c>
+      <c r="D33" s="31">
+        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD33)</f>
+        <v/>
+      </c>
+      <c r="E33" s="32" t="n"/>
+      <c r="F33" s="31">
         <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
         <v/>
       </c>
-      <c r="G33" s="23">
+      <c r="G33" s="31">
         <f>F33</f>
         <v/>
       </c>
-      <c r="H33" s="23">
+      <c r="H33" s="31">
         <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
         <v/>
       </c>
-      <c r="I33" s="23">
+      <c r="I33" s="31">
         <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
         <v/>
       </c>
-      <c r="J33" s="24" t="n">
+      <c r="J33" s="33" t="n">
         <v>15</v>
       </c>
-      <c r="K33" s="7">
+      <c r="K33" s="32">
         <f>L33-AF33</f>
         <v/>
       </c>
-      <c r="L33" s="24" t="n">
+      <c r="L33" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="M33" s="25">
+      <c r="M33" s="34">
         <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
         <v/>
       </c>
-      <c r="N33" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="O33" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="P33" s="25">
+      <c r="N33" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O33" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P33" s="34">
         <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
         <v/>
       </c>
-      <c r="Q33" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="R33" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="S33" s="25">
+      <c r="Q33" s="33" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R33" s="33" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="S33" s="34">
         <f>F33/(J33*0.85*K33)</f>
         <v/>
       </c>
-      <c r="T33" s="25">
+      <c r="T33" s="34">
         <f>G33/(J33*0.85*K33)</f>
         <v/>
       </c>
-      <c r="U33" s="24" t="n">
+      <c r="U33" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="V33" s="24" t="n">
+      <c r="V33" s="33" t="n">
         <v>30</v>
       </c>
-      <c r="W33" s="7">
+      <c r="W33" s="32">
         <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="24" t="inlineStr">
-        <is>
-          <t>Continua</t>
-        </is>
-      </c>
-      <c r="Z33" s="24" t="inlineStr">
+      <c r="X33" s="32" t="n"/>
+      <c r="Y33" s="33" t="inlineStr">
+        <is>
+          <t>Simplemente apoyada</t>
+        </is>
+      </c>
+      <c r="Z33" s="33" t="inlineStr">
         <is>
           <t>Invertida</t>
         </is>
       </c>
-      <c r="AA33" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB33" s="7">
+      <c r="AA33" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB33" s="32">
         <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
         <v/>
       </c>
-      <c r="AC33" s="7">
+      <c r="AC33" s="32">
         <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
         <v/>
       </c>
-      <c r="AD33" s="24" t="n">
-        <v>1.699</v>
-      </c>
-      <c r="AE33" s="24" t="n">
+      <c r="AD33" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="AF33" s="24" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" ht="46" customHeight="1">
-      <c r="A34" s="28" t="n"/>
-      <c r="B34" s="29" t="inlineStr">
-        <is>
-          <t>VI 17</t>
-        </is>
-      </c>
-      <c r="C34" s="30" t="n">
-        <v>4.35</v>
-      </c>
-      <c r="D34" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD34+Datos!$B$7*J34*L34/10000+Datos!$B$16*AE34)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD34)</f>
-        <v/>
-      </c>
-      <c r="E34" s="32" t="n"/>
-      <c r="F34" s="31">
-        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,4,0)*D34*C34</f>
-        <v/>
-      </c>
-      <c r="G34" s="31">
-        <f>F34</f>
-        <v/>
-      </c>
-      <c r="H34" s="31">
-        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,2,0)*D34*C34^2</f>
-        <v/>
-      </c>
-      <c r="I34" s="31">
-        <f>IF(VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)*D34*C34^2)</f>
-        <v/>
-      </c>
-      <c r="J34" s="33" t="n">
-        <v>15</v>
-      </c>
-      <c r="K34" s="32">
-        <f>L34-AF34</f>
-        <v/>
-      </c>
-      <c r="L34" s="33" t="n">
-        <v>70</v>
-      </c>
-      <c r="M34" s="34">
-        <f>IF(NOT(ISNUMBER(H34)),"---",IF(H34&lt;=0,"---",IF(H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)))*AB34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
-        <v/>
-      </c>
-      <c r="N34" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="O34" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P34" s="34">
-        <f>IF(NOT(ISNUMBER(I34)),"---",IF(I34&lt;=0,"---",IF(I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)))*AC34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
-        <v/>
-      </c>
-      <c r="Q34" s="33" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R34" s="33" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="S34" s="34">
-        <f>F34/(J34*0.85*K34)</f>
-        <v/>
-      </c>
-      <c r="T34" s="34">
-        <f>G34/(J34*0.85*K34)</f>
-        <v/>
-      </c>
-      <c r="U34" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="V34" s="33" t="n">
-        <v>30</v>
-      </c>
-      <c r="W34" s="32">
-        <f>IF(OR(M34="REVISAR",P34="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M34&lt;&gt;"REVISAR",P34&lt;&gt;"REVISAR",IF(ISNUMBER(M34),N34*PI()*(O34/10)^2/4&gt;=M34,TRUE),IF(ISNUMBER(P34),Q34*PI()*(R34/10)^2/4&gt;=P34,TRUE),IF(ISNUMBER(M34),M34&lt;=0.0163*AB34*K34,TRUE),IF(ISNUMBER(P34),P34&lt;=0.0163*AC34*K34,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F34&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J34*K34+2*PI()*(U34/10)^2/4*Datos!$B$6*K34/V34)),"NO VERIF. CORTE",IF(NOT(L34&gt;=C34*100/VLOOKUP(Y34,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X34" s="32" t="n"/>
-      <c r="Y34" s="33" t="inlineStr">
-        <is>
-          <t>Simplemente apoyada</t>
-        </is>
-      </c>
-      <c r="Z34" s="33" t="inlineStr">
-        <is>
-          <t>Invertida</t>
-        </is>
-      </c>
-      <c r="AA34" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB34" s="32">
-        <f>IF(Z34="Colgante",MIN(C34*100/4,J34+16*AA34),J34)</f>
-        <v/>
-      </c>
-      <c r="AC34" s="32">
-        <f>IF(Z34="Invertida",MIN(C34*100/4,J34+16*AA34),J34)</f>
-        <v/>
-      </c>
-      <c r="AD34" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE34" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF34" s="33" t="n">
+      <c r="AF33" s="33" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="F2:G2"/>
+    <mergeCell ref="A4:A24"/>
     <mergeCell ref="J2:L2"/>
-    <mergeCell ref="A4:A25"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="A25:A33"/>
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="S2:U2"/>
-    <mergeCell ref="A26:A34"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="V2"/>
     <mergeCell ref="B2:B3"/>
@@ -5641,7 +5497,7 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="W2:W3"/>
   </mergeCells>
-  <conditionalFormatting sqref="W4:W34">
+  <conditionalFormatting sqref="W4:W33">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VERIFICA"</formula>
     </cfRule>
@@ -5656,13 +5512,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="Y4:Y34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y4:Y33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos!$A$19:$A$23</formula1>
     </dataValidation>
-    <dataValidation sqref="Z4:Z34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Z4:Z33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Invertida,Colgante"</formula1>
     </dataValidation>
-    <dataValidation sqref="O4:O34 R4:R34 U4:U34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O33 R4:R33 U4:U33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16,20,25"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5678,7 +5534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B68"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -6001,7 +5857,7 @@
       <c r="A37" s="36" t="inlineStr"/>
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
+          <t>NOTA: el computo metrico lista una VI 06 de 15x70x14,00 que no existe en obra;</t>
         </is>
       </c>
     </row>
@@ -6009,7 +5865,7 @@
       <c r="A38" s="36" t="inlineStr"/>
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
+          <t>por eso no figura en esta planilla. La cuarta cara de L07 apoya en otro elemento.</t>
         </is>
       </c>
     </row>
@@ -6017,7 +5873,7 @@
       <c r="A39" s="36" t="inlineStr"/>
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>Esto define donde la losa aporta ala comprimida:</t>
+          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
@@ -6025,7 +5881,7 @@
       <c r="A40" s="36" t="inlineStr"/>
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
+          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
@@ -6033,7 +5889,7 @@
       <c r="A41" s="36" t="inlineStr"/>
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
+          <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
@@ -6041,7 +5897,7 @@
       <c r="A42" s="36" t="inlineStr"/>
       <c r="B42" s="37" t="inlineStr">
         <is>
-          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
+          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
@@ -6049,7 +5905,7 @@
       <c r="A43" s="36" t="inlineStr"/>
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
+          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
@@ -6057,7 +5913,7 @@
       <c r="A44" s="36" t="inlineStr"/>
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
+          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
@@ -6065,7 +5921,7 @@
       <c r="A45" s="36" t="inlineStr"/>
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
+          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
@@ -6073,39 +5929,39 @@
       <c r="A46" s="36" t="inlineStr"/>
       <c r="B46" s="37" t="inlineStr">
         <is>
-          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
+          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="36" t="inlineStr"/>
-      <c r="B47" s="37" t="inlineStr"/>
+      <c r="B47" s="37" t="inlineStr">
+        <is>
+          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="A48" s="36" t="inlineStr">
-        <is>
-          <t>7. RESULTADO</t>
-        </is>
-      </c>
-      <c r="B48" s="36" t="inlineStr">
-        <is>
-          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
+      <c r="A48" s="36" t="inlineStr"/>
+      <c r="B48" s="37" t="inlineStr">
+        <is>
+          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="36" t="inlineStr"/>
-      <c r="B49" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
-        </is>
-      </c>
+      <c r="B49" s="37" t="inlineStr"/>
     </row>
     <row r="50">
-      <c r="A50" s="36" t="inlineStr"/>
-      <c r="B50" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
+      <c r="A50" s="36" t="inlineStr">
+        <is>
+          <t>7. RESULTADO</t>
+        </is>
+      </c>
+      <c r="B50" s="36" t="inlineStr">
+        <is>
+          <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
         </is>
       </c>
     </row>
@@ -6113,7 +5969,7 @@
       <c r="A51" s="36" t="inlineStr"/>
       <c r="B51" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
+          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
@@ -6121,7 +5977,7 @@
       <c r="A52" s="36" t="inlineStr"/>
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
+          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
@@ -6129,7 +5985,7 @@
       <c r="A53" s="36" t="inlineStr"/>
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
+          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
@@ -6137,7 +5993,7 @@
       <c r="A54" s="36" t="inlineStr"/>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
+          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6001,7 @@
       <c r="A55" s="36" t="inlineStr"/>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
+          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
@@ -6153,7 +6009,7 @@
       <c r="A56" s="36" t="inlineStr"/>
       <c r="B56" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
+          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6017,7 @@
       <c r="A57" s="36" t="inlineStr"/>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
+          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
@@ -6169,7 +6025,7 @@
       <c r="A58" s="36" t="inlineStr"/>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
@@ -6177,63 +6033,63 @@
       <c r="A59" s="36" t="inlineStr"/>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="36" t="inlineStr"/>
-      <c r="B60" s="37" t="inlineStr"/>
+      <c r="B60" s="37" t="inlineStr">
+        <is>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+        </is>
+      </c>
     </row>
     <row r="61">
-      <c r="A61" s="36" t="inlineStr">
-        <is>
-          <t>8. ALCANCE</t>
-        </is>
-      </c>
+      <c r="A61" s="36" t="inlineStr"/>
       <c r="B61" s="37" t="inlineStr">
         <is>
-          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="36" t="inlineStr"/>
-      <c r="B62" s="37" t="inlineStr">
+      <c r="B62" s="37" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="36" t="inlineStr">
+        <is>
+          <t>8. ALCANCE</t>
+        </is>
+      </c>
+      <c r="B63" s="37" t="inlineStr">
+        <is>
+          <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="36" t="inlineStr"/>
+      <c r="B64" s="37" t="inlineStr">
         <is>
           <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="36" t="inlineStr"/>
-      <c r="B63" s="37" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="36" t="inlineStr">
-        <is>
-          <t>LIMITACIONES</t>
-        </is>
-      </c>
-      <c r="B64" s="36" t="inlineStr">
-        <is>
-          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="36" t="inlineStr"/>
-      <c r="B65" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
-        </is>
-      </c>
+      <c r="B65" s="37" t="inlineStr"/>
     </row>
     <row r="66">
-      <c r="A66" s="36" t="inlineStr"/>
-      <c r="B66" s="37" t="inlineStr">
-        <is>
-          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+      <c r="A66" s="36" t="inlineStr">
+        <is>
+          <t>LIMITACIONES</t>
+        </is>
+      </c>
+      <c r="B66" s="36" t="inlineStr">
+        <is>
+          <t>El ancho tributario B esta relevado solo en</t>
         </is>
       </c>
     </row>
@@ -6241,13 +6097,29 @@
       <c r="A67" s="36" t="inlineStr"/>
       <c r="B67" s="37" t="inlineStr">
         <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="36" t="inlineStr"/>
       <c r="B68" s="37" t="inlineStr">
+        <is>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="36" t="inlineStr"/>
+      <c r="B69" s="37" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="36" t="inlineStr"/>
+      <c r="B70" s="37" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>

<commit_message>
Reponer VI 06 y resolverla como viga continua de tres tramos
El proyectista confirma que existe y que L07 apoya en ella. Sobre su
eje, deducido como el cuarto borde de L07, hay cuatro columnas: la
viga de 14 m trabaja como continua de tres tramos de 4,10, 4,32 y
6,53 m. Calculada con el mayor, verifica con 2d20 en el apoyo.
Las vigas quedan en 30 de 31.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Planilla vigas'!$1:$3</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$33</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Planilla vigas'!$A$1:$X$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1123,6 +1123,31 @@
     </pic>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2095500" cy="571500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId31"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1802,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF33"/>
+  <dimension ref="A1:AF34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2760,11 +2785,11 @@
       <c r="A10" s="27" t="n"/>
       <c r="B10" s="21" t="inlineStr">
         <is>
-          <t>VI 07a</t>
+          <t>VI 06</t>
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>3.37</v>
+        <v>6.53</v>
       </c>
       <c r="D10" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AE10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD10)</f>
@@ -2812,10 +2837,10 @@
         <v/>
       </c>
       <c r="Q10" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R10" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="S10" s="25">
         <f>F10/(J10*0.85*K10)</f>
@@ -2837,7 +2862,7 @@
       </c>
       <c r="X10" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07.</t>
         </is>
       </c>
       <c r="Y10" s="24" t="inlineStr">
@@ -2862,7 +2887,7 @@
         <v/>
       </c>
       <c r="AD10" s="24" t="n">
-        <v>0.78</v>
+        <v>1.549</v>
       </c>
       <c r="AE10" s="24" t="n">
         <v>2.6</v>
@@ -2875,11 +2900,11 @@
       <c r="A11" s="27" t="n"/>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>VI 07b</t>
+          <t>VI 07a</t>
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>4.03</v>
+        <v>3.37</v>
       </c>
       <c r="D11" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AE11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD11)</f>
@@ -2977,7 +3002,7 @@
         <v/>
       </c>
       <c r="AD11" s="24" t="n">
-        <v>0</v>
+        <v>0.78</v>
       </c>
       <c r="AE11" s="24" t="n">
         <v>2.6</v>
@@ -2990,11 +3015,11 @@
       <c r="A12" s="27" t="n"/>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>VI 07c</t>
+          <t>VI 07b</t>
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>8.6</v>
+        <v>4.03</v>
       </c>
       <c r="D12" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AE12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD12)</f>
@@ -3032,20 +3057,20 @@
         <v/>
       </c>
       <c r="N12" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O12" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P12" s="25">
         <f>IF(NOT(ISNUMBER(I12)),"---",IF(I12&lt;=0,"---",IF(I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I12*100/(Datos!$B$8*AC12*K12^2*Datos!$B$5)))*AC12*K12*Datos!$B$5/Datos!$B$6,0.0033*J12*K12))))</f>
         <v/>
       </c>
       <c r="Q12" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="R12" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S12" s="25">
         <f>F12/(J12*0.85*K12)</f>
@@ -3056,10 +3081,10 @@
         <v/>
       </c>
       <c r="U12" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="V12" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W12" s="7">
         <f>IF(OR(M12="REVISAR",P12="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M12&lt;&gt;"REVISAR",P12&lt;&gt;"REVISAR",IF(ISNUMBER(M12),N12*PI()*(O12/10)^2/4&gt;=M12,TRUE),IF(ISNUMBER(P12),Q12*PI()*(R12/10)^2/4&gt;=P12,TRUE),IF(ISNUMBER(M12),M12&lt;=0.0163*AB12*K12,TRUE),IF(ISNUMBER(P12),P12&lt;=0.0163*AC12*K12,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F12&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J12*K12+2*PI()*(U12/10)^2/4*Datos!$B$6*K12/V12)),"NO VERIF. CORTE",IF(NOT(L12&gt;=C12*100/VLOOKUP(Y12,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3067,12 +3092,12 @@
       </c>
       <c r="X12" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y12" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z12" s="24" t="inlineStr">
@@ -3092,24 +3117,24 @@
         <v/>
       </c>
       <c r="AD12" s="24" t="n">
-        <v>3.71</v>
+        <v>0</v>
       </c>
       <c r="AE12" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF12" s="24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="27" t="n"/>
       <c r="B13" s="21" t="inlineStr">
         <is>
-          <t>VI 08a</t>
+          <t>VI 07c</t>
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>3.65</v>
+        <v>8.6</v>
       </c>
       <c r="D13" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AE13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD13)</f>
@@ -3147,20 +3172,20 @@
         <v/>
       </c>
       <c r="N13" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O13" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P13" s="25">
         <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)))*AC13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
         <v/>
       </c>
       <c r="Q13" s="24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R13" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S13" s="25">
         <f>F13/(J13*0.85*K13)</f>
@@ -3171,19 +3196,23 @@
         <v/>
       </c>
       <c r="U13" s="24" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V13" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W13" s="7">
         <f>IF(OR(M13="REVISAR",P13="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M13&lt;&gt;"REVISAR",P13&lt;&gt;"REVISAR",IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X13" s="7" t="n"/>
+      <c r="X13" s="26" t="inlineStr">
+        <is>
+          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y13" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z13" s="24" t="inlineStr">
@@ -3203,24 +3232,24 @@
         <v/>
       </c>
       <c r="AD13" s="24" t="n">
-        <v>1.065</v>
+        <v>3.71</v>
       </c>
       <c r="AE13" s="24" t="n">
         <v>2.6</v>
       </c>
       <c r="AF13" s="24" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="27" t="n"/>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>VI 08b</t>
+          <t>VI 08a</t>
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>4.87</v>
+        <v>3.65</v>
       </c>
       <c r="D14" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AE14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD14)</f>
@@ -3327,7 +3356,7 @@
       <c r="A15" s="27" t="n"/>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>VI 09</t>
+          <t>VI 08b</t>
         </is>
       </c>
       <c r="C15" s="22" t="n">
@@ -3378,15 +3407,11 @@
         <f>IF(NOT(ISNUMBER(I15)),"---",IF(I15&lt;=0,"---",IF(I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I15*100/(Datos!$B$8*AC15*K15^2*Datos!$B$5)))*AC15*K15*Datos!$B$5/Datos!$B$6,0.0033*J15*K15))))</f>
         <v/>
       </c>
-      <c r="Q15" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="R15" s="24" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+      <c r="Q15" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="24" t="n">
+        <v>12</v>
       </c>
       <c r="S15" s="25">
         <f>F15/(J15*0.85*K15)</f>
@@ -3409,7 +3434,7 @@
       <c r="X15" s="7" t="n"/>
       <c r="Y15" s="24" t="inlineStr">
         <is>
-          <t>Simplemente apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z15" s="24" t="inlineStr">
@@ -3429,7 +3454,7 @@
         <v/>
       </c>
       <c r="AD15" s="24" t="n">
-        <v>1.549</v>
+        <v>1.065</v>
       </c>
       <c r="AE15" s="24" t="n">
         <v>2.6</v>
@@ -3442,11 +3467,11 @@
       <c r="A16" s="27" t="n"/>
       <c r="B16" s="21" t="inlineStr">
         <is>
-          <t>VI 10a</t>
+          <t>VI 09</t>
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>2.55</v>
+        <v>4.87</v>
       </c>
       <c r="D16" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AE16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD16)</f>
@@ -3493,11 +3518,15 @@
         <f>IF(NOT(ISNUMBER(I16)),"---",IF(I16&lt;=0,"---",IF(I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I16*100/(Datos!$B$8*AC16*K16^2*Datos!$B$5)))*AC16*K16*Datos!$B$5/Datos!$B$6,0.0033*J16*K16))))</f>
         <v/>
       </c>
-      <c r="Q16" s="24" t="n">
-        <v>3</v>
-      </c>
-      <c r="R16" s="24" t="n">
-        <v>12</v>
+      <c r="Q16" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="R16" s="24" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
       </c>
       <c r="S16" s="25">
         <f>F16/(J16*0.85*K16)</f>
@@ -3520,7 +3549,7 @@
       <c r="X16" s="7" t="n"/>
       <c r="Y16" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Simplemente apoyada</t>
         </is>
       </c>
       <c r="Z16" s="24" t="inlineStr">
@@ -3540,7 +3569,7 @@
         <v/>
       </c>
       <c r="AD16" s="24" t="n">
-        <v>0</v>
+        <v>1.549</v>
       </c>
       <c r="AE16" s="24" t="n">
         <v>2.6</v>
@@ -3553,11 +3582,11 @@
       <c r="A17" s="27" t="n"/>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>VI 10b</t>
+          <t>VI 10a</t>
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>4</v>
+        <v>2.55</v>
       </c>
       <c r="D17" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AE17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD17)</f>
@@ -3651,7 +3680,7 @@
         <v/>
       </c>
       <c r="AD17" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE17" s="24" t="n">
         <v>2.6</v>
@@ -3664,11 +3693,11 @@
       <c r="A18" s="27" t="n"/>
       <c r="B18" s="21" t="inlineStr">
         <is>
-          <t>VI 10c</t>
+          <t>VI 10b</t>
         </is>
       </c>
       <c r="C18" s="22" t="n">
-        <v>3.6</v>
+        <v>4</v>
       </c>
       <c r="D18" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AE18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD18)</f>
@@ -3762,7 +3791,7 @@
         <v/>
       </c>
       <c r="AD18" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE18" s="24" t="n">
         <v>2.6</v>
@@ -3775,11 +3804,11 @@
       <c r="A19" s="27" t="n"/>
       <c r="B19" s="21" t="inlineStr">
         <is>
-          <t>VI 11a</t>
+          <t>VI 10c</t>
         </is>
       </c>
       <c r="C19" s="22" t="n">
-        <v>7.68</v>
+        <v>3.6</v>
       </c>
       <c r="D19" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AE19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD19)</f>
@@ -3817,20 +3846,20 @@
         <v/>
       </c>
       <c r="N19" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O19" s="24" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="P19" s="25">
         <f>IF(NOT(ISNUMBER(I19)),"---",IF(I19&lt;=0,"---",IF(I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I19*100/(Datos!$B$8*AC19*K19^2*Datos!$B$5)))*AC19*K19*Datos!$B$5/Datos!$B$6,0.0033*J19*K19))))</f>
         <v/>
       </c>
       <c r="Q19" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="R19" s="24" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="S19" s="25">
         <f>F19/(J19*0.85*K19)</f>
@@ -3844,20 +3873,16 @@
         <v>6</v>
       </c>
       <c r="V19" s="24" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="W19" s="7">
         <f>IF(OR(M19="REVISAR",P19="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M19&lt;&gt;"REVISAR",P19&lt;&gt;"REVISAR",IF(ISNUMBER(M19),N19*PI()*(O19/10)^2/4&gt;=M19,TRUE),IF(ISNUMBER(P19),Q19*PI()*(R19/10)^2/4&gt;=P19,TRUE),IF(ISNUMBER(M19),M19&lt;=0.0163*AB19*K19,TRUE),IF(ISNUMBER(P19),P19&lt;=0.0163*AC19*K19,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F19&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J19*K19+2*PI()*(U19/10)^2/4*Datos!$B$6*K19/V19)),"NO VERIF. CORTE",IF(NOT(L19&gt;=C19*100/VLOOKUP(Y19,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X19" s="26" t="inlineStr">
-        <is>
-          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X19" s="7" t="n"/>
       <c r="Y19" s="24" t="inlineStr">
         <is>
-          <t>Empotrada-apoyada</t>
+          <t>Continua</t>
         </is>
       </c>
       <c r="Z19" s="24" t="inlineStr">
@@ -3877,7 +3902,7 @@
         <v/>
       </c>
       <c r="AD19" s="24" t="n">
-        <v>1.825</v>
+        <v>0</v>
       </c>
       <c r="AE19" s="24" t="n">
         <v>2.6</v>
@@ -3890,11 +3915,11 @@
       <c r="A20" s="27" t="n"/>
       <c r="B20" s="21" t="inlineStr">
         <is>
-          <t>VI 11b</t>
+          <t>VI 11a</t>
         </is>
       </c>
       <c r="C20" s="22" t="n">
-        <v>3.45</v>
+        <v>7.68</v>
       </c>
       <c r="D20" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AE20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD20)</f>
@@ -3932,20 +3957,20 @@
         <v/>
       </c>
       <c r="N20" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O20" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P20" s="25">
         <f>IF(NOT(ISNUMBER(I20)),"---",IF(I20&lt;=0,"---",IF(I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I20*100/(Datos!$B$8*AC20*K20^2*Datos!$B$5)))*AC20*K20*Datos!$B$5/Datos!$B$6,0.0033*J20*K20))))</f>
         <v/>
       </c>
       <c r="Q20" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R20" s="24" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="S20" s="25">
         <f>F20/(J20*0.85*K20)</f>
@@ -3959,7 +3984,7 @@
         <v>6</v>
       </c>
       <c r="V20" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W20" s="7">
         <f>IF(OR(M20="REVISAR",P20="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M20&lt;&gt;"REVISAR",P20&lt;&gt;"REVISAR",IF(ISNUMBER(M20),N20*PI()*(O20/10)^2/4&gt;=M20,TRUE),IF(ISNUMBER(P20),Q20*PI()*(R20/10)^2/4&gt;=P20,TRUE),IF(ISNUMBER(M20),M20&lt;=0.0163*AB20*K20,TRUE),IF(ISNUMBER(P20),P20&lt;=0.0163*AC20*K20,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F20&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J20*K20+2*PI()*(U20/10)^2/4*Datos!$B$6*K20/V20)),"NO VERIF. CORTE",IF(NOT(L20&gt;=C20*100/VLOOKUP(Y20,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3967,12 +3992,12 @@
       </c>
       <c r="X20" s="26" t="inlineStr">
         <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>El plano rotula 'VI 111'; se interpreta 11a por el orden a-b-c. Sin apoyo intermedio, empotrada en tabiques. Apoya en columna COL 02 de 15x30 y en el tabique T08a. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y20" s="24" t="inlineStr">
         <is>
-          <t>Continua</t>
+          <t>Empotrada-apoyada</t>
         </is>
       </c>
       <c r="Z20" s="24" t="inlineStr">
@@ -3992,7 +4017,7 @@
         <v/>
       </c>
       <c r="AD20" s="24" t="n">
-        <v>0</v>
+        <v>1.825</v>
       </c>
       <c r="AE20" s="24" t="n">
         <v>2.6</v>
@@ -4005,11 +4030,11 @@
       <c r="A21" s="27" t="n"/>
       <c r="B21" s="21" t="inlineStr">
         <is>
-          <t>VI 11c</t>
+          <t>VI 11b</t>
         </is>
       </c>
       <c r="C21" s="22" t="n">
-        <v>5.02</v>
+        <v>3.45</v>
       </c>
       <c r="D21" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AE21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD21)</f>
@@ -4107,7 +4132,7 @@
         <v/>
       </c>
       <c r="AD21" s="24" t="n">
-        <v>1.549</v>
+        <v>0</v>
       </c>
       <c r="AE21" s="24" t="n">
         <v>2.6</v>
@@ -4120,11 +4145,11 @@
       <c r="A22" s="27" t="n"/>
       <c r="B22" s="21" t="inlineStr">
         <is>
-          <t>VCH 03a</t>
+          <t>VI 11c</t>
         </is>
       </c>
       <c r="C22" s="22" t="n">
-        <v>3.71</v>
+        <v>5.02</v>
       </c>
       <c r="D22" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AE22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD22)</f>
@@ -4148,21 +4173,21 @@
         <v/>
       </c>
       <c r="J22" s="24" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="K22" s="7">
         <f>L22-AF22</f>
         <v/>
       </c>
       <c r="L22" s="24" t="n">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="M22" s="25">
         <f>IF(NOT(ISNUMBER(H22)),"---",IF(H22&lt;=0,"---",IF(H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H22*100/(Datos!$B$8*AB22*K22^2*Datos!$B$5)))*AB22*K22*Datos!$B$5/Datos!$B$6,0.0033*J22*K22))))</f>
         <v/>
       </c>
       <c r="N22" s="24" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="O22" s="24" t="n">
         <v>12</v>
@@ -4172,10 +4197,10 @@
         <v/>
       </c>
       <c r="Q22" s="24" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="R22" s="24" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="S22" s="25">
         <f>F22/(J22*0.85*K22)</f>
@@ -4186,10 +4211,10 @@
         <v/>
       </c>
       <c r="U22" s="24" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="V22" s="24" t="n">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="W22" s="7">
         <f>IF(OR(M22="REVISAR",P22="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M22&lt;&gt;"REVISAR",P22&lt;&gt;"REVISAR",IF(ISNUMBER(M22),N22*PI()*(O22/10)^2/4&gt;=M22,TRUE),IF(ISNUMBER(P22),Q22*PI()*(R22/10)^2/4&gt;=P22,TRUE),IF(ISNUMBER(M22),M22&lt;=0.0163*AB22*K22,TRUE),IF(ISNUMBER(P22),P22&lt;=0.0163*AC22*K22,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F22&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J22*K22+2*PI()*(U22/10)^2/4*Datos!$B$6*K22/V22)),"NO VERIF. CORTE",IF(NOT(L22&gt;=C22*100/VLOOKUP(Y22,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4197,7 +4222,7 @@
       </c>
       <c r="X22" s="26" t="inlineStr">
         <is>
-          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y22" s="24" t="inlineStr">
@@ -4207,7 +4232,7 @@
       </c>
       <c r="Z22" s="24" t="inlineStr">
         <is>
-          <t>Colgante</t>
+          <t>Invertida</t>
         </is>
       </c>
       <c r="AA22" s="24" t="n">
@@ -4222,7 +4247,7 @@
         <v/>
       </c>
       <c r="AD22" s="24" t="n">
-        <v>2.1</v>
+        <v>1.549</v>
       </c>
       <c r="AE22" s="24" t="n">
         <v>2.6</v>
@@ -4235,11 +4260,11 @@
       <c r="A23" s="27" t="n"/>
       <c r="B23" s="21" t="inlineStr">
         <is>
-          <t>VCH 03b</t>
+          <t>VCH 03a</t>
         </is>
       </c>
       <c r="C23" s="22" t="n">
-        <v>2.13</v>
+        <v>3.71</v>
       </c>
       <c r="D23" s="23">
         <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AE23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD23)</f>
@@ -4277,20 +4302,20 @@
         <v/>
       </c>
       <c r="N23" s="24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="O23" s="24" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="P23" s="25">
         <f>IF(NOT(ISNUMBER(I23)),"---",IF(I23&lt;=0,"---",IF(I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I23*100/(Datos!$B$8*AC23*K23^2*Datos!$B$5)))*AC23*K23*Datos!$B$5/Datos!$B$6,0.0033*J23*K23))))</f>
         <v/>
       </c>
       <c r="Q23" s="24" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="R23" s="24" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="S23" s="25">
         <f>F23/(J23*0.85*K23)</f>
@@ -4312,7 +4337,7 @@
       </c>
       <c r="X23" s="26" t="inlineStr">
         <is>
-          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+          <t>Excede cuantia maxima y no llega a la altura minima por flecha. Revisar el ancho tributario real. Separacion de estribos menor a 10 cm: revisar constructividad.</t>
         </is>
       </c>
       <c r="Y23" s="24" t="inlineStr">
@@ -4347,247 +4372,251 @@
       </c>
     </row>
     <row r="24" ht="46" customHeight="1">
-      <c r="A24" s="28" t="n"/>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="A24" s="27" t="n"/>
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t>VCH 03b</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="D24" s="23">
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="23">
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
+        <v/>
+      </c>
+      <c r="G24" s="23">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="H24" s="23">
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
+        <v/>
+      </c>
+      <c r="I24" s="23">
+        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
+        <v/>
+      </c>
+      <c r="J24" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="K24" s="7">
+        <f>L24-AF24</f>
+        <v/>
+      </c>
+      <c r="L24" s="24" t="n">
+        <v>13</v>
+      </c>
+      <c r="M24" s="25">
+        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <v/>
+      </c>
+      <c r="N24" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="O24" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="P24" s="25">
+        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
+        <v/>
+      </c>
+      <c r="Q24" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="R24" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="S24" s="25">
+        <f>F24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="T24" s="25">
+        <f>G24/(J24*0.85*K24)</f>
+        <v/>
+      </c>
+      <c r="U24" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="V24" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="W24" s="7">
+        <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X24" s="26" t="inlineStr">
+        <is>
+          <t>Separacion de estribos menor a 10 cm: revisar constructividad.</t>
+        </is>
+      </c>
+      <c r="Y24" s="24" t="inlineStr">
+        <is>
+          <t>Continua</t>
+        </is>
+      </c>
+      <c r="Z24" s="24" t="inlineStr">
+        <is>
+          <t>Colgante</t>
+        </is>
+      </c>
+      <c r="AA24" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB24" s="7">
+        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AC24" s="7">
+        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
+        <v/>
+      </c>
+      <c r="AD24" s="24" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="AE24" s="24" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="AF24" s="24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="28" t="n"/>
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>VCH 05</t>
         </is>
       </c>
-      <c r="C24" s="30" t="n">
+      <c r="C25" s="30" t="n">
         <v>3.71</v>
       </c>
-      <c r="D24" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
-        <v/>
-      </c>
-      <c r="E24" s="32" t="n"/>
-      <c r="F24" s="31">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
-        <v/>
-      </c>
-      <c r="G24" s="31">
-        <f>F24</f>
-        <v/>
-      </c>
-      <c r="H24" s="31">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
-        <v/>
-      </c>
-      <c r="I24" s="31">
-        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
-        <v/>
-      </c>
-      <c r="J24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="K24" s="32">
-        <f>L24-AF24</f>
-        <v/>
-      </c>
-      <c r="L24" s="33" t="n">
+      <c r="D25" s="31">
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="32" t="n"/>
+      <c r="F25" s="31">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
+        <v/>
+      </c>
+      <c r="G25" s="31">
+        <f>F25</f>
+        <v/>
+      </c>
+      <c r="H25" s="31">
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
+        <v/>
+      </c>
+      <c r="I25" s="31">
+        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
+        <v/>
+      </c>
+      <c r="J25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="K25" s="32">
+        <f>L25-AF25</f>
+        <v/>
+      </c>
+      <c r="L25" s="33" t="n">
         <v>45</v>
       </c>
-      <c r="M24" s="34">
-        <f>IF(NOT(ISNUMBER(H24)),"---",IF(H24&lt;=0,"---",IF(H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H24*100/(Datos!$B$8*AB24*K24^2*Datos!$B$5)))*AB24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
-        <v/>
-      </c>
-      <c r="N24" s="33" t="n">
+      <c r="M25" s="34">
+        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="N25" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="O24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P24" s="34">
-        <f>IF(NOT(ISNUMBER(I24)),"---",IF(I24&lt;=0,"---",IF(I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I24*100/(Datos!$B$8*AC24*K24^2*Datos!$B$5)))*AC24*K24*Datos!$B$5/Datos!$B$6,0.0033*J24*K24))))</f>
-        <v/>
-      </c>
-      <c r="Q24" s="33" t="inlineStr">
+      <c r="O25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P25" s="34">
+        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
+        <v/>
+      </c>
+      <c r="Q25" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R24" s="33" t="inlineStr">
+      <c r="R25" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="S24" s="34">
-        <f>F24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="T24" s="34">
-        <f>G24/(J24*0.85*K24)</f>
-        <v/>
-      </c>
-      <c r="U24" s="33" t="n">
+      <c r="S25" s="34">
+        <f>F25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="T25" s="34">
+        <f>G25/(J25*0.85*K25)</f>
+        <v/>
+      </c>
+      <c r="U25" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="V24" s="33" t="n">
+      <c r="V25" s="33" t="n">
         <v>20</v>
       </c>
-      <c r="W24" s="32">
-        <f>IF(OR(M24="REVISAR",P24="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M24&lt;&gt;"REVISAR",P24&lt;&gt;"REVISAR",IF(ISNUMBER(M24),N24*PI()*(O24/10)^2/4&gt;=M24,TRUE),IF(ISNUMBER(P24),Q24*PI()*(R24/10)^2/4&gt;=P24,TRUE),IF(ISNUMBER(M24),M24&lt;=0.0163*AB24*K24,TRUE),IF(ISNUMBER(P24),P24&lt;=0.0163*AC24*K24,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F24&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J24*K24+2*PI()*(U24/10)^2/4*Datos!$B$6*K24/V24)),"NO VERIF. CORTE",IF(NOT(L24&gt;=C24*100/VLOOKUP(Y24,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X24" s="32" t="n"/>
-      <c r="Y24" s="33" t="inlineStr">
+      <c r="W25" s="32">
+        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X25" s="32" t="n"/>
+      <c r="Y25" s="33" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z24" s="33" t="inlineStr">
+      <c r="Z25" s="33" t="inlineStr">
         <is>
           <t>Colgante</t>
         </is>
       </c>
-      <c r="AA24" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB24" s="32">
-        <f>IF(Z24="Colgante",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AC24" s="32">
-        <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
-        <v/>
-      </c>
-      <c r="AD24" s="33" t="n">
+      <c r="AA25" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB25" s="32">
+        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AC25" s="32">
+        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
+        <v/>
+      </c>
+      <c r="AD25" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE24" s="33" t="n">
+      <c r="AE25" s="33" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF24" s="33" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" ht="46" customHeight="1">
-      <c r="A25" s="20" t="inlineStr">
+      <c r="AF25" s="33" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" ht="46" customHeight="1">
+      <c r="A26" s="20" t="inlineStr">
         <is>
           <t>TECHO</t>
         </is>
       </c>
-      <c r="B25" s="21" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>VI 12</t>
         </is>
       </c>
-      <c r="C25" s="22" t="n">
+      <c r="C26" s="22" t="n">
         <v>9.9</v>
       </c>
-      <c r="D25" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD25)</f>
-        <v/>
-      </c>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="23">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
-        <v/>
-      </c>
-      <c r="G25" s="23">
-        <f>F25</f>
-        <v/>
-      </c>
-      <c r="H25" s="23">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
-        <v/>
-      </c>
-      <c r="I25" s="23">
-        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
-        <v/>
-      </c>
-      <c r="J25" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="K25" s="7">
-        <f>L25-AF25</f>
-        <v/>
-      </c>
-      <c r="L25" s="24" t="n">
-        <v>70</v>
-      </c>
-      <c r="M25" s="25">
-        <f>IF(NOT(ISNUMBER(H25)),"---",IF(H25&lt;=0,"---",IF(H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H25*100/(Datos!$B$8*AB25*K25^2*Datos!$B$5)))*AB25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="N25" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="O25" s="24" t="n">
-        <v>25</v>
-      </c>
-      <c r="P25" s="25">
-        <f>IF(NOT(ISNUMBER(I25)),"---",IF(I25&lt;=0,"---",IF(I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I25*100/(Datos!$B$8*AC25*K25^2*Datos!$B$5)))*AC25*K25*Datos!$B$5/Datos!$B$6,0.0033*J25*K25))))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="R25" s="24" t="n">
-        <v>25</v>
-      </c>
-      <c r="S25" s="25">
-        <f>F25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="T25" s="25">
-        <f>G25/(J25*0.85*K25)</f>
-        <v/>
-      </c>
-      <c r="U25" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="V25" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="W25" s="7">
-        <f>IF(OR(M25="REVISAR",P25="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M25&lt;&gt;"REVISAR",P25&lt;&gt;"REVISAR",IF(ISNUMBER(M25),N25*PI()*(O25/10)^2/4&gt;=M25,TRUE),IF(ISNUMBER(P25),Q25*PI()*(R25/10)^2/4&gt;=P25,TRUE),IF(ISNUMBER(M25),M25&lt;=0.0163*AB25*K25,TRUE),IF(ISNUMBER(P25),P25&lt;=0.0163*AC25*K25,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F25&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J25*K25+2*PI()*(U25/10)^2/4*Datos!$B$6*K25/V25)),"NO VERIF. CORTE",IF(NOT(L25&gt;=C25*100/VLOOKUP(Y25,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X25" s="7" t="n"/>
-      <c r="Y25" s="24" t="inlineStr">
-        <is>
-          <t>Continua</t>
-        </is>
-      </c>
-      <c r="Z25" s="24" t="inlineStr">
-        <is>
-          <t>Invertida</t>
-        </is>
-      </c>
-      <c r="AA25" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB25" s="7">
-        <f>IF(Z25="Colgante",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AC25" s="7">
-        <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
-        <v/>
-      </c>
-      <c r="AD25" s="24" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="AE25" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF25" s="24" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" ht="46" customHeight="1">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="21" t="inlineStr">
-        <is>
-          <t>VI 13a</t>
-        </is>
-      </c>
-      <c r="C26" s="22" t="n">
-        <v>6</v>
-      </c>
       <c r="D26" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD26)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD26)</f>
         <v/>
       </c>
       <c r="E26" s="7" t="n"/>
@@ -4625,7 +4654,7 @@
         <v>2</v>
       </c>
       <c r="O26" s="24" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="P26" s="25">
         <f>IF(NOT(ISNUMBER(I26)),"---",IF(I26&lt;=0,"---",IF(I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I26*100/(Datos!$B$8*AC26*K26^2*Datos!$B$5)))*AC26*K26*Datos!$B$5/Datos!$B$6,0.0033*J26*K26))))</f>
@@ -4635,7 +4664,7 @@
         <v>2</v>
       </c>
       <c r="R26" s="24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="S26" s="25">
         <f>F26/(J26*0.85*K26)</f>
@@ -4678,7 +4707,7 @@
         <v/>
       </c>
       <c r="AD26" s="24" t="n">
-        <v>3.799</v>
+        <v>2.1</v>
       </c>
       <c r="AE26" s="24" t="n">
         <v>1</v>
@@ -4691,14 +4720,14 @@
       <c r="A27" s="27" t="n"/>
       <c r="B27" s="21" t="inlineStr">
         <is>
-          <t>VI 13b</t>
+          <t>VI 13a</t>
         </is>
       </c>
       <c r="C27" s="22" t="n">
-        <v>3.75</v>
+        <v>6</v>
       </c>
       <c r="D27" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD27)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD27)</f>
         <v/>
       </c>
       <c r="E27" s="7" t="n"/>
@@ -4733,20 +4762,20 @@
         <v/>
       </c>
       <c r="N27" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O27" s="24" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="P27" s="25">
         <f>IF(NOT(ISNUMBER(I27)),"---",IF(I27&lt;=0,"---",IF(I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I27*100/(Datos!$B$8*AC27*K27^2*Datos!$B$5)))*AC27*K27*Datos!$B$5/Datos!$B$6,0.0033*J27*K27))))</f>
         <v/>
       </c>
       <c r="Q27" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R27" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="S27" s="25">
         <f>F27/(J27*0.85*K27)</f>
@@ -4760,7 +4789,7 @@
         <v>6</v>
       </c>
       <c r="V27" s="24" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="W27" s="7">
         <f>IF(OR(M27="REVISAR",P27="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M27&lt;&gt;"REVISAR",P27&lt;&gt;"REVISAR",IF(ISNUMBER(M27),N27*PI()*(O27/10)^2/4&gt;=M27,TRUE),IF(ISNUMBER(P27),Q27*PI()*(R27/10)^2/4&gt;=P27,TRUE),IF(ISNUMBER(M27),M27&lt;=0.0163*AB27*K27,TRUE),IF(ISNUMBER(P27),P27&lt;=0.0163*AC27*K27,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F27&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J27*K27+2*PI()*(U27/10)^2/4*Datos!$B$6*K27/V27)),"NO VERIF. CORTE",IF(NOT(L27&gt;=C27*100/VLOOKUP(Y27,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -4789,7 +4818,7 @@
         <v/>
       </c>
       <c r="AD27" s="24" t="n">
-        <v>2.1</v>
+        <v>3.799</v>
       </c>
       <c r="AE27" s="24" t="n">
         <v>1</v>
@@ -4802,14 +4831,14 @@
       <c r="A28" s="27" t="n"/>
       <c r="B28" s="21" t="inlineStr">
         <is>
-          <t>VI 14</t>
+          <t>VI 13b</t>
         </is>
       </c>
       <c r="C28" s="22" t="n">
-        <v>6</v>
+        <v>3.75</v>
       </c>
       <c r="D28" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD28)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD28)</f>
         <v/>
       </c>
       <c r="E28" s="7" t="n"/>
@@ -4900,7 +4929,7 @@
         <v/>
       </c>
       <c r="AD28" s="24" t="n">
-        <v>1.699</v>
+        <v>2.1</v>
       </c>
       <c r="AE28" s="24" t="n">
         <v>1</v>
@@ -4913,14 +4942,14 @@
       <c r="A29" s="27" t="n"/>
       <c r="B29" s="21" t="inlineStr">
         <is>
-          <t>VI 15a</t>
+          <t>VI 14</t>
         </is>
       </c>
       <c r="C29" s="22" t="n">
-        <v>4.03</v>
+        <v>6</v>
       </c>
       <c r="D29" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD29)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD29)</f>
         <v/>
       </c>
       <c r="E29" s="7" t="n"/>
@@ -4988,11 +5017,7 @@
         <f>IF(OR(M29="REVISAR",P29="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M29&lt;&gt;"REVISAR",P29&lt;&gt;"REVISAR",IF(ISNUMBER(M29),N29*PI()*(O29/10)^2/4&gt;=M29,TRUE),IF(ISNUMBER(P29),Q29*PI()*(R29/10)^2/4&gt;=P29,TRUE),IF(ISNUMBER(M29),M29&lt;=0.0163*AB29*K29,TRUE),IF(ISNUMBER(P29),P29&lt;=0.0163*AC29*K29,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F29&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J29*K29+2*PI()*(U29/10)^2/4*Datos!$B$6*K29/V29)),"NO VERIF. CORTE",IF(NOT(L29&gt;=C29*100/VLOOKUP(Y29,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X29" s="26" t="inlineStr">
-        <is>
-          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
-        </is>
-      </c>
+      <c r="X29" s="7" t="n"/>
       <c r="Y29" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5015,7 +5040,7 @@
         <v/>
       </c>
       <c r="AD29" s="24" t="n">
-        <v>0</v>
+        <v>1.699</v>
       </c>
       <c r="AE29" s="24" t="n">
         <v>1</v>
@@ -5028,14 +5053,14 @@
       <c r="A30" s="27" t="n"/>
       <c r="B30" s="21" t="inlineStr">
         <is>
-          <t>VI 15b</t>
+          <t>VI 15a</t>
         </is>
       </c>
       <c r="C30" s="22" t="n">
-        <v>4.85</v>
+        <v>4.03</v>
       </c>
       <c r="D30" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD30)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD30)</f>
         <v/>
       </c>
       <c r="E30" s="7" t="n"/>
@@ -5130,7 +5155,7 @@
         <v/>
       </c>
       <c r="AD30" s="24" t="n">
-        <v>1.699</v>
+        <v>0</v>
       </c>
       <c r="AE30" s="24" t="n">
         <v>1</v>
@@ -5143,14 +5168,14 @@
       <c r="A31" s="27" t="n"/>
       <c r="B31" s="21" t="inlineStr">
         <is>
-          <t>VI 16a</t>
+          <t>VI 15b</t>
         </is>
       </c>
       <c r="C31" s="22" t="n">
-        <v>3.58</v>
+        <v>4.85</v>
       </c>
       <c r="D31" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD31)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD31)</f>
         <v/>
       </c>
       <c r="E31" s="7" t="n"/>
@@ -5218,7 +5243,11 @@
         <f>IF(OR(M31="REVISAR",P31="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M31&lt;&gt;"REVISAR",P31&lt;&gt;"REVISAR",IF(ISNUMBER(M31),N31*PI()*(O31/10)^2/4&gt;=M31,TRUE),IF(ISNUMBER(P31),Q31*PI()*(R31/10)^2/4&gt;=P31,TRUE),IF(ISNUMBER(M31),M31&lt;=0.0163*AB31*K31,TRUE),IF(ISNUMBER(P31),P31&lt;=0.0163*AC31*K31,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F31&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J31*K31+2*PI()*(U31/10)^2/4*Datos!$B$6*K31/V31)),"NO VERIF. CORTE",IF(NOT(L31&gt;=C31*100/VLOOKUP(Y31,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X31" s="7" t="n"/>
+      <c r="X31" s="26" t="inlineStr">
+        <is>
+          <t>Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+        </is>
+      </c>
       <c r="Y31" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -5254,14 +5283,14 @@
       <c r="A32" s="27" t="n"/>
       <c r="B32" s="21" t="inlineStr">
         <is>
-          <t>VI 16b</t>
+          <t>VI 16a</t>
         </is>
       </c>
       <c r="C32" s="22" t="n">
-        <v>1.12</v>
+        <v>3.58</v>
       </c>
       <c r="D32" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD32)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD32)</f>
         <v/>
       </c>
       <c r="E32" s="7" t="n"/>
@@ -5362,130 +5391,241 @@
       </c>
     </row>
     <row r="33" ht="46" customHeight="1">
-      <c r="A33" s="28" t="n"/>
-      <c r="B33" s="29" t="inlineStr">
+      <c r="A33" s="27" t="n"/>
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>VI 16b</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="n">
+        <v>1.12</v>
+      </c>
+      <c r="D33" s="23">
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD33)</f>
+        <v/>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="23">
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
+        <v/>
+      </c>
+      <c r="G33" s="23">
+        <f>F33</f>
+        <v/>
+      </c>
+      <c r="H33" s="23">
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
+        <v/>
+      </c>
+      <c r="I33" s="23">
+        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
+        <v/>
+      </c>
+      <c r="J33" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="K33" s="7">
+        <f>L33-AF33</f>
+        <v/>
+      </c>
+      <c r="L33" s="24" t="n">
+        <v>70</v>
+      </c>
+      <c r="M33" s="25">
+        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <v/>
+      </c>
+      <c r="N33" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="O33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="P33" s="25">
+        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
+        <v/>
+      </c>
+      <c r="Q33" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="R33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="S33" s="25">
+        <f>F33/(J33*0.85*K33)</f>
+        <v/>
+      </c>
+      <c r="T33" s="25">
+        <f>G33/(J33*0.85*K33)</f>
+        <v/>
+      </c>
+      <c r="U33" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="V33" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="W33" s="7">
+        <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X33" s="7" t="n"/>
+      <c r="Y33" s="24" t="inlineStr">
+        <is>
+          <t>Continua</t>
+        </is>
+      </c>
+      <c r="Z33" s="24" t="inlineStr">
+        <is>
+          <t>Invertida</t>
+        </is>
+      </c>
+      <c r="AA33" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB33" s="7">
+        <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AC33" s="7">
+        <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
+        <v/>
+      </c>
+      <c r="AD33" s="24" t="n">
+        <v>1.699</v>
+      </c>
+      <c r="AE33" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF33" s="24" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" ht="46" customHeight="1">
+      <c r="A34" s="28" t="n"/>
+      <c r="B34" s="29" t="inlineStr">
         <is>
           <t>VI 17</t>
         </is>
       </c>
-      <c r="C33" s="30" t="n">
+      <c r="C34" s="30" t="n">
         <v>4.35</v>
       </c>
-      <c r="D33" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$25,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$25,Datos!$A$14:$E$15,3,0)*AD33)</f>
-        <v/>
-      </c>
-      <c r="E33" s="32" t="n"/>
-      <c r="F33" s="31">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
-        <v/>
-      </c>
-      <c r="G33" s="31">
-        <f>F33</f>
-        <v/>
-      </c>
-      <c r="H33" s="31">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
-        <v/>
-      </c>
-      <c r="I33" s="31">
-        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
-        <v/>
-      </c>
-      <c r="J33" s="33" t="n">
+      <c r="D34" s="31">
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD34+Datos!$B$7*J34*L34/10000+Datos!$B$16*AE34)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD34)</f>
+        <v/>
+      </c>
+      <c r="E34" s="32" t="n"/>
+      <c r="F34" s="31">
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,4,0)*D34*C34</f>
+        <v/>
+      </c>
+      <c r="G34" s="31">
+        <f>F34</f>
+        <v/>
+      </c>
+      <c r="H34" s="31">
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,2,0)*D34*C34^2</f>
+        <v/>
+      </c>
+      <c r="I34" s="31">
+        <f>IF(VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)*D34*C34^2)</f>
+        <v/>
+      </c>
+      <c r="J34" s="33" t="n">
         <v>15</v>
       </c>
-      <c r="K33" s="32">
-        <f>L33-AF33</f>
-        <v/>
-      </c>
-      <c r="L33" s="33" t="n">
+      <c r="K34" s="32">
+        <f>L34-AF34</f>
+        <v/>
+      </c>
+      <c r="L34" s="33" t="n">
         <v>70</v>
       </c>
-      <c r="M33" s="34">
-        <f>IF(NOT(ISNUMBER(H33)),"---",IF(H33&lt;=0,"---",IF(H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H33*100/(Datos!$B$8*AB33*K33^2*Datos!$B$5)))*AB33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
-        <v/>
-      </c>
-      <c r="N33" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="O33" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="P33" s="34">
-        <f>IF(NOT(ISNUMBER(I33)),"---",IF(I33&lt;=0,"---",IF(I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I33*100/(Datos!$B$8*AC33*K33^2*Datos!$B$5)))*AC33*K33*Datos!$B$5/Datos!$B$6,0.0033*J33*K33))))</f>
-        <v/>
-      </c>
-      <c r="Q33" s="33" t="inlineStr">
+      <c r="M34" s="34">
+        <f>IF(NOT(ISNUMBER(H34)),"---",IF(H34&lt;=0,"---",IF(H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*H34*100/(Datos!$B$8*AB34*K34^2*Datos!$B$5)))*AB34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
+        <v/>
+      </c>
+      <c r="N34" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="O34" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="P34" s="34">
+        <f>IF(NOT(ISNUMBER(I34)),"---",IF(I34&lt;=0,"---",IF(I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I34*100/(Datos!$B$8*AC34*K34^2*Datos!$B$5)))*AC34*K34*Datos!$B$5/Datos!$B$6,0.0033*J34*K34))))</f>
+        <v/>
+      </c>
+      <c r="Q34" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="R33" s="33" t="inlineStr">
+      <c r="R34" s="33" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="S33" s="34">
-        <f>F33/(J33*0.85*K33)</f>
-        <v/>
-      </c>
-      <c r="T33" s="34">
-        <f>G33/(J33*0.85*K33)</f>
-        <v/>
-      </c>
-      <c r="U33" s="33" t="n">
+      <c r="S34" s="34">
+        <f>F34/(J34*0.85*K34)</f>
+        <v/>
+      </c>
+      <c r="T34" s="34">
+        <f>G34/(J34*0.85*K34)</f>
+        <v/>
+      </c>
+      <c r="U34" s="33" t="n">
         <v>6</v>
       </c>
-      <c r="V33" s="33" t="n">
+      <c r="V34" s="33" t="n">
         <v>30</v>
       </c>
-      <c r="W33" s="32">
-        <f>IF(OR(M33="REVISAR",P33="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M33&lt;&gt;"REVISAR",P33&lt;&gt;"REVISAR",IF(ISNUMBER(M33),N33*PI()*(O33/10)^2/4&gt;=M33,TRUE),IF(ISNUMBER(P33),Q33*PI()*(R33/10)^2/4&gt;=P33,TRUE),IF(ISNUMBER(M33),M33&lt;=0.0163*AB33*K33,TRUE),IF(ISNUMBER(P33),P33&lt;=0.0163*AC33*K33,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F33&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J33*K33+2*PI()*(U33/10)^2/4*Datos!$B$6*K33/V33)),"NO VERIF. CORTE",IF(NOT(L33&gt;=C33*100/VLOOKUP(Y33,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
-        <v/>
-      </c>
-      <c r="X33" s="32" t="n"/>
-      <c r="Y33" s="33" t="inlineStr">
+      <c r="W34" s="32">
+        <f>IF(OR(M34="REVISAR",P34="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M34&lt;&gt;"REVISAR",P34&lt;&gt;"REVISAR",IF(ISNUMBER(M34),N34*PI()*(O34/10)^2/4&gt;=M34,TRUE),IF(ISNUMBER(P34),Q34*PI()*(R34/10)^2/4&gt;=P34,TRUE),IF(ISNUMBER(M34),M34&lt;=0.0163*AB34*K34,TRUE),IF(ISNUMBER(P34),P34&lt;=0.0163*AC34*K34,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F34&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J34*K34+2*PI()*(U34/10)^2/4*Datos!$B$6*K34/V34)),"NO VERIF. CORTE",IF(NOT(L34&gt;=C34*100/VLOOKUP(Y34,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
+        <v/>
+      </c>
+      <c r="X34" s="32" t="n"/>
+      <c r="Y34" s="33" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>
         </is>
       </c>
-      <c r="Z33" s="33" t="inlineStr">
+      <c r="Z34" s="33" t="inlineStr">
         <is>
           <t>Invertida</t>
         </is>
       </c>
-      <c r="AA33" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="AB33" s="32">
-        <f>IF(Z33="Colgante",MIN(C33*100/4,J33+16*AA33),J33)</f>
-        <v/>
-      </c>
-      <c r="AC33" s="32">
-        <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
-        <v/>
-      </c>
-      <c r="AD33" s="33" t="n">
+      <c r="AA34" s="33" t="n">
+        <v>12</v>
+      </c>
+      <c r="AB34" s="32">
+        <f>IF(Z34="Colgante",MIN(C34*100/4,J34+16*AA34),J34)</f>
+        <v/>
+      </c>
+      <c r="AC34" s="32">
+        <f>IF(Z34="Invertida",MIN(C34*100/4,J34+16*AA34),J34)</f>
+        <v/>
+      </c>
+      <c r="AD34" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE33" s="33" t="n">
+      <c r="AE34" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="AF33" s="33" t="n">
+      <c r="AF34" s="33" t="n">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
     <mergeCell ref="F2:G2"/>
-    <mergeCell ref="A4:A24"/>
     <mergeCell ref="J2:L2"/>
+    <mergeCell ref="A4:A25"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A25:A33"/>
     <mergeCell ref="A1:AF1"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="S2:U2"/>
+    <mergeCell ref="A26:A34"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="V2"/>
     <mergeCell ref="B2:B3"/>
@@ -5497,7 +5637,7 @@
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="W2:W3"/>
   </mergeCells>
-  <conditionalFormatting sqref="W4:W33">
+  <conditionalFormatting sqref="W4:W34">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"VERIFICA"</formula>
     </cfRule>
@@ -5512,13 +5652,13 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="Y4:Y33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Y4:Y34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Datos!$A$19:$A$23</formula1>
     </dataValidation>
-    <dataValidation sqref="Z4:Z33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="Z4:Z34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Invertida,Colgante"</formula1>
     </dataValidation>
-    <dataValidation sqref="O4:O33 R4:R33 U4:U33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="O4:O34 R4:R34 U4:U34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"6,8,10,12,16,20,25"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5534,7 +5674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B70"/>
+  <dimension ref="A1:B71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -5857,7 +5997,7 @@
       <c r="A37" s="36" t="inlineStr"/>
       <c r="B37" s="37" t="inlineStr">
         <is>
-          <t>NOTA: el computo metrico lista una VI 06 de 15x70x14,00 que no existe en obra;</t>
+          <t>VI 06 mide 14,00 m en total y es el cuarto borde de L07. Sobre su eje hay cuatro</t>
         </is>
       </c>
     </row>
@@ -5865,7 +6005,7 @@
       <c r="A38" s="36" t="inlineStr"/>
       <c r="B38" s="37" t="inlineStr">
         <is>
-          <t>por eso no figura en esta planilla. La cuarta cara de L07 apoya en otro elemento.</t>
+          <t>columnas, de modo que trabaja como viga continua de tres tramos de 4,10, 4,32 y</t>
         </is>
       </c>
     </row>
@@ -5873,7 +6013,7 @@
       <c r="A39" s="36" t="inlineStr"/>
       <c r="B39" s="37" t="inlineStr">
         <is>
-          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
+          <t>6,53 m. Se calcula con el mayor, 6,53 m, que es el que gobierna.</t>
         </is>
       </c>
     </row>
@@ -5881,7 +6021,7 @@
       <c r="A40" s="36" t="inlineStr"/>
       <c r="B40" s="37" t="inlineStr">
         <is>
-          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
+          <t>hormigon visto: una viga colgante quedaria a la vista. El computo metrico las</t>
         </is>
       </c>
     </row>
@@ -5889,7 +6029,7 @@
       <c r="A41" s="36" t="inlineStr"/>
       <c r="B41" s="37" t="inlineStr">
         <is>
-          <t>Esto define donde la losa aporta ala comprimida:</t>
+          <t>agrupa a las 28 bajo el rubro Vigas invertidas 15x70.</t>
         </is>
       </c>
     </row>
@@ -5897,7 +6037,7 @@
       <c r="A42" s="36" t="inlineStr"/>
       <c r="B42" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
+          <t>Esto define donde la losa aporta ala comprimida:</t>
         </is>
       </c>
     </row>
@@ -5905,7 +6045,7 @@
       <c r="A43" s="36" t="inlineStr"/>
       <c r="B43" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
+          <t xml:space="preserve">  viga COLGANTE  -&gt; la losa esta arriba  -&gt; ala util en el TRAMO (momento positivo)</t>
         </is>
       </c>
     </row>
@@ -5913,7 +6053,7 @@
       <c r="A44" s="36" t="inlineStr"/>
       <c r="B44" s="37" t="inlineStr">
         <is>
-          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
+          <t xml:space="preserve">  viga INVERTIDA -&gt; la losa esta abajo   -&gt; ala util en el APOYO (momento negativo)</t>
         </is>
       </c>
     </row>
@@ -5921,7 +6061,7 @@
       <c r="A45" s="36" t="inlineStr"/>
       <c r="B45" s="37" t="inlineStr">
         <is>
-          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
+          <t>En la zona con ala se adopta b efectivo = min(L/4 ; b + 16 hf); en la otra, la</t>
         </is>
       </c>
     </row>
@@ -5929,7 +6069,7 @@
       <c r="A46" s="36" t="inlineStr"/>
       <c r="B46" s="37" t="inlineStr">
         <is>
-          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
+          <t>seccion es rectangular de ancho b. Las columnas b ef tramo y b ef apoyo lo muestran.</t>
         </is>
       </c>
     </row>
@@ -5937,7 +6077,7 @@
       <c r="A47" s="36" t="inlineStr"/>
       <c r="B47" s="37" t="inlineStr">
         <is>
-          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
+          <t>PENDIENTE: las invertidas de BORDE (VI 01a, 01b, 07a, 07b, 07c, 11a, 11b, 11c,</t>
         </is>
       </c>
     </row>
@@ -5945,31 +6085,31 @@
       <c r="A48" s="36" t="inlineStr"/>
       <c r="B48" s="37" t="inlineStr">
         <is>
-          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
+          <t>15a y 15b) reciben la reaccion de la losa de un solo lado, excentrica respecto</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="36" t="inlineStr"/>
-      <c r="B49" s="37" t="inlineStr"/>
+      <c r="B49" s="37" t="inlineStr">
+        <is>
+          <t>de su eje, y quedan sometidas a TORSION. Esta planilla no la verifica.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="36" t="inlineStr">
+      <c r="A50" s="36" t="inlineStr"/>
+      <c r="B50" s="37" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="36" t="inlineStr">
         <is>
           <t>7. RESULTADO</t>
         </is>
       </c>
-      <c r="B50" s="36" t="inlineStr">
+      <c r="B51" s="36" t="inlineStr">
         <is>
           <t>30 vigas: 21 del entrepiso PA y 9 de la losa de techo. 28 verifican.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="36" t="inlineStr"/>
-      <c r="B51" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
@@ -5977,7 +6117,7 @@
       <c r="A52" s="36" t="inlineStr"/>
       <c r="B52" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
+          <t>VI 02 (15x60, 9,88 m): recibe L02 y L03, B = 2,88 m. La armadura de apoyo</t>
         </is>
       </c>
     </row>
@@ -5985,7 +6125,7 @@
       <c r="A53" s="36" t="inlineStr"/>
       <c r="B53" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
+          <t xml:space="preserve">   necesaria ronda los 25 cm2 y supera la cuantia maxima. Los apoyos estan</t>
         </is>
       </c>
     </row>
@@ -5993,7 +6133,7 @@
       <c r="A54" s="36" t="inlineStr"/>
       <c r="B54" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
+          <t xml:space="preserve">   confirmados en obra: tabique T07 perpendicular arriba y COL 02 abajo, sin apoyo</t>
         </is>
       </c>
     </row>
@@ -6001,7 +6141,7 @@
       <c r="A55" s="36" t="inlineStr"/>
       <c r="B55" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
+          <t xml:space="preserve">   intermedio. Para esta carga la seccion necesaria es 15x75.</t>
         </is>
       </c>
     </row>
@@ -6009,7 +6149,7 @@
       <c r="A56" s="36" t="inlineStr"/>
       <c r="B56" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
+          <t>VCH 03a (40x13, 3,83 m). Recibe L03, B = 2,08 m, y no</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6157,7 @@
       <c r="A57" s="36" t="inlineStr"/>
       <c r="B57" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
+          <t xml:space="preserve">   verifica: haria falta mas espesor. Tampoco verifica con B = 0,60 m, asi</t>
         </is>
       </c>
     </row>
@@ -6025,7 +6165,7 @@
       <c r="A58" s="36" t="inlineStr"/>
       <c r="B58" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
+          <t xml:space="preserve">   que el problema no es la hipotesis de carga sino la relacion luz/espesor. Una viga</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6173,7 @@
       <c r="A59" s="36" t="inlineStr"/>
       <c r="B59" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
+          <t xml:space="preserve">   chata del mismo espesor que la losa no puede ser apoyo lineal de un pano de 4,15 m.</t>
         </is>
       </c>
     </row>
@@ -6041,7 +6181,7 @@
       <c r="A60" s="36" t="inlineStr"/>
       <c r="B60" s="37" t="inlineStr">
         <is>
-          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
+          <t xml:space="preserve">   Revisar si tiene un muro debajo que acorte su luz libre.</t>
         </is>
       </c>
     </row>
@@ -6049,55 +6189,55 @@
       <c r="A61" s="36" t="inlineStr"/>
       <c r="B61" s="37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+          <t>VCH 03a (40x13, 3,71 m): excede la cuantia maxima y no llega a la altura minima por</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="36" t="inlineStr"/>
-      <c r="B62" s="37" t="inlineStr"/>
+      <c r="B62" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   flecha. Revisar el ancho tributario: si solo recibe el muro y no losa, baja mucho.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="36" t="inlineStr">
+      <c r="A63" s="36" t="inlineStr"/>
+      <c r="B63" s="37" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="36" t="inlineStr">
         <is>
           <t>8. ALCANCE</t>
         </is>
       </c>
-      <c r="B63" s="37" t="inlineStr">
+      <c r="B64" s="37" t="inlineStr">
         <is>
           <t>No se incluyen las 31 vigas de fundacion (VF01 a VF18c): su calculo depende de las</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="36" t="inlineStr"/>
-      <c r="B64" s="37" t="inlineStr">
-        <is>
-          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="36" t="inlineStr"/>
-      <c r="B65" s="37" t="inlineStr"/>
+      <c r="B65" s="37" t="inlineStr">
+        <is>
+          <t>cargas que bajan por las columnas y corresponde hacerlo despues. Tampoco losas ni columnas.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
-      <c r="A66" s="36" t="inlineStr">
+      <c r="A66" s="36" t="inlineStr"/>
+      <c r="B66" s="37" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="36" t="inlineStr">
         <is>
           <t>LIMITACIONES</t>
         </is>
       </c>
-      <c r="B66" s="36" t="inlineStr">
+      <c r="B67" s="36" t="inlineStr">
         <is>
           <t>El ancho tributario B esta relevado solo en</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="36" t="inlineStr"/>
-      <c r="B67" s="37" t="inlineStr">
-        <is>
-          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
@@ -6105,7 +6245,7 @@
       <c r="A68" s="36" t="inlineStr"/>
       <c r="B68" s="37" t="inlineStr">
         <is>
-          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
+          <t>VI 02 (0,80 m) y VCH 03a (2,08 m). En las demas sigue adoptado en 2,00 m, a falta</t>
         </is>
       </c>
     </row>
@@ -6113,13 +6253,21 @@
       <c r="A69" s="36" t="inlineStr"/>
       <c r="B69" s="37" t="inlineStr">
         <is>
-          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+          <t>hipotesis mas influyente del calculo: ajustarla viga por viga en la columna B trib.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="36" t="inlineStr"/>
       <c r="B70" s="37" t="inlineStr">
+        <is>
+          <t>El esquema se asigno por criterio: continua si integra una serie a-b-c o si supera 5,5 m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="36" t="inlineStr"/>
+      <c r="B71" s="37" t="inlineStr">
         <is>
           <t>Trabajo academico. Requiere verificacion y firma de profesional matriculado.</t>
         </is>

</xml_diff>

<commit_message>
Incorporar la carga puntual que VCH 05 descarga sobre VI 07c
VCH 05 apoya en el tabique T06b y en VI 07c, a 3,60 m del apoyo, y
le entrega 1.735 kg. Se superpone el momento isostatico P a b / L
repartido 0,75 al tramo y 0,50 al apoyo, y la reaccion isostatica al
corte. VI 07c pasa a 3d25 en tramo, 4d25 en apoyo y estribos d10
c/15, y sigue verificando. Se agregan las columnas P puntual y a en
el bloque de datos auxiliares.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -1827,7 +1827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF34"/>
+  <dimension ref="A1:AH34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1859,9 +1859,11 @@
     <col width="8" customWidth="1" min="27" max="27"/>
     <col width="10" customWidth="1" min="28" max="28"/>
     <col width="10" customWidth="1" min="29" max="29"/>
-    <col width="8" customWidth="1" min="30" max="30"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
     <col width="8" customWidth="1" min="31" max="31"/>
-    <col width="7" customWidth="1" min="32" max="32"/>
+    <col width="8" customWidth="1" min="32" max="32"/>
+    <col width="8" customWidth="1" min="33" max="33"/>
+    <col width="7" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1964,6 +1966,8 @@
       <c r="AD2" s="18" t="n"/>
       <c r="AE2" s="18" t="n"/>
       <c r="AF2" s="18" t="n"/>
+      <c r="AG2" s="18" t="n"/>
+      <c r="AH2" s="18" t="n"/>
     </row>
     <row r="3" ht="28" customHeight="1">
       <c r="A3" s="18" t="n"/>
@@ -2085,15 +2089,25 @@
       </c>
       <c r="AD3" s="19" t="inlineStr">
         <is>
+          <t>P punt. (kg)</t>
+        </is>
+      </c>
+      <c r="AE3" s="19" t="inlineStr">
+        <is>
+          <t>a (m)</t>
+        </is>
+      </c>
+      <c r="AF3" s="19" t="inlineStr">
+        <is>
           <t>B trib.</t>
         </is>
       </c>
-      <c r="AE3" s="19" t="inlineStr">
+      <c r="AG3" s="19" t="inlineStr">
         <is>
           <t>h muro</t>
         </is>
       </c>
-      <c r="AF3" s="19" t="inlineStr">
+      <c r="AH3" s="19" t="inlineStr">
         <is>
           <t>rec.</t>
         </is>
@@ -2114,12 +2128,12 @@
         <v>9.9</v>
       </c>
       <c r="D4" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD4+Datos!$B$7*J4*L4/10000+Datos!$B$16*AE4)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD4)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF4+Datos!$B$7*J4*L4/10000+Datos!$B$16*AG4)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF4)</f>
         <v/>
       </c>
       <c r="E4" s="7" t="n"/>
       <c r="F4" s="23">
-        <f>VLOOKUP(Y4,Datos!$A$19:$E$23,4,0)*D4*C4</f>
+        <f>VLOOKUP(Y4,Datos!$A$19:$E$23,4,0)*D4*C4+IF(OR(AD4="",AE4=""),0,AD4*MAX(AE4,C4-AE4)/C4)</f>
         <v/>
       </c>
       <c r="G4" s="23">
@@ -2127,18 +2141,18 @@
         <v/>
       </c>
       <c r="H4" s="23">
-        <f>VLOOKUP(Y4,Datos!$A$19:$E$23,2,0)*D4*C4^2</f>
+        <f>VLOOKUP(Y4,Datos!$A$19:$E$23,2,0)*D4*C4^2+0.75*1000*IF(OR(AD4="",AE4=""),0,AD4*AE4*(C4-AE4)/C4/1000)</f>
         <v/>
       </c>
       <c r="I4" s="23">
-        <f>IF(VLOOKUP(Y4,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y4,Datos!$A$19:$E$23,3,0)*D4*C4^2)</f>
+        <f>IF(VLOOKUP(Y4,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y4,Datos!$A$19:$E$23,3,0)*D4*C4^2+0.50*1000*IF(OR(AD4="",AE4=""),0,AD4*AE4*(C4-AE4)/C4/1000))</f>
         <v/>
       </c>
       <c r="J4" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K4" s="7">
-        <f>L4-AF4</f>
+        <f>L4-AH4</f>
         <v/>
       </c>
       <c r="L4" s="24" t="n">
@@ -2208,13 +2222,15 @@
         <f>IF(Z4="Invertida",MIN(C4*100/4,J4+16*AA4),J4)</f>
         <v/>
       </c>
-      <c r="AD4" s="24" t="n">
+      <c r="AD4" s="24" t="n"/>
+      <c r="AE4" s="24" t="n"/>
+      <c r="AF4" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE4" s="24" t="n">
+      <c r="AG4" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF4" s="24" t="n">
+      <c r="AH4" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2229,12 +2245,12 @@
         <v>3.95</v>
       </c>
       <c r="D5" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD5+Datos!$B$7*J5*L5/10000+Datos!$B$16*AE5)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD5)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF5+Datos!$B$7*J5*L5/10000+Datos!$B$16*AG5)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF5)</f>
         <v/>
       </c>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="23">
-        <f>VLOOKUP(Y5,Datos!$A$19:$E$23,4,0)*D5*C5</f>
+        <f>VLOOKUP(Y5,Datos!$A$19:$E$23,4,0)*D5*C5+IF(OR(AD5="",AE5=""),0,AD5*MAX(AE5,C5-AE5)/C5)</f>
         <v/>
       </c>
       <c r="G5" s="23">
@@ -2242,18 +2258,18 @@
         <v/>
       </c>
       <c r="H5" s="23">
-        <f>VLOOKUP(Y5,Datos!$A$19:$E$23,2,0)*D5*C5^2</f>
+        <f>VLOOKUP(Y5,Datos!$A$19:$E$23,2,0)*D5*C5^2+0.75*1000*IF(OR(AD5="",AE5=""),0,AD5*AE5*(C5-AE5)/C5/1000)</f>
         <v/>
       </c>
       <c r="I5" s="23">
-        <f>IF(VLOOKUP(Y5,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y5,Datos!$A$19:$E$23,3,0)*D5*C5^2)</f>
+        <f>IF(VLOOKUP(Y5,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y5,Datos!$A$19:$E$23,3,0)*D5*C5^2+0.50*1000*IF(OR(AD5="",AE5=""),0,AD5*AE5*(C5-AE5)/C5/1000))</f>
         <v/>
       </c>
       <c r="J5" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K5" s="7">
-        <f>L5-AF5</f>
+        <f>L5-AH5</f>
         <v/>
       </c>
       <c r="L5" s="24" t="n">
@@ -2323,13 +2339,15 @@
         <f>IF(Z5="Invertida",MIN(C5*100/4,J5+16*AA5),J5)</f>
         <v/>
       </c>
-      <c r="AD5" s="24" t="n">
+      <c r="AD5" s="24" t="n"/>
+      <c r="AE5" s="24" t="n"/>
+      <c r="AF5" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE5" s="24" t="n">
+      <c r="AG5" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF5" s="24" t="n">
+      <c r="AH5" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2344,12 +2362,12 @@
         <v>9.880000000000001</v>
       </c>
       <c r="D6" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD6+Datos!$B$7*J6*L6/10000+Datos!$B$16*AE6)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD6)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF6+Datos!$B$7*J6*L6/10000+Datos!$B$16*AG6)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF6)</f>
         <v/>
       </c>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="23">
-        <f>VLOOKUP(Y6,Datos!$A$19:$E$23,4,0)*D6*C6</f>
+        <f>VLOOKUP(Y6,Datos!$A$19:$E$23,4,0)*D6*C6+IF(OR(AD6="",AE6=""),0,AD6*MAX(AE6,C6-AE6)/C6)</f>
         <v/>
       </c>
       <c r="G6" s="23">
@@ -2357,18 +2375,18 @@
         <v/>
       </c>
       <c r="H6" s="23">
-        <f>VLOOKUP(Y6,Datos!$A$19:$E$23,2,0)*D6*C6^2</f>
+        <f>VLOOKUP(Y6,Datos!$A$19:$E$23,2,0)*D6*C6^2+0.75*1000*IF(OR(AD6="",AE6=""),0,AD6*AE6*(C6-AE6)/C6/1000)</f>
         <v/>
       </c>
       <c r="I6" s="23">
-        <f>IF(VLOOKUP(Y6,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y6,Datos!$A$19:$E$23,3,0)*D6*C6^2)</f>
+        <f>IF(VLOOKUP(Y6,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y6,Datos!$A$19:$E$23,3,0)*D6*C6^2+0.50*1000*IF(OR(AD6="",AE6=""),0,AD6*AE6*(C6-AE6)/C6/1000))</f>
         <v/>
       </c>
       <c r="J6" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K6" s="7">
-        <f>L6-AF6</f>
+        <f>L6-AH6</f>
         <v/>
       </c>
       <c r="L6" s="24" t="n">
@@ -2438,13 +2456,15 @@
         <f>IF(Z6="Invertida",MIN(C6*100/4,J6+16*AA6),J6)</f>
         <v/>
       </c>
-      <c r="AD6" s="24" t="n">
+      <c r="AD6" s="24" t="n"/>
+      <c r="AE6" s="24" t="n"/>
+      <c r="AF6" s="24" t="n">
         <v>2.689</v>
       </c>
-      <c r="AE6" s="24" t="n">
+      <c r="AG6" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF6" s="24" t="n">
+      <c r="AH6" s="24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -2459,12 +2479,12 @@
         <v>3.75</v>
       </c>
       <c r="D7" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD7+Datos!$B$7*J7*L7/10000+Datos!$B$16*AE7)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD7)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF7+Datos!$B$7*J7*L7/10000+Datos!$B$16*AG7)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF7)</f>
         <v/>
       </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="23">
-        <f>VLOOKUP(Y7,Datos!$A$19:$E$23,4,0)*D7*C7</f>
+        <f>VLOOKUP(Y7,Datos!$A$19:$E$23,4,0)*D7*C7+IF(OR(AD7="",AE7=""),0,AD7*MAX(AE7,C7-AE7)/C7)</f>
         <v/>
       </c>
       <c r="G7" s="23">
@@ -2472,18 +2492,18 @@
         <v/>
       </c>
       <c r="H7" s="23">
-        <f>VLOOKUP(Y7,Datos!$A$19:$E$23,2,0)*D7*C7^2</f>
+        <f>VLOOKUP(Y7,Datos!$A$19:$E$23,2,0)*D7*C7^2+0.75*1000*IF(OR(AD7="",AE7=""),0,AD7*AE7*(C7-AE7)/C7/1000)</f>
         <v/>
       </c>
       <c r="I7" s="23">
-        <f>IF(VLOOKUP(Y7,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y7,Datos!$A$19:$E$23,3,0)*D7*C7^2)</f>
+        <f>IF(VLOOKUP(Y7,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y7,Datos!$A$19:$E$23,3,0)*D7*C7^2+0.50*1000*IF(OR(AD7="",AE7=""),0,AD7*AE7*(C7-AE7)/C7/1000))</f>
         <v/>
       </c>
       <c r="J7" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K7" s="7">
-        <f>L7-AF7</f>
+        <f>L7-AH7</f>
         <v/>
       </c>
       <c r="L7" s="24" t="n">
@@ -2549,13 +2569,15 @@
         <f>IF(Z7="Invertida",MIN(C7*100/4,J7+16*AA7),J7)</f>
         <v/>
       </c>
-      <c r="AD7" s="24" t="n">
+      <c r="AD7" s="24" t="n"/>
+      <c r="AE7" s="24" t="n"/>
+      <c r="AF7" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE7" s="24" t="n">
+      <c r="AG7" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF7" s="24" t="n">
+      <c r="AH7" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2570,12 +2592,12 @@
         <v>3.75</v>
       </c>
       <c r="D8" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD8+Datos!$B$7*J8*L8/10000+Datos!$B$16*AE8)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD8)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF8+Datos!$B$7*J8*L8/10000+Datos!$B$16*AG8)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF8)</f>
         <v/>
       </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="23">
-        <f>VLOOKUP(Y8,Datos!$A$19:$E$23,4,0)*D8*C8</f>
+        <f>VLOOKUP(Y8,Datos!$A$19:$E$23,4,0)*D8*C8+IF(OR(AD8="",AE8=""),0,AD8*MAX(AE8,C8-AE8)/C8)</f>
         <v/>
       </c>
       <c r="G8" s="23">
@@ -2583,18 +2605,18 @@
         <v/>
       </c>
       <c r="H8" s="23">
-        <f>VLOOKUP(Y8,Datos!$A$19:$E$23,2,0)*D8*C8^2</f>
+        <f>VLOOKUP(Y8,Datos!$A$19:$E$23,2,0)*D8*C8^2+0.75*1000*IF(OR(AD8="",AE8=""),0,AD8*AE8*(C8-AE8)/C8/1000)</f>
         <v/>
       </c>
       <c r="I8" s="23">
-        <f>IF(VLOOKUP(Y8,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y8,Datos!$A$19:$E$23,3,0)*D8*C8^2)</f>
+        <f>IF(VLOOKUP(Y8,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y8,Datos!$A$19:$E$23,3,0)*D8*C8^2+0.50*1000*IF(OR(AD8="",AE8=""),0,AD8*AE8*(C8-AE8)/C8/1000))</f>
         <v/>
       </c>
       <c r="J8" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K8" s="7">
-        <f>L8-AF8</f>
+        <f>L8-AH8</f>
         <v/>
       </c>
       <c r="L8" s="24" t="n">
@@ -2660,13 +2682,15 @@
         <f>IF(Z8="Invertida",MIN(C8*100/4,J8+16*AA8),J8)</f>
         <v/>
       </c>
-      <c r="AD8" s="24" t="n">
+      <c r="AD8" s="24" t="n"/>
+      <c r="AE8" s="24" t="n"/>
+      <c r="AF8" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE8" s="24" t="n">
+      <c r="AG8" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF8" s="24" t="n">
+      <c r="AH8" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2681,12 +2705,12 @@
         <v>3.8</v>
       </c>
       <c r="D9" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD9+Datos!$B$7*J9*L9/10000+Datos!$B$16*AE9)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD9)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF9+Datos!$B$7*J9*L9/10000+Datos!$B$16*AG9)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF9)</f>
         <v/>
       </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="23">
-        <f>VLOOKUP(Y9,Datos!$A$19:$E$23,4,0)*D9*C9</f>
+        <f>VLOOKUP(Y9,Datos!$A$19:$E$23,4,0)*D9*C9+IF(OR(AD9="",AE9=""),0,AD9*MAX(AE9,C9-AE9)/C9)</f>
         <v/>
       </c>
       <c r="G9" s="23">
@@ -2694,18 +2718,18 @@
         <v/>
       </c>
       <c r="H9" s="23">
-        <f>VLOOKUP(Y9,Datos!$A$19:$E$23,2,0)*D9*C9^2</f>
+        <f>VLOOKUP(Y9,Datos!$A$19:$E$23,2,0)*D9*C9^2+0.75*1000*IF(OR(AD9="",AE9=""),0,AD9*AE9*(C9-AE9)/C9/1000)</f>
         <v/>
       </c>
       <c r="I9" s="23">
-        <f>IF(VLOOKUP(Y9,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y9,Datos!$A$19:$E$23,3,0)*D9*C9^2)</f>
+        <f>IF(VLOOKUP(Y9,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y9,Datos!$A$19:$E$23,3,0)*D9*C9^2+0.50*1000*IF(OR(AD9="",AE9=""),0,AD9*AE9*(C9-AE9)/C9/1000))</f>
         <v/>
       </c>
       <c r="J9" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K9" s="7">
-        <f>L9-AF9</f>
+        <f>L9-AH9</f>
         <v/>
       </c>
       <c r="L9" s="24" t="n">
@@ -2771,13 +2795,15 @@
         <f>IF(Z9="Invertida",MIN(C9*100/4,J9+16*AA9),J9)</f>
         <v/>
       </c>
-      <c r="AD9" s="24" t="n">
+      <c r="AD9" s="24" t="n"/>
+      <c r="AE9" s="24" t="n"/>
+      <c r="AF9" s="24" t="n">
         <v>1.549</v>
       </c>
-      <c r="AE9" s="24" t="n">
+      <c r="AG9" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF9" s="24" t="n">
+      <c r="AH9" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2792,12 +2818,12 @@
         <v>6.53</v>
       </c>
       <c r="D10" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AE10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD10)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF10+Datos!$B$7*J10*L10/10000+Datos!$B$16*AG10)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF10)</f>
         <v/>
       </c>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="23">
-        <f>VLOOKUP(Y10,Datos!$A$19:$E$23,4,0)*D10*C10</f>
+        <f>VLOOKUP(Y10,Datos!$A$19:$E$23,4,0)*D10*C10+IF(OR(AD10="",AE10=""),0,AD10*MAX(AE10,C10-AE10)/C10)</f>
         <v/>
       </c>
       <c r="G10" s="23">
@@ -2805,18 +2831,18 @@
         <v/>
       </c>
       <c r="H10" s="23">
-        <f>VLOOKUP(Y10,Datos!$A$19:$E$23,2,0)*D10*C10^2</f>
+        <f>VLOOKUP(Y10,Datos!$A$19:$E$23,2,0)*D10*C10^2+0.75*1000*IF(OR(AD10="",AE10=""),0,AD10*AE10*(C10-AE10)/C10/1000)</f>
         <v/>
       </c>
       <c r="I10" s="23">
-        <f>IF(VLOOKUP(Y10,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y10,Datos!$A$19:$E$23,3,0)*D10*C10^2)</f>
+        <f>IF(VLOOKUP(Y10,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y10,Datos!$A$19:$E$23,3,0)*D10*C10^2+0.50*1000*IF(OR(AD10="",AE10=""),0,AD10*AE10*(C10-AE10)/C10/1000))</f>
         <v/>
       </c>
       <c r="J10" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K10" s="7">
-        <f>L10-AF10</f>
+        <f>L10-AH10</f>
         <v/>
       </c>
       <c r="L10" s="24" t="n">
@@ -2886,13 +2912,15 @@
         <f>IF(Z10="Invertida",MIN(C10*100/4,J10+16*AA10),J10)</f>
         <v/>
       </c>
-      <c r="AD10" s="24" t="n">
+      <c r="AD10" s="24" t="n"/>
+      <c r="AE10" s="24" t="n"/>
+      <c r="AF10" s="24" t="n">
         <v>1.549</v>
       </c>
-      <c r="AE10" s="24" t="n">
+      <c r="AG10" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF10" s="24" t="n">
+      <c r="AH10" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -2907,12 +2935,12 @@
         <v>3.37</v>
       </c>
       <c r="D11" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AE11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD11)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF11+Datos!$B$7*J11*L11/10000+Datos!$B$16*AG11)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF11)</f>
         <v/>
       </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="23">
-        <f>VLOOKUP(Y11,Datos!$A$19:$E$23,4,0)*D11*C11</f>
+        <f>VLOOKUP(Y11,Datos!$A$19:$E$23,4,0)*D11*C11+IF(OR(AD11="",AE11=""),0,AD11*MAX(AE11,C11-AE11)/C11)</f>
         <v/>
       </c>
       <c r="G11" s="23">
@@ -2920,18 +2948,18 @@
         <v/>
       </c>
       <c r="H11" s="23">
-        <f>VLOOKUP(Y11,Datos!$A$19:$E$23,2,0)*D11*C11^2</f>
+        <f>VLOOKUP(Y11,Datos!$A$19:$E$23,2,0)*D11*C11^2+0.75*1000*IF(OR(AD11="",AE11=""),0,AD11*AE11*(C11-AE11)/C11/1000)</f>
         <v/>
       </c>
       <c r="I11" s="23">
-        <f>IF(VLOOKUP(Y11,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y11,Datos!$A$19:$E$23,3,0)*D11*C11^2)</f>
+        <f>IF(VLOOKUP(Y11,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y11,Datos!$A$19:$E$23,3,0)*D11*C11^2+0.50*1000*IF(OR(AD11="",AE11=""),0,AD11*AE11*(C11-AE11)/C11/1000))</f>
         <v/>
       </c>
       <c r="J11" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K11" s="7">
-        <f>L11-AF11</f>
+        <f>L11-AH11</f>
         <v/>
       </c>
       <c r="L11" s="24" t="n">
@@ -3001,13 +3029,15 @@
         <f>IF(Z11="Invertida",MIN(C11*100/4,J11+16*AA11),J11)</f>
         <v/>
       </c>
-      <c r="AD11" s="24" t="n">
+      <c r="AD11" s="24" t="n"/>
+      <c r="AE11" s="24" t="n"/>
+      <c r="AF11" s="24" t="n">
         <v>0.78</v>
       </c>
-      <c r="AE11" s="24" t="n">
+      <c r="AG11" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF11" s="24" t="n">
+      <c r="AH11" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3022,12 +3052,12 @@
         <v>4.03</v>
       </c>
       <c r="D12" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AE12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD12)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF12+Datos!$B$7*J12*L12/10000+Datos!$B$16*AG12)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF12)</f>
         <v/>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="23">
-        <f>VLOOKUP(Y12,Datos!$A$19:$E$23,4,0)*D12*C12</f>
+        <f>VLOOKUP(Y12,Datos!$A$19:$E$23,4,0)*D12*C12+IF(OR(AD12="",AE12=""),0,AD12*MAX(AE12,C12-AE12)/C12)</f>
         <v/>
       </c>
       <c r="G12" s="23">
@@ -3035,18 +3065,18 @@
         <v/>
       </c>
       <c r="H12" s="23">
-        <f>VLOOKUP(Y12,Datos!$A$19:$E$23,2,0)*D12*C12^2</f>
+        <f>VLOOKUP(Y12,Datos!$A$19:$E$23,2,0)*D12*C12^2+0.75*1000*IF(OR(AD12="",AE12=""),0,AD12*AE12*(C12-AE12)/C12/1000)</f>
         <v/>
       </c>
       <c r="I12" s="23">
-        <f>IF(VLOOKUP(Y12,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y12,Datos!$A$19:$E$23,3,0)*D12*C12^2)</f>
+        <f>IF(VLOOKUP(Y12,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y12,Datos!$A$19:$E$23,3,0)*D12*C12^2+0.50*1000*IF(OR(AD12="",AE12=""),0,AD12*AE12*(C12-AE12)/C12/1000))</f>
         <v/>
       </c>
       <c r="J12" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K12" s="7">
-        <f>L12-AF12</f>
+        <f>L12-AH12</f>
         <v/>
       </c>
       <c r="L12" s="24" t="n">
@@ -3116,13 +3146,15 @@
         <f>IF(Z12="Invertida",MIN(C12*100/4,J12+16*AA12),J12)</f>
         <v/>
       </c>
-      <c r="AD12" s="24" t="n">
+      <c r="AD12" s="24" t="n"/>
+      <c r="AE12" s="24" t="n"/>
+      <c r="AF12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE12" s="24" t="n">
+      <c r="AG12" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF12" s="24" t="n">
+      <c r="AH12" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3137,12 +3169,12 @@
         <v>8.6</v>
       </c>
       <c r="D13" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AE13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD13)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF13+Datos!$B$7*J13*L13/10000+Datos!$B$16*AG13)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF13)</f>
         <v/>
       </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="23">
-        <f>VLOOKUP(Y13,Datos!$A$19:$E$23,4,0)*D13*C13</f>
+        <f>VLOOKUP(Y13,Datos!$A$19:$E$23,4,0)*D13*C13+IF(OR(AD13="",AE13=""),0,AD13*MAX(AE13,C13-AE13)/C13)</f>
         <v/>
       </c>
       <c r="G13" s="23">
@@ -3150,18 +3182,18 @@
         <v/>
       </c>
       <c r="H13" s="23">
-        <f>VLOOKUP(Y13,Datos!$A$19:$E$23,2,0)*D13*C13^2</f>
+        <f>VLOOKUP(Y13,Datos!$A$19:$E$23,2,0)*D13*C13^2+0.75*1000*IF(OR(AD13="",AE13=""),0,AD13*AE13*(C13-AE13)/C13/1000)</f>
         <v/>
       </c>
       <c r="I13" s="23">
-        <f>IF(VLOOKUP(Y13,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y13,Datos!$A$19:$E$23,3,0)*D13*C13^2)</f>
+        <f>IF(VLOOKUP(Y13,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y13,Datos!$A$19:$E$23,3,0)*D13*C13^2+0.50*1000*IF(OR(AD13="",AE13=""),0,AD13*AE13*(C13-AE13)/C13/1000))</f>
         <v/>
       </c>
       <c r="J13" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K13" s="7">
-        <f>L13-AF13</f>
+        <f>L13-AH13</f>
         <v/>
       </c>
       <c r="L13" s="24" t="n">
@@ -3172,10 +3204,10 @@
         <v/>
       </c>
       <c r="N13" s="24" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O13" s="24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="P13" s="25">
         <f>IF(NOT(ISNUMBER(I13)),"---",IF(I13&lt;=0,"---",IF(I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I13*100/(Datos!$B$8*AC13*K13^2*Datos!$B$5)))*AC13*K13*Datos!$B$5/Datos!$B$6,0.0033*J13*K13))))</f>
@@ -3196,10 +3228,10 @@
         <v/>
       </c>
       <c r="U13" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V13" s="24" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="W13" s="7">
         <f>IF(OR(M13="REVISAR",P13="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M13&lt;&gt;"REVISAR",P13&lt;&gt;"REVISAR",IF(ISNUMBER(M13),N13*PI()*(O13/10)^2/4&gt;=M13,TRUE),IF(ISNUMBER(P13),Q13*PI()*(R13/10)^2/4&gt;=P13,TRUE),IF(ISNUMBER(M13),M13&lt;=0.0163*AB13*K13,TRUE),IF(ISNUMBER(P13),P13&lt;=0.0163*AC13*K13,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F13&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J13*K13+2*PI()*(U13/10)^2/4*Datos!$B$6*K13/V13)),"NO VERIF. CORTE",IF(NOT(L13&gt;=C13*100/VLOOKUP(Y13,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -3207,7 +3239,7 @@
       </c>
       <c r="X13" s="26" t="inlineStr">
         <is>
-          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
+          <t>Armadura en 2 capas (rec. 6 cm). Apoya en columna COL 02 de 15x30 y en el tabique T05b. La viga chata VCH 05 le descarga 1.735 kg a 3,60 m del apoyo. Se superpone el momento isostatico P a b / L repartido 0,75 al tramo y 0,50 al apoyo, y la reaccion isostatica al corte. Viga de borde: recibe la reaccion de la losa excentrica y queda sometida a TORSION, no verificada en esta planilla.</t>
         </is>
       </c>
       <c r="Y13" s="24" t="inlineStr">
@@ -3232,12 +3264,18 @@
         <v/>
       </c>
       <c r="AD13" s="24" t="n">
+        <v>1735</v>
+      </c>
+      <c r="AE13" s="24" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="AF13" s="24" t="n">
         <v>3.71</v>
       </c>
-      <c r="AE13" s="24" t="n">
+      <c r="AG13" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF13" s="24" t="n">
+      <c r="AH13" s="24" t="n">
         <v>6</v>
       </c>
     </row>
@@ -3252,12 +3290,12 @@
         <v>3.65</v>
       </c>
       <c r="D14" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AE14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD14)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF14+Datos!$B$7*J14*L14/10000+Datos!$B$16*AG14)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF14)</f>
         <v/>
       </c>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="23">
-        <f>VLOOKUP(Y14,Datos!$A$19:$E$23,4,0)*D14*C14</f>
+        <f>VLOOKUP(Y14,Datos!$A$19:$E$23,4,0)*D14*C14+IF(OR(AD14="",AE14=""),0,AD14*MAX(AE14,C14-AE14)/C14)</f>
         <v/>
       </c>
       <c r="G14" s="23">
@@ -3265,18 +3303,18 @@
         <v/>
       </c>
       <c r="H14" s="23">
-        <f>VLOOKUP(Y14,Datos!$A$19:$E$23,2,0)*D14*C14^2</f>
+        <f>VLOOKUP(Y14,Datos!$A$19:$E$23,2,0)*D14*C14^2+0.75*1000*IF(OR(AD14="",AE14=""),0,AD14*AE14*(C14-AE14)/C14/1000)</f>
         <v/>
       </c>
       <c r="I14" s="23">
-        <f>IF(VLOOKUP(Y14,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y14,Datos!$A$19:$E$23,3,0)*D14*C14^2)</f>
+        <f>IF(VLOOKUP(Y14,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y14,Datos!$A$19:$E$23,3,0)*D14*C14^2+0.50*1000*IF(OR(AD14="",AE14=""),0,AD14*AE14*(C14-AE14)/C14/1000))</f>
         <v/>
       </c>
       <c r="J14" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K14" s="7">
-        <f>L14-AF14</f>
+        <f>L14-AH14</f>
         <v/>
       </c>
       <c r="L14" s="24" t="n">
@@ -3342,13 +3380,15 @@
         <f>IF(Z14="Invertida",MIN(C14*100/4,J14+16*AA14),J14)</f>
         <v/>
       </c>
-      <c r="AD14" s="24" t="n">
+      <c r="AD14" s="24" t="n"/>
+      <c r="AE14" s="24" t="n"/>
+      <c r="AF14" s="24" t="n">
         <v>1.065</v>
       </c>
-      <c r="AE14" s="24" t="n">
+      <c r="AG14" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF14" s="24" t="n">
+      <c r="AH14" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3363,12 +3403,12 @@
         <v>4.87</v>
       </c>
       <c r="D15" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD15+Datos!$B$7*J15*L15/10000+Datos!$B$16*AE15)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD15)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF15+Datos!$B$7*J15*L15/10000+Datos!$B$16*AG15)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF15)</f>
         <v/>
       </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="23">
-        <f>VLOOKUP(Y15,Datos!$A$19:$E$23,4,0)*D15*C15</f>
+        <f>VLOOKUP(Y15,Datos!$A$19:$E$23,4,0)*D15*C15+IF(OR(AD15="",AE15=""),0,AD15*MAX(AE15,C15-AE15)/C15)</f>
         <v/>
       </c>
       <c r="G15" s="23">
@@ -3376,18 +3416,18 @@
         <v/>
       </c>
       <c r="H15" s="23">
-        <f>VLOOKUP(Y15,Datos!$A$19:$E$23,2,0)*D15*C15^2</f>
+        <f>VLOOKUP(Y15,Datos!$A$19:$E$23,2,0)*D15*C15^2+0.75*1000*IF(OR(AD15="",AE15=""),0,AD15*AE15*(C15-AE15)/C15/1000)</f>
         <v/>
       </c>
       <c r="I15" s="23">
-        <f>IF(VLOOKUP(Y15,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y15,Datos!$A$19:$E$23,3,0)*D15*C15^2)</f>
+        <f>IF(VLOOKUP(Y15,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y15,Datos!$A$19:$E$23,3,0)*D15*C15^2+0.50*1000*IF(OR(AD15="",AE15=""),0,AD15*AE15*(C15-AE15)/C15/1000))</f>
         <v/>
       </c>
       <c r="J15" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K15" s="7">
-        <f>L15-AF15</f>
+        <f>L15-AH15</f>
         <v/>
       </c>
       <c r="L15" s="24" t="n">
@@ -3453,13 +3493,15 @@
         <f>IF(Z15="Invertida",MIN(C15*100/4,J15+16*AA15),J15)</f>
         <v/>
       </c>
-      <c r="AD15" s="24" t="n">
+      <c r="AD15" s="24" t="n"/>
+      <c r="AE15" s="24" t="n"/>
+      <c r="AF15" s="24" t="n">
         <v>1.065</v>
       </c>
-      <c r="AE15" s="24" t="n">
+      <c r="AG15" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF15" s="24" t="n">
+      <c r="AH15" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3474,12 +3516,12 @@
         <v>4.87</v>
       </c>
       <c r="D16" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AE16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD16)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF16+Datos!$B$7*J16*L16/10000+Datos!$B$16*AG16)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF16)</f>
         <v/>
       </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="23">
-        <f>VLOOKUP(Y16,Datos!$A$19:$E$23,4,0)*D16*C16</f>
+        <f>VLOOKUP(Y16,Datos!$A$19:$E$23,4,0)*D16*C16+IF(OR(AD16="",AE16=""),0,AD16*MAX(AE16,C16-AE16)/C16)</f>
         <v/>
       </c>
       <c r="G16" s="23">
@@ -3487,18 +3529,18 @@
         <v/>
       </c>
       <c r="H16" s="23">
-        <f>VLOOKUP(Y16,Datos!$A$19:$E$23,2,0)*D16*C16^2</f>
+        <f>VLOOKUP(Y16,Datos!$A$19:$E$23,2,0)*D16*C16^2+0.75*1000*IF(OR(AD16="",AE16=""),0,AD16*AE16*(C16-AE16)/C16/1000)</f>
         <v/>
       </c>
       <c r="I16" s="23">
-        <f>IF(VLOOKUP(Y16,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y16,Datos!$A$19:$E$23,3,0)*D16*C16^2)</f>
+        <f>IF(VLOOKUP(Y16,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y16,Datos!$A$19:$E$23,3,0)*D16*C16^2+0.50*1000*IF(OR(AD16="",AE16=""),0,AD16*AE16*(C16-AE16)/C16/1000))</f>
         <v/>
       </c>
       <c r="J16" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K16" s="7">
-        <f>L16-AF16</f>
+        <f>L16-AH16</f>
         <v/>
       </c>
       <c r="L16" s="24" t="n">
@@ -3568,13 +3610,15 @@
         <f>IF(Z16="Invertida",MIN(C16*100/4,J16+16*AA16),J16)</f>
         <v/>
       </c>
-      <c r="AD16" s="24" t="n">
+      <c r="AD16" s="24" t="n"/>
+      <c r="AE16" s="24" t="n"/>
+      <c r="AF16" s="24" t="n">
         <v>1.549</v>
       </c>
-      <c r="AE16" s="24" t="n">
+      <c r="AG16" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF16" s="24" t="n">
+      <c r="AH16" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3589,12 +3633,12 @@
         <v>2.55</v>
       </c>
       <c r="D17" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AE17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD17)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF17+Datos!$B$7*J17*L17/10000+Datos!$B$16*AG17)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF17)</f>
         <v/>
       </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="23">
-        <f>VLOOKUP(Y17,Datos!$A$19:$E$23,4,0)*D17*C17</f>
+        <f>VLOOKUP(Y17,Datos!$A$19:$E$23,4,0)*D17*C17+IF(OR(AD17="",AE17=""),0,AD17*MAX(AE17,C17-AE17)/C17)</f>
         <v/>
       </c>
       <c r="G17" s="23">
@@ -3602,18 +3646,18 @@
         <v/>
       </c>
       <c r="H17" s="23">
-        <f>VLOOKUP(Y17,Datos!$A$19:$E$23,2,0)*D17*C17^2</f>
+        <f>VLOOKUP(Y17,Datos!$A$19:$E$23,2,0)*D17*C17^2+0.75*1000*IF(OR(AD17="",AE17=""),0,AD17*AE17*(C17-AE17)/C17/1000)</f>
         <v/>
       </c>
       <c r="I17" s="23">
-        <f>IF(VLOOKUP(Y17,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y17,Datos!$A$19:$E$23,3,0)*D17*C17^2)</f>
+        <f>IF(VLOOKUP(Y17,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y17,Datos!$A$19:$E$23,3,0)*D17*C17^2+0.50*1000*IF(OR(AD17="",AE17=""),0,AD17*AE17*(C17-AE17)/C17/1000))</f>
         <v/>
       </c>
       <c r="J17" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K17" s="7">
-        <f>L17-AF17</f>
+        <f>L17-AH17</f>
         <v/>
       </c>
       <c r="L17" s="24" t="n">
@@ -3679,13 +3723,15 @@
         <f>IF(Z17="Invertida",MIN(C17*100/4,J17+16*AA17),J17)</f>
         <v/>
       </c>
-      <c r="AD17" s="24" t="n">
+      <c r="AD17" s="24" t="n"/>
+      <c r="AE17" s="24" t="n"/>
+      <c r="AF17" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE17" s="24" t="n">
+      <c r="AG17" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF17" s="24" t="n">
+      <c r="AH17" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3700,12 +3746,12 @@
         <v>4</v>
       </c>
       <c r="D18" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AE18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD18)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF18+Datos!$B$7*J18*L18/10000+Datos!$B$16*AG18)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF18)</f>
         <v/>
       </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="23">
-        <f>VLOOKUP(Y18,Datos!$A$19:$E$23,4,0)*D18*C18</f>
+        <f>VLOOKUP(Y18,Datos!$A$19:$E$23,4,0)*D18*C18+IF(OR(AD18="",AE18=""),0,AD18*MAX(AE18,C18-AE18)/C18)</f>
         <v/>
       </c>
       <c r="G18" s="23">
@@ -3713,18 +3759,18 @@
         <v/>
       </c>
       <c r="H18" s="23">
-        <f>VLOOKUP(Y18,Datos!$A$19:$E$23,2,0)*D18*C18^2</f>
+        <f>VLOOKUP(Y18,Datos!$A$19:$E$23,2,0)*D18*C18^2+0.75*1000*IF(OR(AD18="",AE18=""),0,AD18*AE18*(C18-AE18)/C18/1000)</f>
         <v/>
       </c>
       <c r="I18" s="23">
-        <f>IF(VLOOKUP(Y18,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y18,Datos!$A$19:$E$23,3,0)*D18*C18^2)</f>
+        <f>IF(VLOOKUP(Y18,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y18,Datos!$A$19:$E$23,3,0)*D18*C18^2+0.50*1000*IF(OR(AD18="",AE18=""),0,AD18*AE18*(C18-AE18)/C18/1000))</f>
         <v/>
       </c>
       <c r="J18" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K18" s="7">
-        <f>L18-AF18</f>
+        <f>L18-AH18</f>
         <v/>
       </c>
       <c r="L18" s="24" t="n">
@@ -3790,13 +3836,15 @@
         <f>IF(Z18="Invertida",MIN(C18*100/4,J18+16*AA18),J18)</f>
         <v/>
       </c>
-      <c r="AD18" s="24" t="n">
+      <c r="AD18" s="24" t="n"/>
+      <c r="AE18" s="24" t="n"/>
+      <c r="AF18" s="24" t="n">
         <v>1.825</v>
       </c>
-      <c r="AE18" s="24" t="n">
+      <c r="AG18" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF18" s="24" t="n">
+      <c r="AH18" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3811,12 +3859,12 @@
         <v>3.6</v>
       </c>
       <c r="D19" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AE19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD19)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF19+Datos!$B$7*J19*L19/10000+Datos!$B$16*AG19)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF19)</f>
         <v/>
       </c>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="23">
-        <f>VLOOKUP(Y19,Datos!$A$19:$E$23,4,0)*D19*C19</f>
+        <f>VLOOKUP(Y19,Datos!$A$19:$E$23,4,0)*D19*C19+IF(OR(AD19="",AE19=""),0,AD19*MAX(AE19,C19-AE19)/C19)</f>
         <v/>
       </c>
       <c r="G19" s="23">
@@ -3824,18 +3872,18 @@
         <v/>
       </c>
       <c r="H19" s="23">
-        <f>VLOOKUP(Y19,Datos!$A$19:$E$23,2,0)*D19*C19^2</f>
+        <f>VLOOKUP(Y19,Datos!$A$19:$E$23,2,0)*D19*C19^2+0.75*1000*IF(OR(AD19="",AE19=""),0,AD19*AE19*(C19-AE19)/C19/1000)</f>
         <v/>
       </c>
       <c r="I19" s="23">
-        <f>IF(VLOOKUP(Y19,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y19,Datos!$A$19:$E$23,3,0)*D19*C19^2)</f>
+        <f>IF(VLOOKUP(Y19,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y19,Datos!$A$19:$E$23,3,0)*D19*C19^2+0.50*1000*IF(OR(AD19="",AE19=""),0,AD19*AE19*(C19-AE19)/C19/1000))</f>
         <v/>
       </c>
       <c r="J19" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K19" s="7">
-        <f>L19-AF19</f>
+        <f>L19-AH19</f>
         <v/>
       </c>
       <c r="L19" s="24" t="n">
@@ -3901,13 +3949,15 @@
         <f>IF(Z19="Invertida",MIN(C19*100/4,J19+16*AA19),J19)</f>
         <v/>
       </c>
-      <c r="AD19" s="24" t="n">
+      <c r="AD19" s="24" t="n"/>
+      <c r="AE19" s="24" t="n"/>
+      <c r="AF19" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE19" s="24" t="n">
+      <c r="AG19" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF19" s="24" t="n">
+      <c r="AH19" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -3922,12 +3972,12 @@
         <v>7.68</v>
       </c>
       <c r="D20" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AE20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD20)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF20+Datos!$B$7*J20*L20/10000+Datos!$B$16*AG20)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF20)</f>
         <v/>
       </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="23">
-        <f>VLOOKUP(Y20,Datos!$A$19:$E$23,4,0)*D20*C20</f>
+        <f>VLOOKUP(Y20,Datos!$A$19:$E$23,4,0)*D20*C20+IF(OR(AD20="",AE20=""),0,AD20*MAX(AE20,C20-AE20)/C20)</f>
         <v/>
       </c>
       <c r="G20" s="23">
@@ -3935,18 +3985,18 @@
         <v/>
       </c>
       <c r="H20" s="23">
-        <f>VLOOKUP(Y20,Datos!$A$19:$E$23,2,0)*D20*C20^2</f>
+        <f>VLOOKUP(Y20,Datos!$A$19:$E$23,2,0)*D20*C20^2+0.75*1000*IF(OR(AD20="",AE20=""),0,AD20*AE20*(C20-AE20)/C20/1000)</f>
         <v/>
       </c>
       <c r="I20" s="23">
-        <f>IF(VLOOKUP(Y20,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y20,Datos!$A$19:$E$23,3,0)*D20*C20^2)</f>
+        <f>IF(VLOOKUP(Y20,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y20,Datos!$A$19:$E$23,3,0)*D20*C20^2+0.50*1000*IF(OR(AD20="",AE20=""),0,AD20*AE20*(C20-AE20)/C20/1000))</f>
         <v/>
       </c>
       <c r="J20" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K20" s="7">
-        <f>L20-AF20</f>
+        <f>L20-AH20</f>
         <v/>
       </c>
       <c r="L20" s="24" t="n">
@@ -4016,13 +4066,15 @@
         <f>IF(Z20="Invertida",MIN(C20*100/4,J20+16*AA20),J20)</f>
         <v/>
       </c>
-      <c r="AD20" s="24" t="n">
+      <c r="AD20" s="24" t="n"/>
+      <c r="AE20" s="24" t="n"/>
+      <c r="AF20" s="24" t="n">
         <v>1.825</v>
       </c>
-      <c r="AE20" s="24" t="n">
+      <c r="AG20" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF20" s="24" t="n">
+      <c r="AH20" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4037,12 +4089,12 @@
         <v>3.45</v>
       </c>
       <c r="D21" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AE21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD21)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF21+Datos!$B$7*J21*L21/10000+Datos!$B$16*AG21)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF21)</f>
         <v/>
       </c>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="23">
-        <f>VLOOKUP(Y21,Datos!$A$19:$E$23,4,0)*D21*C21</f>
+        <f>VLOOKUP(Y21,Datos!$A$19:$E$23,4,0)*D21*C21+IF(OR(AD21="",AE21=""),0,AD21*MAX(AE21,C21-AE21)/C21)</f>
         <v/>
       </c>
       <c r="G21" s="23">
@@ -4050,18 +4102,18 @@
         <v/>
       </c>
       <c r="H21" s="23">
-        <f>VLOOKUP(Y21,Datos!$A$19:$E$23,2,0)*D21*C21^2</f>
+        <f>VLOOKUP(Y21,Datos!$A$19:$E$23,2,0)*D21*C21^2+0.75*1000*IF(OR(AD21="",AE21=""),0,AD21*AE21*(C21-AE21)/C21/1000)</f>
         <v/>
       </c>
       <c r="I21" s="23">
-        <f>IF(VLOOKUP(Y21,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y21,Datos!$A$19:$E$23,3,0)*D21*C21^2)</f>
+        <f>IF(VLOOKUP(Y21,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y21,Datos!$A$19:$E$23,3,0)*D21*C21^2+0.50*1000*IF(OR(AD21="",AE21=""),0,AD21*AE21*(C21-AE21)/C21/1000))</f>
         <v/>
       </c>
       <c r="J21" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K21" s="7">
-        <f>L21-AF21</f>
+        <f>L21-AH21</f>
         <v/>
       </c>
       <c r="L21" s="24" t="n">
@@ -4131,13 +4183,15 @@
         <f>IF(Z21="Invertida",MIN(C21*100/4,J21+16*AA21),J21)</f>
         <v/>
       </c>
-      <c r="AD21" s="24" t="n">
+      <c r="AD21" s="24" t="n"/>
+      <c r="AE21" s="24" t="n"/>
+      <c r="AF21" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE21" s="24" t="n">
+      <c r="AG21" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF21" s="24" t="n">
+      <c r="AH21" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4152,12 +4206,12 @@
         <v>5.02</v>
       </c>
       <c r="D22" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AE22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD22)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF22+Datos!$B$7*J22*L22/10000+Datos!$B$16*AG22)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF22)</f>
         <v/>
       </c>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="23">
-        <f>VLOOKUP(Y22,Datos!$A$19:$E$23,4,0)*D22*C22</f>
+        <f>VLOOKUP(Y22,Datos!$A$19:$E$23,4,0)*D22*C22+IF(OR(AD22="",AE22=""),0,AD22*MAX(AE22,C22-AE22)/C22)</f>
         <v/>
       </c>
       <c r="G22" s="23">
@@ -4165,18 +4219,18 @@
         <v/>
       </c>
       <c r="H22" s="23">
-        <f>VLOOKUP(Y22,Datos!$A$19:$E$23,2,0)*D22*C22^2</f>
+        <f>VLOOKUP(Y22,Datos!$A$19:$E$23,2,0)*D22*C22^2+0.75*1000*IF(OR(AD22="",AE22=""),0,AD22*AE22*(C22-AE22)/C22/1000)</f>
         <v/>
       </c>
       <c r="I22" s="23">
-        <f>IF(VLOOKUP(Y22,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y22,Datos!$A$19:$E$23,3,0)*D22*C22^2)</f>
+        <f>IF(VLOOKUP(Y22,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y22,Datos!$A$19:$E$23,3,0)*D22*C22^2+0.50*1000*IF(OR(AD22="",AE22=""),0,AD22*AE22*(C22-AE22)/C22/1000))</f>
         <v/>
       </c>
       <c r="J22" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K22" s="7">
-        <f>L22-AF22</f>
+        <f>L22-AH22</f>
         <v/>
       </c>
       <c r="L22" s="24" t="n">
@@ -4246,13 +4300,15 @@
         <f>IF(Z22="Invertida",MIN(C22*100/4,J22+16*AA22),J22)</f>
         <v/>
       </c>
-      <c r="AD22" s="24" t="n">
+      <c r="AD22" s="24" t="n"/>
+      <c r="AE22" s="24" t="n"/>
+      <c r="AF22" s="24" t="n">
         <v>1.549</v>
       </c>
-      <c r="AE22" s="24" t="n">
+      <c r="AG22" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF22" s="24" t="n">
+      <c r="AH22" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4267,12 +4323,12 @@
         <v>3.71</v>
       </c>
       <c r="D23" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AE23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD23)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF23+Datos!$B$7*J23*L23/10000+Datos!$B$16*AG23)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF23)</f>
         <v/>
       </c>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="23">
-        <f>VLOOKUP(Y23,Datos!$A$19:$E$23,4,0)*D23*C23</f>
+        <f>VLOOKUP(Y23,Datos!$A$19:$E$23,4,0)*D23*C23+IF(OR(AD23="",AE23=""),0,AD23*MAX(AE23,C23-AE23)/C23)</f>
         <v/>
       </c>
       <c r="G23" s="23">
@@ -4280,18 +4336,18 @@
         <v/>
       </c>
       <c r="H23" s="23">
-        <f>VLOOKUP(Y23,Datos!$A$19:$E$23,2,0)*D23*C23^2</f>
+        <f>VLOOKUP(Y23,Datos!$A$19:$E$23,2,0)*D23*C23^2+0.75*1000*IF(OR(AD23="",AE23=""),0,AD23*AE23*(C23-AE23)/C23/1000)</f>
         <v/>
       </c>
       <c r="I23" s="23">
-        <f>IF(VLOOKUP(Y23,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y23,Datos!$A$19:$E$23,3,0)*D23*C23^2)</f>
+        <f>IF(VLOOKUP(Y23,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y23,Datos!$A$19:$E$23,3,0)*D23*C23^2+0.50*1000*IF(OR(AD23="",AE23=""),0,AD23*AE23*(C23-AE23)/C23/1000))</f>
         <v/>
       </c>
       <c r="J23" s="24" t="n">
         <v>40</v>
       </c>
       <c r="K23" s="7">
-        <f>L23-AF23</f>
+        <f>L23-AH23</f>
         <v/>
       </c>
       <c r="L23" s="24" t="n">
@@ -4361,13 +4417,15 @@
         <f>IF(Z23="Invertida",MIN(C23*100/4,J23+16*AA23),J23)</f>
         <v/>
       </c>
-      <c r="AD23" s="24" t="n">
+      <c r="AD23" s="24" t="n"/>
+      <c r="AE23" s="24" t="n"/>
+      <c r="AF23" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE23" s="24" t="n">
+      <c r="AG23" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF23" s="24" t="n">
+      <c r="AH23" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4382,12 +4440,12 @@
         <v>2.13</v>
       </c>
       <c r="D24" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AE24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD24)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF24+Datos!$B$7*J24*L24/10000+Datos!$B$16*AG24)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF24)</f>
         <v/>
       </c>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="23">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24</f>
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,4,0)*D24*C24+IF(OR(AD24="",AE24=""),0,AD24*MAX(AE24,C24-AE24)/C24)</f>
         <v/>
       </c>
       <c r="G24" s="23">
@@ -4395,18 +4453,18 @@
         <v/>
       </c>
       <c r="H24" s="23">
-        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2</f>
+        <f>VLOOKUP(Y24,Datos!$A$19:$E$23,2,0)*D24*C24^2+0.75*1000*IF(OR(AD24="",AE24=""),0,AD24*AE24*(C24-AE24)/C24/1000)</f>
         <v/>
       </c>
       <c r="I24" s="23">
-        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2)</f>
+        <f>IF(VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y24,Datos!$A$19:$E$23,3,0)*D24*C24^2+0.50*1000*IF(OR(AD24="",AE24=""),0,AD24*AE24*(C24-AE24)/C24/1000))</f>
         <v/>
       </c>
       <c r="J24" s="24" t="n">
         <v>40</v>
       </c>
       <c r="K24" s="7">
-        <f>L24-AF24</f>
+        <f>L24-AH24</f>
         <v/>
       </c>
       <c r="L24" s="24" t="n">
@@ -4476,13 +4534,15 @@
         <f>IF(Z24="Invertida",MIN(C24*100/4,J24+16*AA24),J24)</f>
         <v/>
       </c>
-      <c r="AD24" s="24" t="n">
+      <c r="AD24" s="24" t="n"/>
+      <c r="AE24" s="24" t="n"/>
+      <c r="AF24" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE24" s="24" t="n">
+      <c r="AG24" s="24" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF24" s="24" t="n">
+      <c r="AH24" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4497,12 +4557,12 @@
         <v>3.71</v>
       </c>
       <c r="D25" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AD25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AE25)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AD25)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$4,Datos!$A$14:$E$15,2,0)*AF25+Datos!$B$7*J25*L25/10000+Datos!$B$16*AG25)+Datos!$B$11*VLOOKUP($A$4,Datos!$A$14:$E$15,3,0)*AF25)</f>
         <v/>
       </c>
       <c r="E25" s="32" t="n"/>
       <c r="F25" s="31">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25</f>
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,4,0)*D25*C25+IF(OR(AD25="",AE25=""),0,AD25*MAX(AE25,C25-AE25)/C25)</f>
         <v/>
       </c>
       <c r="G25" s="31">
@@ -4510,18 +4570,18 @@
         <v/>
       </c>
       <c r="H25" s="31">
-        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2</f>
+        <f>VLOOKUP(Y25,Datos!$A$19:$E$23,2,0)*D25*C25^2+0.75*1000*IF(OR(AD25="",AE25=""),0,AD25*AE25*(C25-AE25)/C25/1000)</f>
         <v/>
       </c>
       <c r="I25" s="31">
-        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2)</f>
+        <f>IF(VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y25,Datos!$A$19:$E$23,3,0)*D25*C25^2+0.50*1000*IF(OR(AD25="",AE25=""),0,AD25*AE25*(C25-AE25)/C25/1000))</f>
         <v/>
       </c>
       <c r="J25" s="33" t="n">
         <v>12</v>
       </c>
       <c r="K25" s="32">
-        <f>L25-AF25</f>
+        <f>L25-AH25</f>
         <v/>
       </c>
       <c r="L25" s="33" t="n">
@@ -4591,13 +4651,15 @@
         <f>IF(Z25="Invertida",MIN(C25*100/4,J25+16*AA25),J25)</f>
         <v/>
       </c>
-      <c r="AD25" s="33" t="n">
+      <c r="AD25" s="33" t="n"/>
+      <c r="AE25" s="33" t="n"/>
+      <c r="AF25" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE25" s="33" t="n">
+      <c r="AG25" s="33" t="n">
         <v>2.6</v>
       </c>
-      <c r="AF25" s="33" t="n">
+      <c r="AH25" s="33" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4616,12 +4678,12 @@
         <v>9.9</v>
       </c>
       <c r="D26" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AE26)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD26)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF26+Datos!$B$7*J26*L26/10000+Datos!$B$16*AG26)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF26)</f>
         <v/>
       </c>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="23">
-        <f>VLOOKUP(Y26,Datos!$A$19:$E$23,4,0)*D26*C26</f>
+        <f>VLOOKUP(Y26,Datos!$A$19:$E$23,4,0)*D26*C26+IF(OR(AD26="",AE26=""),0,AD26*MAX(AE26,C26-AE26)/C26)</f>
         <v/>
       </c>
       <c r="G26" s="23">
@@ -4629,18 +4691,18 @@
         <v/>
       </c>
       <c r="H26" s="23">
-        <f>VLOOKUP(Y26,Datos!$A$19:$E$23,2,0)*D26*C26^2</f>
+        <f>VLOOKUP(Y26,Datos!$A$19:$E$23,2,0)*D26*C26^2+0.75*1000*IF(OR(AD26="",AE26=""),0,AD26*AE26*(C26-AE26)/C26/1000)</f>
         <v/>
       </c>
       <c r="I26" s="23">
-        <f>IF(VLOOKUP(Y26,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y26,Datos!$A$19:$E$23,3,0)*D26*C26^2)</f>
+        <f>IF(VLOOKUP(Y26,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y26,Datos!$A$19:$E$23,3,0)*D26*C26^2+0.50*1000*IF(OR(AD26="",AE26=""),0,AD26*AE26*(C26-AE26)/C26/1000))</f>
         <v/>
       </c>
       <c r="J26" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K26" s="7">
-        <f>L26-AF26</f>
+        <f>L26-AH26</f>
         <v/>
       </c>
       <c r="L26" s="24" t="n">
@@ -4706,13 +4768,15 @@
         <f>IF(Z26="Invertida",MIN(C26*100/4,J26+16*AA26),J26)</f>
         <v/>
       </c>
-      <c r="AD26" s="24" t="n">
+      <c r="AD26" s="24" t="n"/>
+      <c r="AE26" s="24" t="n"/>
+      <c r="AF26" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE26" s="24" t="n">
+      <c r="AG26" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF26" s="24" t="n">
+      <c r="AH26" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4727,12 +4791,12 @@
         <v>6</v>
       </c>
       <c r="D27" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AE27)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD27)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF27+Datos!$B$7*J27*L27/10000+Datos!$B$16*AG27)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF27)</f>
         <v/>
       </c>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="23">
-        <f>VLOOKUP(Y27,Datos!$A$19:$E$23,4,0)*D27*C27</f>
+        <f>VLOOKUP(Y27,Datos!$A$19:$E$23,4,0)*D27*C27+IF(OR(AD27="",AE27=""),0,AD27*MAX(AE27,C27-AE27)/C27)</f>
         <v/>
       </c>
       <c r="G27" s="23">
@@ -4740,18 +4804,18 @@
         <v/>
       </c>
       <c r="H27" s="23">
-        <f>VLOOKUP(Y27,Datos!$A$19:$E$23,2,0)*D27*C27^2</f>
+        <f>VLOOKUP(Y27,Datos!$A$19:$E$23,2,0)*D27*C27^2+0.75*1000*IF(OR(AD27="",AE27=""),0,AD27*AE27*(C27-AE27)/C27/1000)</f>
         <v/>
       </c>
       <c r="I27" s="23">
-        <f>IF(VLOOKUP(Y27,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y27,Datos!$A$19:$E$23,3,0)*D27*C27^2)</f>
+        <f>IF(VLOOKUP(Y27,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y27,Datos!$A$19:$E$23,3,0)*D27*C27^2+0.50*1000*IF(OR(AD27="",AE27=""),0,AD27*AE27*(C27-AE27)/C27/1000))</f>
         <v/>
       </c>
       <c r="J27" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K27" s="7">
-        <f>L27-AF27</f>
+        <f>L27-AH27</f>
         <v/>
       </c>
       <c r="L27" s="24" t="n">
@@ -4817,13 +4881,15 @@
         <f>IF(Z27="Invertida",MIN(C27*100/4,J27+16*AA27),J27)</f>
         <v/>
       </c>
-      <c r="AD27" s="24" t="n">
+      <c r="AD27" s="24" t="n"/>
+      <c r="AE27" s="24" t="n"/>
+      <c r="AF27" s="24" t="n">
         <v>3.799</v>
       </c>
-      <c r="AE27" s="24" t="n">
+      <c r="AG27" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF27" s="24" t="n">
+      <c r="AH27" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4838,12 +4904,12 @@
         <v>3.75</v>
       </c>
       <c r="D28" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AE28)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD28)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF28+Datos!$B$7*J28*L28/10000+Datos!$B$16*AG28)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF28)</f>
         <v/>
       </c>
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="23">
-        <f>VLOOKUP(Y28,Datos!$A$19:$E$23,4,0)*D28*C28</f>
+        <f>VLOOKUP(Y28,Datos!$A$19:$E$23,4,0)*D28*C28+IF(OR(AD28="",AE28=""),0,AD28*MAX(AE28,C28-AE28)/C28)</f>
         <v/>
       </c>
       <c r="G28" s="23">
@@ -4851,18 +4917,18 @@
         <v/>
       </c>
       <c r="H28" s="23">
-        <f>VLOOKUP(Y28,Datos!$A$19:$E$23,2,0)*D28*C28^2</f>
+        <f>VLOOKUP(Y28,Datos!$A$19:$E$23,2,0)*D28*C28^2+0.75*1000*IF(OR(AD28="",AE28=""),0,AD28*AE28*(C28-AE28)/C28/1000)</f>
         <v/>
       </c>
       <c r="I28" s="23">
-        <f>IF(VLOOKUP(Y28,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y28,Datos!$A$19:$E$23,3,0)*D28*C28^2)</f>
+        <f>IF(VLOOKUP(Y28,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y28,Datos!$A$19:$E$23,3,0)*D28*C28^2+0.50*1000*IF(OR(AD28="",AE28=""),0,AD28*AE28*(C28-AE28)/C28/1000))</f>
         <v/>
       </c>
       <c r="J28" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K28" s="7">
-        <f>L28-AF28</f>
+        <f>L28-AH28</f>
         <v/>
       </c>
       <c r="L28" s="24" t="n">
@@ -4928,13 +4994,15 @@
         <f>IF(Z28="Invertida",MIN(C28*100/4,J28+16*AA28),J28)</f>
         <v/>
       </c>
-      <c r="AD28" s="24" t="n">
+      <c r="AD28" s="24" t="n"/>
+      <c r="AE28" s="24" t="n"/>
+      <c r="AF28" s="24" t="n">
         <v>2.1</v>
       </c>
-      <c r="AE28" s="24" t="n">
+      <c r="AG28" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF28" s="24" t="n">
+      <c r="AH28" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -4949,12 +5017,12 @@
         <v>6</v>
       </c>
       <c r="D29" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AE29)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD29)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF29+Datos!$B$7*J29*L29/10000+Datos!$B$16*AG29)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF29)</f>
         <v/>
       </c>
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="23">
-        <f>VLOOKUP(Y29,Datos!$A$19:$E$23,4,0)*D29*C29</f>
+        <f>VLOOKUP(Y29,Datos!$A$19:$E$23,4,0)*D29*C29+IF(OR(AD29="",AE29=""),0,AD29*MAX(AE29,C29-AE29)/C29)</f>
         <v/>
       </c>
       <c r="G29" s="23">
@@ -4962,18 +5030,18 @@
         <v/>
       </c>
       <c r="H29" s="23">
-        <f>VLOOKUP(Y29,Datos!$A$19:$E$23,2,0)*D29*C29^2</f>
+        <f>VLOOKUP(Y29,Datos!$A$19:$E$23,2,0)*D29*C29^2+0.75*1000*IF(OR(AD29="",AE29=""),0,AD29*AE29*(C29-AE29)/C29/1000)</f>
         <v/>
       </c>
       <c r="I29" s="23">
-        <f>IF(VLOOKUP(Y29,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y29,Datos!$A$19:$E$23,3,0)*D29*C29^2)</f>
+        <f>IF(VLOOKUP(Y29,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y29,Datos!$A$19:$E$23,3,0)*D29*C29^2+0.50*1000*IF(OR(AD29="",AE29=""),0,AD29*AE29*(C29-AE29)/C29/1000))</f>
         <v/>
       </c>
       <c r="J29" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K29" s="7">
-        <f>L29-AF29</f>
+        <f>L29-AH29</f>
         <v/>
       </c>
       <c r="L29" s="24" t="n">
@@ -5039,13 +5107,15 @@
         <f>IF(Z29="Invertida",MIN(C29*100/4,J29+16*AA29),J29)</f>
         <v/>
       </c>
-      <c r="AD29" s="24" t="n">
+      <c r="AD29" s="24" t="n"/>
+      <c r="AE29" s="24" t="n"/>
+      <c r="AF29" s="24" t="n">
         <v>1.699</v>
       </c>
-      <c r="AE29" s="24" t="n">
+      <c r="AG29" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF29" s="24" t="n">
+      <c r="AH29" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5060,12 +5130,12 @@
         <v>4.03</v>
       </c>
       <c r="D30" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AE30)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD30)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF30+Datos!$B$7*J30*L30/10000+Datos!$B$16*AG30)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF30)</f>
         <v/>
       </c>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="23">
-        <f>VLOOKUP(Y30,Datos!$A$19:$E$23,4,0)*D30*C30</f>
+        <f>VLOOKUP(Y30,Datos!$A$19:$E$23,4,0)*D30*C30+IF(OR(AD30="",AE30=""),0,AD30*MAX(AE30,C30-AE30)/C30)</f>
         <v/>
       </c>
       <c r="G30" s="23">
@@ -5073,18 +5143,18 @@
         <v/>
       </c>
       <c r="H30" s="23">
-        <f>VLOOKUP(Y30,Datos!$A$19:$E$23,2,0)*D30*C30^2</f>
+        <f>VLOOKUP(Y30,Datos!$A$19:$E$23,2,0)*D30*C30^2+0.75*1000*IF(OR(AD30="",AE30=""),0,AD30*AE30*(C30-AE30)/C30/1000)</f>
         <v/>
       </c>
       <c r="I30" s="23">
-        <f>IF(VLOOKUP(Y30,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y30,Datos!$A$19:$E$23,3,0)*D30*C30^2)</f>
+        <f>IF(VLOOKUP(Y30,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y30,Datos!$A$19:$E$23,3,0)*D30*C30^2+0.50*1000*IF(OR(AD30="",AE30=""),0,AD30*AE30*(C30-AE30)/C30/1000))</f>
         <v/>
       </c>
       <c r="J30" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K30" s="7">
-        <f>L30-AF30</f>
+        <f>L30-AH30</f>
         <v/>
       </c>
       <c r="L30" s="24" t="n">
@@ -5154,13 +5224,15 @@
         <f>IF(Z30="Invertida",MIN(C30*100/4,J30+16*AA30),J30)</f>
         <v/>
       </c>
-      <c r="AD30" s="24" t="n">
+      <c r="AD30" s="24" t="n"/>
+      <c r="AE30" s="24" t="n"/>
+      <c r="AF30" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="AE30" s="24" t="n">
+      <c r="AG30" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF30" s="24" t="n">
+      <c r="AH30" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5175,12 +5247,12 @@
         <v>4.85</v>
       </c>
       <c r="D31" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AE31)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD31)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF31+Datos!$B$7*J31*L31/10000+Datos!$B$16*AG31)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF31)</f>
         <v/>
       </c>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="23">
-        <f>VLOOKUP(Y31,Datos!$A$19:$E$23,4,0)*D31*C31</f>
+        <f>VLOOKUP(Y31,Datos!$A$19:$E$23,4,0)*D31*C31+IF(OR(AD31="",AE31=""),0,AD31*MAX(AE31,C31-AE31)/C31)</f>
         <v/>
       </c>
       <c r="G31" s="23">
@@ -5188,18 +5260,18 @@
         <v/>
       </c>
       <c r="H31" s="23">
-        <f>VLOOKUP(Y31,Datos!$A$19:$E$23,2,0)*D31*C31^2</f>
+        <f>VLOOKUP(Y31,Datos!$A$19:$E$23,2,0)*D31*C31^2+0.75*1000*IF(OR(AD31="",AE31=""),0,AD31*AE31*(C31-AE31)/C31/1000)</f>
         <v/>
       </c>
       <c r="I31" s="23">
-        <f>IF(VLOOKUP(Y31,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y31,Datos!$A$19:$E$23,3,0)*D31*C31^2)</f>
+        <f>IF(VLOOKUP(Y31,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y31,Datos!$A$19:$E$23,3,0)*D31*C31^2+0.50*1000*IF(OR(AD31="",AE31=""),0,AD31*AE31*(C31-AE31)/C31/1000))</f>
         <v/>
       </c>
       <c r="J31" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K31" s="7">
-        <f>L31-AF31</f>
+        <f>L31-AH31</f>
         <v/>
       </c>
       <c r="L31" s="24" t="n">
@@ -5269,13 +5341,15 @@
         <f>IF(Z31="Invertida",MIN(C31*100/4,J31+16*AA31),J31)</f>
         <v/>
       </c>
-      <c r="AD31" s="24" t="n">
+      <c r="AD31" s="24" t="n"/>
+      <c r="AE31" s="24" t="n"/>
+      <c r="AF31" s="24" t="n">
         <v>1.699</v>
       </c>
-      <c r="AE31" s="24" t="n">
+      <c r="AG31" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF31" s="24" t="n">
+      <c r="AH31" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5290,12 +5364,12 @@
         <v>3.58</v>
       </c>
       <c r="D32" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AE32)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD32)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF32+Datos!$B$7*J32*L32/10000+Datos!$B$16*AG32)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF32)</f>
         <v/>
       </c>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="23">
-        <f>VLOOKUP(Y32,Datos!$A$19:$E$23,4,0)*D32*C32</f>
+        <f>VLOOKUP(Y32,Datos!$A$19:$E$23,4,0)*D32*C32+IF(OR(AD32="",AE32=""),0,AD32*MAX(AE32,C32-AE32)/C32)</f>
         <v/>
       </c>
       <c r="G32" s="23">
@@ -5303,18 +5377,18 @@
         <v/>
       </c>
       <c r="H32" s="23">
-        <f>VLOOKUP(Y32,Datos!$A$19:$E$23,2,0)*D32*C32^2</f>
+        <f>VLOOKUP(Y32,Datos!$A$19:$E$23,2,0)*D32*C32^2+0.75*1000*IF(OR(AD32="",AE32=""),0,AD32*AE32*(C32-AE32)/C32/1000)</f>
         <v/>
       </c>
       <c r="I32" s="23">
-        <f>IF(VLOOKUP(Y32,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y32,Datos!$A$19:$E$23,3,0)*D32*C32^2)</f>
+        <f>IF(VLOOKUP(Y32,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y32,Datos!$A$19:$E$23,3,0)*D32*C32^2+0.50*1000*IF(OR(AD32="",AE32=""),0,AD32*AE32*(C32-AE32)/C32/1000))</f>
         <v/>
       </c>
       <c r="J32" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K32" s="7">
-        <f>L32-AF32</f>
+        <f>L32-AH32</f>
         <v/>
       </c>
       <c r="L32" s="24" t="n">
@@ -5380,13 +5454,15 @@
         <f>IF(Z32="Invertida",MIN(C32*100/4,J32+16*AA32),J32)</f>
         <v/>
       </c>
-      <c r="AD32" s="24" t="n">
+      <c r="AD32" s="24" t="n"/>
+      <c r="AE32" s="24" t="n"/>
+      <c r="AF32" s="24" t="n">
         <v>1.699</v>
       </c>
-      <c r="AE32" s="24" t="n">
+      <c r="AG32" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF32" s="24" t="n">
+      <c r="AH32" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5401,12 +5477,12 @@
         <v>1.12</v>
       </c>
       <c r="D33" s="23">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AE33)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD33)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF33+Datos!$B$7*J33*L33/10000+Datos!$B$16*AG33)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF33)</f>
         <v/>
       </c>
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="23">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33</f>
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,4,0)*D33*C33+IF(OR(AD33="",AE33=""),0,AD33*MAX(AE33,C33-AE33)/C33)</f>
         <v/>
       </c>
       <c r="G33" s="23">
@@ -5414,18 +5490,18 @@
         <v/>
       </c>
       <c r="H33" s="23">
-        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2</f>
+        <f>VLOOKUP(Y33,Datos!$A$19:$E$23,2,0)*D33*C33^2+0.75*1000*IF(OR(AD33="",AE33=""),0,AD33*AE33*(C33-AE33)/C33/1000)</f>
         <v/>
       </c>
       <c r="I33" s="23">
-        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2)</f>
+        <f>IF(VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y33,Datos!$A$19:$E$23,3,0)*D33*C33^2+0.50*1000*IF(OR(AD33="",AE33=""),0,AD33*AE33*(C33-AE33)/C33/1000))</f>
         <v/>
       </c>
       <c r="J33" s="24" t="n">
         <v>15</v>
       </c>
       <c r="K33" s="7">
-        <f>L33-AF33</f>
+        <f>L33-AH33</f>
         <v/>
       </c>
       <c r="L33" s="24" t="n">
@@ -5491,13 +5567,15 @@
         <f>IF(Z33="Invertida",MIN(C33*100/4,J33+16*AA33),J33)</f>
         <v/>
       </c>
-      <c r="AD33" s="24" t="n">
+      <c r="AD33" s="24" t="n"/>
+      <c r="AE33" s="24" t="n"/>
+      <c r="AF33" s="24" t="n">
         <v>1.699</v>
       </c>
-      <c r="AE33" s="24" t="n">
+      <c r="AG33" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="AF33" s="24" t="n">
+      <c r="AH33" s="24" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5512,12 +5590,12 @@
         <v>4.35</v>
       </c>
       <c r="D34" s="31">
-        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AD34+Datos!$B$7*J34*L34/10000+Datos!$B$16*AE34)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AD34)</f>
+        <f>(Datos!$B$10*(VLOOKUP($A$26,Datos!$A$14:$E$15,2,0)*AF34+Datos!$B$7*J34*L34/10000+Datos!$B$16*AG34)+Datos!$B$11*VLOOKUP($A$26,Datos!$A$14:$E$15,3,0)*AF34)</f>
         <v/>
       </c>
       <c r="E34" s="32" t="n"/>
       <c r="F34" s="31">
-        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,4,0)*D34*C34</f>
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,4,0)*D34*C34+IF(OR(AD34="",AE34=""),0,AD34*MAX(AE34,C34-AE34)/C34)</f>
         <v/>
       </c>
       <c r="G34" s="31">
@@ -5525,18 +5603,18 @@
         <v/>
       </c>
       <c r="H34" s="31">
-        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,2,0)*D34*C34^2</f>
+        <f>VLOOKUP(Y34,Datos!$A$19:$E$23,2,0)*D34*C34^2+0.75*1000*IF(OR(AD34="",AE34=""),0,AD34*AE34*(C34-AE34)/C34/1000)</f>
         <v/>
       </c>
       <c r="I34" s="31">
-        <f>IF(VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)*D34*C34^2)</f>
+        <f>IF(VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)=0,"---",VLOOKUP(Y34,Datos!$A$19:$E$23,3,0)*D34*C34^2+0.50*1000*IF(OR(AD34="",AE34=""),0,AD34*AE34*(C34-AE34)/C34/1000))</f>
         <v/>
       </c>
       <c r="J34" s="33" t="n">
         <v>15</v>
       </c>
       <c r="K34" s="32">
-        <f>L34-AF34</f>
+        <f>L34-AH34</f>
         <v/>
       </c>
       <c r="L34" s="33" t="n">
@@ -5606,13 +5684,15 @@
         <f>IF(Z34="Invertida",MIN(C34*100/4,J34+16*AA34),J34)</f>
         <v/>
       </c>
-      <c r="AD34" s="33" t="n">
+      <c r="AD34" s="33" t="n"/>
+      <c r="AE34" s="33" t="n"/>
+      <c r="AF34" s="33" t="n">
         <v>0</v>
       </c>
-      <c r="AE34" s="33" t="n">
+      <c r="AG34" s="33" t="n">
         <v>1</v>
       </c>
-      <c r="AF34" s="33" t="n">
+      <c r="AH34" s="33" t="n">
         <v>3</v>
       </c>
     </row>
@@ -5622,20 +5702,20 @@
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="A4:A25"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="A1:AF1"/>
     <mergeCell ref="P2:R2"/>
     <mergeCell ref="S2:U2"/>
     <mergeCell ref="A26:A34"/>
     <mergeCell ref="I2:I3"/>
-    <mergeCell ref="V2"/>
+    <mergeCell ref="A1:AH1"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
-    <mergeCell ref="Y2:AF2"/>
+    <mergeCell ref="V2"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="X2:X3"/>
     <mergeCell ref="M2:O2"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="W2:W3"/>
+    <mergeCell ref="Y2:AH2"/>
   </mergeCells>
   <conditionalFormatting sqref="W4:W34">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">

</xml_diff>

<commit_message>
Cargar la puntual de VI 09 sobre VI 04a
VI 09 es una viga secundaria: sus dos extremos descargan en VI 04a
y en VI 06. Sobre VI 04a apoya a 1,80 m, practicamente al medio de
sus 3,75 m, con 6.332 kg. Como esa viga no recibe losa, la puntual
es casi toda su carga: el momento de tramo pasa de 1.087 a 5.532
kgm y verifica con 3d12. Queda pendiente cargar las dos puntuales
que recibe VI 06, a la espera de su posicion.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -2660,7 +2660,11 @@
         <f>IF(OR(M8="REVISAR",P8="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M8&lt;&gt;"REVISAR",P8&lt;&gt;"REVISAR",IF(ISNUMBER(M8),N8*PI()*(O8/10)^2/4&gt;=M8,TRUE),IF(ISNUMBER(P8),Q8*PI()*(R8/10)^2/4&gt;=P8,TRUE),IF(ISNUMBER(M8),M8&lt;=0.0163*AB8*K8,TRUE),IF(ISNUMBER(P8),P8&lt;=0.0163*AC8*K8,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F8&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J8*K8+2*PI()*(U8/10)^2/4*Datos!$B$6*K8/V8)),"NO VERIF. CORTE",IF(NOT(L8&gt;=C8*100/VLOOKUP(Y8,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X8" s="7" t="n"/>
+      <c r="X8" s="26" t="inlineStr">
+        <is>
+          <t>VI 09 le descarga 6.332 kg a 1,80 m del apoyo, practicamente al medio de sus 3,75 m. Esta viga no recibe losa, de modo que la puntual es casi toda su carga. Se superpone el momento isostatico P a b / L repartido 0,75 al tramo y 0,50 al apoyo, y la reaccion isostatica al corte.</t>
+        </is>
+      </c>
       <c r="Y8" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -2682,8 +2686,12 @@
         <f>IF(Z8="Invertida",MIN(C8*100/4,J8+16*AA8),J8)</f>
         <v/>
       </c>
-      <c r="AD8" s="24" t="n"/>
-      <c r="AE8" s="24" t="n"/>
+      <c r="AD8" s="24" t="n">
+        <v>6332</v>
+      </c>
+      <c r="AE8" s="24" t="n">
+        <v>1.8</v>
+      </c>
       <c r="AF8" s="24" t="n">
         <v>0</v>
       </c>
@@ -2888,7 +2896,7 @@
       </c>
       <c r="X10" s="26" t="inlineStr">
         <is>
-          <t>Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07.</t>
+          <t>Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. PENDIENTE: recibe las puntuales de VI 09 (6,3 t) y VI 08b (6,0 t) y todavia no estan cargadas, porque falta saber en que tramo y a que distancia caen. Con ambas al medio del tramo mayor el momento de tramo pasaria de 7.920 a 22.963 kgm.</t>
         </is>
       </c>
       <c r="Y10" s="24" t="inlineStr">
@@ -3471,7 +3479,11 @@
         <f>IF(OR(M15="REVISAR",P15="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M15&lt;&gt;"REVISAR",P15&lt;&gt;"REVISAR",IF(ISNUMBER(M15),N15*PI()*(O15/10)^2/4&gt;=M15,TRUE),IF(ISNUMBER(P15),Q15*PI()*(R15/10)^2/4&gt;=P15,TRUE),IF(ISNUMBER(M15),M15&lt;=0.0163*AB15*K15,TRUE),IF(ISNUMBER(P15),P15&lt;=0.0163*AC15*K15,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F15&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J15*K15+2*PI()*(U15/10)^2/4*Datos!$B$6*K15/V15)),"NO VERIF. CORTE",IF(NOT(L15&gt;=C15*100/VLOOKUP(Y15,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X15" s="7" t="n"/>
+      <c r="X15" s="26" t="inlineStr">
+        <is>
+          <t>Descarga en la COL 04 de 20x20 y en VI 06.</t>
+        </is>
+      </c>
       <c r="Y15" s="24" t="inlineStr">
         <is>
           <t>Continua</t>
@@ -3588,7 +3600,11 @@
         <f>IF(OR(M16="REVISAR",P16="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M16&lt;&gt;"REVISAR",P16&lt;&gt;"REVISAR",IF(ISNUMBER(M16),N16*PI()*(O16/10)^2/4&gt;=M16,TRUE),IF(ISNUMBER(P16),Q16*PI()*(R16/10)^2/4&gt;=P16,TRUE),IF(ISNUMBER(M16),M16&lt;=0.0163*AB16*K16,TRUE),IF(ISNUMBER(P16),P16&lt;=0.0163*AC16*K16,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F16&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J16*K16+2*PI()*(U16/10)^2/4*Datos!$B$6*K16/V16)),"NO VERIF. CORTE",IF(NOT(L16&gt;=C16*100/VLOOKUP(Y16,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
         <v/>
       </c>
-      <c r="X16" s="7" t="n"/>
+      <c r="X16" s="26" t="inlineStr">
+        <is>
+          <t>Viga secundaria: sus dos extremos descargan en otras vigas, VI 04a y VI 06, no en columnas ni tabiques.</t>
+        </is>
+      </c>
       <c r="Y16" s="24" t="inlineStr">
         <is>
           <t>Simplemente apoyada</t>

</xml_diff>

<commit_message>
Cargar la puntual de VI 08b sobre VI 06
Cae a 6,00 m del extremo inferior, dentro del tramo de 6,53 m y a
solo 53 cm del apoyo siguiente: aporta poco momento y mucho corte.
El momento de tramo pasa de 7.919 a 10.095 kgm y la reaccion de
9.764 a 15.235 kg. VI 06 verifica con 2d20 en tramo y en apoyo y
estribos d6 c/10. El tramo del medio, con la puntual de VI 09, da
7.993 kgm y no gobierna.
Con esto la bajada de cargas queda completa.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NNMcFTBbEuLfDho1wCZzu7
</commit_message>
<xml_diff>
--- a/planillas/planilla_vigas.xlsx
+++ b/planillas/planilla_vigas.xlsx
@@ -2861,10 +2861,10 @@
         <v/>
       </c>
       <c r="N10" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="O10" s="24" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="P10" s="25">
         <f>IF(NOT(ISNUMBER(I10)),"---",IF(I10&lt;=0,"---",IF(I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)&gt;=0.5,"REVISAR",MAX((1-SQRT(1-2*I10*100/(Datos!$B$8*AC10*K10^2*Datos!$B$5)))*AC10*K10*Datos!$B$5/Datos!$B$6,0.0033*J10*K10))))</f>
@@ -2888,7 +2888,7 @@
         <v>6</v>
       </c>
       <c r="V10" s="24" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="W10" s="7">
         <f>IF(OR(M10="REVISAR",P10="REVISAR"),"SECCION INSUF.",IF(NOT(AND(M10&lt;&gt;"REVISAR",P10&lt;&gt;"REVISAR",IF(ISNUMBER(M10),N10*PI()*(O10/10)^2/4&gt;=M10,TRUE),IF(ISNUMBER(P10),Q10*PI()*(R10/10)^2/4&gt;=P10,TRUE),IF(ISNUMBER(M10),M10&lt;=0.0163*AB10*K10,TRUE),IF(ISNUMBER(P10),P10&lt;=0.0163*AC10*K10,TRUE))),"NO VERIFICA FLEX.",IF(NOT(F10&lt;=Datos!$B$9*(0.53*SQRT(Datos!$B$5)*J10*K10+2*PI()*(U10/10)^2/4*Datos!$B$6*K10/V10)),"NO VERIF. CORTE",IF(NOT(L10&gt;=C10*100/VLOOKUP(Y10,Datos!$A$19:$E$23,5,0)),"VERIFICAR FLECHA","VERIFICA"))))</f>
@@ -2896,7 +2896,7 @@
       </c>
       <c r="X10" s="26" t="inlineStr">
         <is>
-          <t>Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. PENDIENTE: recibe las puntuales de VI 09 (6,3 t) y VI 08b (6,0 t) y todavia no estan cargadas, porque falta saber en que tramo y a que distancia caen. Con ambas al medio del tramo mayor el momento de tramo pasaria de 7.920 a 22.963 kgm.</t>
+          <t>Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. Longitud total 14,00 m. Sobre su eje hay cuatro columnas: trabaja como viga continua de tres tramos de 4,10, 4,32 y 6,53 m. Se calcula con el mayor. Es el cuarto borde de la losa cruzada L07. VI 08b le descarga 5.954 kg a 6,00 m del extremo inferior, dentro del tramo de 6,53 m y a solo 53 cm del apoyo siguiente: aporta poco momento y mucho corte, por eso la reaccion sube de 9.764 a 15.235 kg. Se superpone el momento isostatico P a b / L repartido 0,75 al tramo y 0,50 al apoyo, y la reaccion isostatica al corte. Viga principal: recibe a VI 08b y a VI 09. VI 09 apoya a 7,95 m del extremo inferior, o sea en el tramo del medio de 4,32 m, que con esa puntual llega a 7.993 kgm y no gobierna. El tramo que gobierna es el de 6,53 m con la puntual de VI 08b.</t>
         </is>
       </c>
       <c r="Y10" s="24" t="inlineStr">
@@ -2920,8 +2920,12 @@
         <f>IF(Z10="Invertida",MIN(C10*100/4,J10+16*AA10),J10)</f>
         <v/>
       </c>
-      <c r="AD10" s="24" t="n"/>
-      <c r="AE10" s="24" t="n"/>
+      <c r="AD10" s="24" t="n">
+        <v>5954</v>
+      </c>
+      <c r="AE10" s="24" t="n">
+        <v>6</v>
+      </c>
       <c r="AF10" s="24" t="n">
         <v>1.549</v>
       </c>

</xml_diff>